<commit_message>
test(vibe): run VR-019..VR-022 and sync verdicts into TC-MASTER [AI]
Record the TS and DLV sessions with per-TC evidence and add the TS
coverage ledger. Align the Status column of TC-MASTER v1.0/v1.1
with the coverage ledgers, move deferred reasons into Notes, and
flag the 54 v1.0 rows superseded by v1.1 so round stats do not
double count them.

Regenerate PROGRESS-v1.1: the previous table missed VR-020/VR-021
and counted four DLV cases as not run although they passed.

Refs: N/A
</commit_message>
<xml_diff>
--- a/03_test-cases/v1.0/TC-MASTER-v1.0.xlsx
+++ b/03_test-cases/v1.0/TC-MASTER-v1.0.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="ALL" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Hoạt động (Đơn của tôi)" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Ghép nối" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Huỷ đơn · Huỷ nhận đơn" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Giao nhận &amp; Theo dõi đơn" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Bảng tin &amp; Chi tiết tin" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Quà cảm ơn" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Trang chủ" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Thông báo" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Đăng tin &amp; Quản lý tin" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Trust &amp; Safety" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Tài khoản &amp; Hồ sơ" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ALL" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Hoạt động (Đơn của tôi)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Ghép nối" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Huỷ đơn · Huỷ nhận đơn" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Giao nhận &amp; Theo dõi đơn" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bảng tin &amp; Chi tiết tin" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quà cảm ơn" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trang chủ" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Thông báo" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Đăng tin &amp; Quản lý tin" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trust &amp; Safety" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tài khoản &amp; Hồ sơ" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'ALL'!$A$1:$P$220</definedName>
@@ -1207,7 +1207,7 @@
           <t>1 đơn `MATCHED` có khai người nhận (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="n"/>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L319-320 (`NTF-01` và `NTF-02`). Danh sách loại thông báo chính thức còn chờ `C-NTF-01`; nội dung lệch ⇒ dẫn `C-NTF-01` để BA chốt, ⛔ không tự sửa chuỗi trong TC.</t>
@@ -1283,7 +1283,7 @@
           <t>1 tin OFFER + 1 tin NEED khớp tuyến (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="n"/>
       <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L321 (`NTF-03`) + `US-D12` §D1b L186. ⛔ Không assert độ trễ hay chu kỳ quét — chưa chốt (`C-NTF-02` Partially Resolved).</t>
@@ -1361,7 +1361,7 @@
           <t>1 đơn `MATCHED` đủ 3 vai (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Mục đích: `NTF-04` có **2 người nhận** ⇒ phải kiểm cả hai, thiếu một vai là bỏ sót nửa rule. · Căn cứ: `§D6` L322.</t>
@@ -1439,7 +1439,7 @@
           <t>1 đơn `IN_TRANSIT` đủ 3 vai (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Mục đích: `NTF-05` có 2 người nhận. · Căn cứ: `§D6` L323.</t>
@@ -1520,7 +1520,7 @@
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn 2 chuỗi text cho cùng `NTF-06`. · Căn cứ: assert theo BRD `§D6` L324 vì bản PRD+Figma ("Đơn đã hoàn thành — đánh giá ngay") dẫn tới cơ chế **đánh giá đã bị `C-GIFT-01` loại khỏi v1.0** ⇒ chuỗi đó không nhất quán với scope đã chốt. App hiện bản PRD ⇒ FAIL và dẫn `C-NTF-01` để BA chốt text.</t>
+          <t>Mục đích: 2 nguồn 2 chuỗi text cho cùng `NTF-06`. · Căn cứ: assert theo BRD `§D6` L324 vì bản PRD+Figma ("Đơn đã hoàn thành — đánh giá ngay") dẫn tới cơ chế **đánh giá đã bị `C-GIFT-01` loại khỏi v1.0** ⇒ chuỗi đó không nhất quán với scope đã chốt. App hiện bản PRD ⇒ FAIL và dẫn `C-NTF-01` để BA chốt text. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -1595,7 +1595,7 @@
           <t>1 đơn `MATCHED`; lý do huỷ ≥5 ký tự (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L326 (`NTF-08`). Nhánh Carrier huỷ nhận có thêm câu "Đơn đang chờ người vận chuyển mới…" theo Figma (`KP-07` hàng #8) — nhánh đó thuộc `TC-CNL-007`, ⛔ không nhồi vào TC này.</t>
@@ -1671,7 +1671,7 @@
           <t>1 tin NEED "Hết hạn" (test_data_catalog §NTF — ⛔ không seed được qua UI)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L327 (`NTF-09`).</t>
@@ -1753,7 +1753,7 @@
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: ranh giới hợp lệ/vi phạm — `NTF-01` **được phép nhắc** "SĐT đã được lộ" nhưng ⛔ không được kèm số. Push là kênh dễ lọt nhất vì nội dung do backend đẩy, không qua UI. · Căn cứ: `OPR-07` §D7 L343 + `§D6` L315. Có thông báo chứa số ⇒ FAIL và log bug mức cao (rò rỉ dữ liệu cá nhân).</t>
+          <t>Mục đích: ranh giới hợp lệ/vi phạm — `NTF-01` **được phép nhắc** "SĐT đã được lộ" nhưng ⛔ không được kèm số. Push là kênh dễ lọt nhất vì nội dung do backend đẩy, không qua UI. · Căn cứ: `OPR-07` §D7 L343 + `§D6` L315. Có thông báo chứa số ⇒ FAIL và log bug mức cao (rò rỉ dữ liệu cá nhân). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
@@ -1826,7 +1826,7 @@
           <t>Thông báo ở 3 mốc thời gian (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.2 + ảnh Figma `3e626d39…`. ⛔ Không assert nhóm cho thông báo cũ hơn 1 tuần — không có nguồn mô tả.</t>
@@ -1903,7 +1903,7 @@
           <t>3 thông báo cùng nhóm thời gian, 1 đã đọc (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-NTF-01` + ảnh Figma `3e626d39…` — trạng thái đọc theo **từng item**.</t>
@@ -1981,7 +1981,7 @@
           <t>2 thông báo chưa đọc (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-NTF-03(a)` Open — chỉ assert vế suy được từ `KB-NTF-01` (trạng thái theo từng item). · Căn cứ: ⛔ không assert nút "Đánh dấu đã đọc" là mark-all hay mark-per-item; cơ chế nút chờ BA chốt.</t>
@@ -2059,7 +2059,7 @@
           <t>Danh sách thông báo dài hơn 1 trang (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="n"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-NTF-02`. ⛔ Không assert số item mỗi trang — không có nguồn mô tả.</t>
@@ -2139,7 +2139,7 @@
           <t>Đúng 2 thông báo chưa đọc (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
           <t>Mục đích: ranh giới của chấm đỏ là **thông báo chưa đọc cuối cùng** — bước 4 tồn tại để bắt lỗi tắt chấm đỏ quá sớm.</t>
@@ -2220,7 +2220,7 @@
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-NTF-01` Open — 3 nguồn cho 3 danh sách khác nhau nên ⛔ không assert danh sách nào là đủ; TC chỉ assert 2 loại **đã bị loại khỏi scope**. · Căn cứ: `KP-07` hàng #6b (`C-GIFT-01` loại rating) và hàng #11 (`C-USR-01` loại CO₂/điểm). Nếu app bắn loại ngoài `§D6` như `KP-07` hàng #10 ("Sắp đến khung giờ hẹn giao") thì **không tính FAIL** — ghi vào `C-NTF-01` làm ứng viên bổ sung.</t>
+          <t>Mục đích: neo vào `C-NTF-01` Open — 3 nguồn cho 3 danh sách khác nhau nên ⛔ không assert danh sách nào là đủ; TC chỉ assert 2 loại **đã bị loại khỏi scope**. · Căn cứ: `KP-07` hàng #6b (`C-GIFT-01` loại rating) và hàng #11 (`C-USR-01` loại CO₂/điểm). Nếu app bắn loại ngoài `§D6` như `KP-07` hàng #10 ("Sắp đến khung giờ hẹn giao") thì **không tính FAIL** — ghi vào `C-NTF-01` làm ứng viên bổ sung. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -2293,7 +2293,7 @@
           <t>Tài khoản 0 thông báo (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="n"/>
       <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-06` Open — text empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được; ⛔ không assert chuỗi hay ảnh empty state.</t>
@@ -2370,7 +2370,7 @@
           <t>Tài khoản có ≥1 thông báo (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: đích "Trang chủ" suy từ đường vào (chuông ở header Trang chủ) — `KP-05 §3` #6 ghi nhận nút back này chưa có mô tả trong doc. Mở chuông từ màn khác là ca khác, ⛔ không nhồi vào TC này.</t>
@@ -2570,7 +2570,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: đối chiếu cấu trúc theo ảnh Figma `f821ba30…`.</t>
@@ -2647,7 +2651,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M4" s="7" t="inlineStr"/>
       <c r="N4" s="7" t="inlineStr">
         <is>
@@ -2720,7 +2728,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng cấu trúc với luồng NEED 3 bước ở TC-ORD-002.</t>
@@ -2808,7 +2820,11 @@
           <t>Loại hàng "Giấy tờ, hồ sơ", giá trị "Thấp", email nội bộ tra được, khung giờ tương đối so với hiện tại (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Mục đích: happy path xuyên 3 bước — nền để so mọi nhánh negative của module. · Căn cứ: `ORD-02` §D3 L240 + `US-D01` §D1b L164. ⛔ Khung giờ chọn **tương đối** so với hiện tại, không hardcode giờ.</t>
@@ -2889,7 +2905,7 @@
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `D8.1` §D8.1 L357 + `KB-VIBE-01`/`KB-VIBE-02`.</t>
+          <t>Căn cứ: `D8.1` §D8.1 L357 + `KB-VIBE-01`/`KB-VIBE-02`. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -2963,7 +2979,11 @@
           <t>8 chip app STG; nhãn "Tài liệu" là giá trị assert-absent (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Mục đích: ⭐ CL lan rộng nhất dự án — mọi TC đợt cũ nhắc "Tài liệu" đều sai chữ. · Căn cứ: assert theo `DOC-v1.0-06` KP-01 §10.2 (`KB-VIBE-01`, có screenshot `VR-002 TC_04.5`) — nguồn có bằng chứng app thắng doc (`MASTER-MEMORY §2`); BRD `D8.1` ghi 5 giá trị và PRD §3.5.1 ghi 8 chip, cả hai đều có "Tài liệu". App xuất hiện chip "Tài liệu" ⇒ FAIL và dẫn `C-ORD-09` để BA chốt danh mục.</t>
@@ -3041,7 +3061,11 @@
           <t>8 chip app STG (test_data_catalog §ORD, biên "không tái hiện được trạng thái chưa chọn")</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt bằng TC lý do **không viết được TC negative "để trống loại hàng"** — cơ chế UI không cho tạo tiền đề đó. · Căn cứ: `KB-VIBE-02`; rule "Không cho để trống" của `D8.1` vì vậy không kiểm chứng được qua UI.</t>
@@ -3120,7 +3144,11 @@
           <t>Giá trị hàng rỗng (test_data_catalog §ORD, biên chặn bước)</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L359 + `KP-01` §10.4.</t>
@@ -3196,7 +3224,11 @@
           <t>Giá trị hàng "Cao" (test_data_catalog §ORD, biên)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-ORD-010. · Căn cứ: `D8.1` §D8.1 L359 + `KB-ORD-05` (nguyên văn banner lấy từ app). ⚠ Phân biệt: cảnh báo theo **mức định tính "Cao"** là CÓ ở v1.0; ngưỡng bằng **số tiền** (`BR-ORD-03`) thì out of scope (`TC-ORD-054`).</t>
@@ -3273,7 +3305,11 @@
           <t>Giá trị hàng "Thấp" và "Vừa" (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-ORD-009 — banner chỉ gắn với mức "Cao".</t>
@@ -3352,7 +3388,11 @@
           <t>Ghi chú 300 ký tự và 301 ký tự (test_data_catalog §ORD, biên)</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L358.</t>
@@ -3435,7 +3475,7 @@
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh hợp lệ của ràng buộc ảnh — cặp với TC-ORD-013 (nhánh bị chặn). · Căn cứ: `D8.1` §D8.1 L360.</t>
+          <t>Mục đích: nhánh hợp lệ của ràng buộc ảnh — cặp với TC-ORD-013 (nhánh bị chặn). · Căn cứ: `D8.1` §D8.1 L360. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -3515,7 +3555,7 @@
       <c r="L16" s="5" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh bị chặn — tách khỏi TC-ORD-012 vì 2 lớp lỗi khác nhau (dung lượng ⟷ định dạng) và để khi FAIL biết ngay lớp nào sai.</t>
+          <t>Mục đích: nhánh bị chặn — tách khỏi TC-ORD-012 vì 2 lớp lỗi khác nhau (dung lượng ⟷ định dạng) và để khi FAIL biết ngay lớp nào sai. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
@@ -3588,7 +3628,11 @@
           <t>Ảnh rỗng (test_data_catalog §ORD, biên hợp lệ)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L360 — ảnh là trường tuỳ chọn.</t>
@@ -3671,7 +3715,11 @@
           <t>Tên và SĐT từ hồ sơ nhân viên (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M19" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L362-363. ⛔ Không assert giá trị SĐT cụ thể — dữ liệu `Master` không seed được, và đang có nghi vấn tự đổi giá trị (`TC-ORD-018`).</t>
@@ -3748,7 +3796,11 @@
           <t>Tên người gửi pre-fill, chỉ đọc (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr"/>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L362 ghi rõ "Chỉ đọc". ⚠ Dự kiến FAIL — `KP-01` §10.5 đã live-verify app cho sửa và **xoá trắng khi chạm**, không tự phục hồi trong phiên ⇒ **log bug** (`KP-05 §5` #1), ⛔ không hạ chuẩn TC theo hành vi app.</t>
@@ -3824,7 +3876,11 @@
           <t>Địa chỉ lấy hàng pre-fill theo nơi làm việc (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-10` Open — quyết định đây là **bug hay tài khoản test chưa cấu hình**. · Căn cứ: `D8.1` §D8.1 L364. ⚠ Dự kiến FAIL — `KP-01` §10.6 ghi app để trống, chỉ có placeholder (`VR-002 TC_04.21` FAIL). ⇒ **Xác nhận với dev trước khi log bug**: nếu hồ sơ tài khoản test thiếu nơi làm việc thì là lỗi dữ liệu test, không phải bug app.</t>
@@ -3901,7 +3957,11 @@
           <t>SĐT người gửi pre-fill (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L22" s="7" t="inlineStr"/>
+      <c r="L22" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M22" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt bằng TC nghi vấn đã quan sát 1 lần — SĐT tự đổi từ `0000142378` sang `0964633313` giữa phiên. · Căn cứ: `KB-VIBE-09` (`KP-01` §10.10). Nếu tái hiện ⇒ **log bug** (`KP-05 §5` #5).</t>
@@ -3979,7 +4039,11 @@
           <t>Email nội bộ tra được `stag_anhdc4@fpt.com` (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L23" s="5" t="inlineStr"/>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M23" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-ORD-020. · Căn cứ: `USR-EML` §D3 L253 + `US-D18` §D1b L168.</t>
@@ -4057,7 +4121,11 @@
           <t>Email nội bộ không có trong danh bạ (test_data_catalog §ORD, biên)</t>
         </is>
       </c>
-      <c r="L24" s="7" t="inlineStr"/>
+      <c r="L24" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M24" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-ORD-019 — phân biệt "không tra thấy" với "email sai định dạng" ở TC-ORD-021. · Căn cứ: `US-D18` §D1b L168 + `D8.1` L366.</t>
@@ -4136,7 +4204,11 @@
           <t>Email thiếu "@" và email ngoài tên miền nội bộ (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr"/>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M25" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L366 — 2 lớp lỗi cùng field, cùng hệ quả "không tra danh bạ" nên giữ trong 1 TC với 2 dòng expected riêng.</t>
@@ -4214,7 +4286,11 @@
           <t>SĐT người nhận do app auto-fill, vd `0000286248` (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L26" s="7" t="inlineStr"/>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M26" s="7" t="inlineStr">
         <is>
           <t>Mục đích: dữ liệu do chính app điền phải qua được validate của chính nó. · Căn cứ: `KB-VIBE-08` (`KP-01` §10.9). ⚠ Dự kiến FAIL — app báo "Số điện thoại không hợp lệ" cho `0000286248` do chính nó điền ⇒ **log bug** (`KP-05 §5` #4); bug có thể ở tầng dữ liệu danh bạ hoặc tầng validate, ghi rõ cả 2 khả năng khi log.</t>
@@ -4291,7 +4367,11 @@
           <t>Nhóm người nhận để trống (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M27" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-01` Resolved 2026-07-28 — nhóm Người nhận là **bắt buộc**. · Căn cứ: `KB-ORD-01` + `DOC-v1.0-02` §7 dòng 2 ghi nhận hành vi prototype cho để trống mà vẫn đăng thành công là **giới hạn bản demo**. ⚠ Dự kiến FAIL nếu app còn hành vi prototype ⇒ log bug.</t>
@@ -4372,7 +4452,11 @@
           <t>Tên người nhận 1 / 2 / 60 / 61 ký tự (test_data_catalog §ORD, 4 mốc biên)</t>
         </is>
       </c>
-      <c r="L28" s="7" t="inlineStr"/>
+      <c r="L28" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M28" s="7" t="inlineStr">
         <is>
           <t>Mục đích: bộ 4 mốc biên của cùng 1 field, chạy liền mạch trong 1 form nên giữ 1 TC; tách khỏi TC-ORD-025 vì SĐT là lớp validate khác. · Căn cứ: `D8.1` §D8.1 L367.</t>
@@ -4455,7 +4539,11 @@
           <t>SĐT 9 / 10 / 11 số, không bắt đầu bằng 0, có chữ (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr"/>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M29" s="5" t="inlineStr">
         <is>
           <t>Mục đích: 5 lớp lỗi của cùng field SĐT — tách khỏi biên độ dài tên ở TC-ORD-024 để khi FAIL biết ngay lớp nào sai. · Căn cứ: `D8.1` §D8.1 L368.</t>
@@ -4532,7 +4620,11 @@
           <t>2 địa chỉ trùng nhau (test_data_catalog §ORD, biên chặn)</t>
         </is>
       </c>
-      <c r="L30" s="7" t="inlineStr"/>
+      <c r="L30" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M30" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L369.</t>
@@ -4620,7 +4712,7 @@
       <c r="L32" s="5" t="inlineStr"/>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `KB-ORD-06` (`KP-01` §3).</t>
+          <t>Căn cứ: `KB-ORD-06` (`KP-01` §3). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
@@ -4700,7 +4792,7 @@
       <c r="L33" s="7" t="inlineStr"/>
       <c r="M33" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: cặp đối chứng (a)/(b) của cùng cơ chế. · Căn cứ: `KB-ORD-06`. Ghi chú cho automation về sau: `set text` đơn thuần **không lưu** giá trị, phải tap suggestion (`KP-01` §10.12).</t>
+          <t>Mục đích: cặp đối chứng (a)/(b) của cùng cơ chế. · Căn cứ: `KB-ORD-06`. Ghi chú cho automation về sau: `set text` đơn thuần **không lưu** giá trị, phải tap suggestion (`KP-01` §10.12). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr">
@@ -4774,7 +4866,11 @@
           <t>Cơ chế field địa chỉ (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-11` Open — 3 nguồn nêu 3 cơ chế cho cùng field. · Căn cứ: assert theo `KB-ORD-06` (nguồn có bằng chứng app, thắng doc); `LOC-03` §D3 L246 nói preset 6 văn phòng và `US-D01` nói không có chip gợi ý. App hiện 6 chip preset ⇒ FAIL và dẫn `C-ORD-11` để BA chốt.</t>
@@ -4855,7 +4951,7 @@
       <c r="L35" s="7" t="inlineStr"/>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh mặc định và nhánh quá khứ — tách khỏi quan hệ Đến/Từ ở TC-ORD-031 vì hai rule khác nhau. · Căn cứ: `D8.1` §D8.1 L370.</t>
+          <t>Mục đích: nhánh mặc định và nhánh quá khứ — tách khỏi quan hệ Đến/Từ ở TC-ORD-031 vì hai rule khác nhau. · Căn cứ: `D8.1` §D8.1 L370. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
@@ -4934,7 +5030,7 @@
       <c r="L36" s="5" t="inlineStr"/>
       <c r="M36" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: biên "= nhau" là mốc hợp lệ dễ bị chặn oan. · Căn cứ: `D8.1` §D8.1 L371.</t>
+          <t>Mục đích: biên "= nhau" là mốc hợp lệ dễ bị chặn oan. · Căn cứ: `D8.1` §D8.1 L371. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N36" s="5" t="inlineStr">
@@ -5013,7 +5109,7 @@
       <c r="L37" s="7" t="inlineStr"/>
       <c r="M37" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `D8.1` §D8.1 L372. ⛔ Chọn giờ **tương đối** so với hiện tại, không hardcode giờ — app validate theo đồng hồ thật (`KP-01` §10.11).</t>
+          <t>Căn cứ: `D8.1` §D8.1 L372. ⛔ Chọn giờ **tương đối** so với hiện tại, không hardcode giờ — app validate theo đồng hồ thật (`KP-01` §10.11). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr">
@@ -5087,7 +5183,11 @@
           <t>Khung giờ mặc định đã trôi qua (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Mục đích: **đây là hành vi ĐÚNG, không phải bug** — ghi thành TC để lượt sau không log bug oan khi form mở lâu. · Căn cứ: `KB-VIBE-10` (`KP-01` §10.11). ⛔ Không assert giá trị mặc định cụ thể — 3 nguồn cho 3 giá trị khác nhau.</t>
@@ -5172,7 +5272,11 @@
           <t>Bộ dữ liệu xác định ở B1 và B2 (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L40" s="7" t="inlineStr"/>
+      <c r="L40" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M40" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.5.3.</t>
@@ -5247,7 +5351,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L41" s="5" t="inlineStr"/>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M41" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.5.3 + `§A8` L115.</t>
@@ -5322,7 +5430,11 @@
           <t>Checkbox điều khoản mặc định (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L42" s="7" t="inlineStr"/>
+      <c r="L42" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M42" s="7" t="inlineStr">
         <is>
           <t>Mục đích: 2 nguồn trái nhau, và TC `TC_04.71` của đợt cũ expected "tick sẵn" là **sai nguồn**. · Căn cứ: `C-ORD-12` Resolved 2026-09-07 theo `D8.1` L373 + app STG (`KP-01` §10.7); PRD §3.5.3 ghi "mặc định đã tick sẵn" là nguồn thua.</t>
@@ -5401,7 +5513,11 @@
           <t>Checkbox chưa tick và đã tick (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L43" s="5" t="inlineStr"/>
+      <c r="L43" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M43" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `ORD-09` §D3 L245 + `D8.1` L373 — đây là điểm chặn consent bắt buộc, cùng rule với `TC-TS-004`.</t>
@@ -5478,7 +5594,11 @@
           <t>Chip loại hàng "Thuốc/Y tế" (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L44" s="7" t="inlineStr"/>
+      <c r="L44" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M44" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt bằng TC rằng banner hàng cấm ở v1.0 **chỉ là thông tin tĩnh**, không phải cơ chế chặn — để lượt sau không viết TC negative "bị chặn". · Căn cứ: `C-ORD-04` Resolved 2026-07-27 + `KB-ORD-03`; `BR-ORD-04` §D4 L263 là rule của phase sau.</t>
@@ -5557,7 +5677,7 @@
       <c r="L45" s="5" t="inlineStr"/>
       <c r="M45" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `US-D02` §D1b L165.</t>
+          <t>Căn cứ: `US-D02` §D1b L165. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N45" s="5" t="inlineStr">
@@ -5633,7 +5753,11 @@
           <t>2 tin NEED (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L46" s="7" t="inlineStr"/>
+      <c r="L46" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M46" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.5.4.</t>
@@ -5708,7 +5832,11 @@
           <t>Mã tin là giá trị assert-absent (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L47" s="5" t="inlineStr"/>
+      <c r="L47" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M47" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-05` Open — Figma có **2 biến thể** màn này (1 bản có "Mã tin", 1 bản không). · Căn cứ: assert theo `US-D02` §D1b L165 *"KHÔNG hiển thị mã đơn — mã kỹ thuật vô nghĩa với người dùng"* (BRD thắng khi mâu thuẫn về rule). App hiện mã tin ⇒ FAIL và dẫn `C-ORD-05` để BA chốt biến thể.</t>
@@ -5791,7 +5919,11 @@
           <t>Hồ sơ đầy đủ tên + SĐT + nơi làm việc (test_data_catalog §ORD, bảng OFFER)</t>
         </is>
       </c>
-      <c r="L49" s="7" t="inlineStr"/>
+      <c r="L49" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M49" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D10` §D1b L184 + `DOC-v1.0-02` §4.4 + `KB-ORD-11`.</t>
@@ -5871,7 +6003,11 @@
           <t>Điểm xuất phát pre-fill; điểm đến trùng điểm xuất phát (test_data_catalog §ORD, bảng OFFER)</t>
         </is>
       </c>
-      <c r="L50" s="5" t="inlineStr"/>
+      <c r="L50" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M50" s="5" t="inlineStr">
         <is>
           <t>Mục đích: khác biệt cần chốt — điểm xuất phát của OFFER **sửa được**, trong khi tên người gửi của NEED là chỉ đọc (`TC-ORD-016`). · Căn cứ: `D8.2` §D8.2 L381-382.</t>
@@ -5952,7 +6088,7 @@
       <c r="L51" s="7" t="inlineStr"/>
       <c r="M51" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `US-D11` §D1b L185.</t>
+          <t>Căn cứ: `US-D11` §D1b L185. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
@@ -6027,7 +6163,11 @@
           <t>1 tin OFFER (test_data_catalog §ORD, bảng OFFER)</t>
         </is>
       </c>
-      <c r="L52" s="5" t="inlineStr"/>
+      <c r="L52" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M52" s="5" t="inlineStr">
         <is>
           <t>Mục đích: tuyến OFFER là dữ liệu **không công khai** — lộ lên Bảng tin là rò rỉ lịch trình di chuyển của nhân viên. · Căn cứ: `US-D11` §D1b L185 + `ORD-01` §D3 L240.</t>
@@ -6116,7 +6256,7 @@
       <c r="L54" s="7" t="inlineStr"/>
       <c r="M54" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `ORD-10` §D3 L252 + `US-D19` §D1b L169.</t>
+          <t>Căn cứ: `ORD-10` §D3 L252 + `US-D19` §D1b L169. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr">
@@ -6193,7 +6333,7 @@
       <c r="L55" s="5" t="inlineStr"/>
       <c r="M55" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: ranh giới khoá sửa là "Chờ ghép" → "Đã ghép"; cặp với TC-ORD-046. · Căn cứ: `BR-EDIT-01` §D4 L269 + `OPR-10` §D7 L346. Sửa được sau khi ghép ⇒ Carrier đã nhận đơn theo thông tin cũ, log bug mức cao.</t>
+          <t>Mục đích: ranh giới khoá sửa là "Chờ ghép" → "Đã ghép"; cặp với TC-ORD-046. · Căn cứ: `BR-EDIT-01` §D4 L269 + `OPR-10` §D7 L346. Sửa được sau khi ghép ⇒ Carrier đã nhận đơn theo thông tin cũ, log bug mức cao. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N55" s="5" t="inlineStr">
@@ -6269,7 +6409,7 @@
       <c r="L56" s="7" t="inlineStr"/>
       <c r="M56" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `US-D04` §D1b L166 + `KB-ORD-02`. Bản text đầy đủ của dòng lý do assert ở `TC-ACT-008`; TC này chỉ assert transition trạng thái và sự có mặt của lý do.</t>
+          <t>Căn cứ: `US-D04` §D1b L166 + `KB-ORD-02`. Bản text đầy đủ của dòng lý do assert ở `TC-ACT-008`; TC này chỉ assert transition trạng thái và sự có mặt của lý do. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N56" s="7" t="inlineStr">
@@ -6342,7 +6482,11 @@
           <t>1 tin NEED vừa đăng (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L57" s="5" t="inlineStr"/>
+      <c r="L57" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M57" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `ORD-04` §D3 L243.</t>
@@ -6423,7 +6567,11 @@
           <t>Bộ dữ liệu thiếu trường bắt buộc và bộ đủ trường (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L58" s="7" t="inlineStr"/>
+      <c r="L58" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M58" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `VAL-01` §D8.3 L392 — rule áp cho **cả 2 luồng đăng tin**, nên TC kiểm cả hai.</t>
@@ -6502,7 +6650,11 @@
           <t>Tên 1 ký tự; nhiều field lỗi cùng lúc (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L59" s="5" t="inlineStr"/>
+      <c r="L59" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M59" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `VAL-02` §D8.3 L393.</t>
@@ -6579,7 +6731,11 @@
           <t>Tên có khoảng trắng đầu cuối; SĐT "090 123.4567" (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L60" s="7" t="inlineStr"/>
+      <c r="L60" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M60" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `VAL-03` §D8.3 L394. Cùng rule trim với lý do huỷ đơn ở `TC-CNL-012` — nếu TC này PASS mà TC-CNL-012 FAIL thì trim chỉ được áp ở một số form, ghi rõ khi log bug.</t>
@@ -6660,7 +6816,7 @@
       <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: chỉ assert vế có nguồn (điểm vào wizard luôn là bước 1, theo `SC-ORD-002`). · Căn cứ: ⛔ **KHÔNG assert** form giữ hay xoá dữ liệu đã nhập — `C-ORD-08` Open, chưa có đặc tả, áp `§Custom Rules §10.1`. Khi chạy thì ghi lại hành vi thật vào `C-ORD-08` để BA chốt.</t>
+          <t>Mục đích: chỉ assert vế có nguồn (điểm vào wizard luôn là bước 1, theo `SC-ORD-002`). · Căn cứ: ⛔ **KHÔNG assert** form giữ hay xoá dữ liệu đã nhập — `C-ORD-08` Open, chưa có đặc tả, áp `§Custom Rules §10.1`. Khi chạy thì ghi lại hành vi thật vào `C-ORD-08` để BA chốt. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N61" s="5" t="inlineStr">
@@ -6734,7 +6890,11 @@
           <t>Field số tiền là giá trị assert-absent (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L62" s="7" t="inlineStr"/>
+      <c r="L62" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M62" s="7" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding chốt ranh giới dễ trộn nhất của module — ngưỡng bằng **số tiền** (`BR-ORD-03`) out of scope, còn cảnh báo theo **mức định tính "Cao"** thì CÓ ở v1.0 (`TC-ORD-009`). · Căn cứ: `C-ORD-02` Resolved 2026-07-27 (từng là blocker cứng duy nhất của đợt cũ, đã gỡ) + `KB-ORD-04`.</t>
@@ -6935,7 +7095,7 @@
           <t>1 đơn đi thẳng tới "Hoàn thành" (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="n"/>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `TS-01` §A8 L121 + `ORD-04` §D3 L243. ⛔ Không dùng đơn từng bị huỷ nhận — đơn đó thiếu mốc "Ghép thành công" do bug đã biết, sẽ chẩn đoán sai nguyên nhân.</t>
@@ -7011,7 +7171,7 @@
           <t>1 đơn đi thẳng, 3 vai thao tác khác nhau (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="n"/>
       <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `TS-01` §A8 L121 — nhóm thông tin "ai thực hiện". Nhóm thứ 5 của rule (actor + lý do của mốc huỷ) verify ở `TC-CNL-009`, không nhồi vào TC này.</t>
@@ -7092,7 +7252,7 @@
           <t>Đơn `MATCHED` có ≥2 mốc log; 3 hành động thử: huỷ nhận · sửa tin · huỷ đơn (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Mục đích: mở rộng hơn `TC-CNL-010` — không chỉ kiểm 1 hành động đã biết vi phạm mà tìm xem còn đường nào khác cũng làm đổi log. · Căn cứ: `TS-02` §A8 L122 + `BR-INT-04` §A5 L80 (audit bất biến). ⚠ Dự kiến FAIL ở bước 4 — `KB-CNL-01` đã live-verify app XOÁ dòng "Ghép thành công" ⇒ **log bug**; nếu bước 5 hoặc 6 cũng lệch thì log thêm bug riêng cho từng đường.</t>
@@ -7171,7 +7331,7 @@
           <t>Checkbox điều khoản ở NEED B3 và form OFFER (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chỉ assert vế đã chốt (consent ở luồng **đăng tin**). · Căn cứ: `§A8` L115 + `ORD-09` §D3 L245 + `D8.1` L373 + `D8.2` L386. ⚠ Rule `§A8` yêu cầu consent trước khi đăng **VÀ** trước khi ghép, nhưng luồng ghép hiện chỉ có modal xác nhận lộ SĐT — `RISK-TS-04` nghi đây là **gap tuân thủ pháp lý**, đang chờ BA ⇒ ⛔ không assert checkbox ở luồng ghép trong TC này để không trộn 2 phán quyết.</t>
@@ -7251,7 +7411,7 @@
           <t>Cơ chế chặn user dùng làm giá trị assert-absent (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding chứng minh app **đúng phạm vi** — `§A8` L125 khai rõ v1.0 "KHÔNG có chặn (block) người dùng". · Căn cứ: app xuất hiện chức năng này ⇒ FAIL và mở CL scope, không phải log bug.</t>
@@ -7329,7 +7489,7 @@
           <t>1 đơn "Đã giao" quá 4 giờ chưa xác nhận (test_data_catalog §TS — cùng tiền đề `SC-DLV-024`)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chỉ verify **hệ quả phía end-user**; nhánh xử lý của admin thuộc Admin Portal, ⛔ ngoài phạm vi test v1.0. · Căn cứ: `TS-03` §A8 L123 + `BR-CNF-04` §D4 L266 (2 giờ nhắc + 2 giờ admin). Chưa chạy đủ mốc thời gian thì đánh `Blocked` và ghi rõ, ⛔ không đánh PASS.</t>
@@ -7408,7 +7568,7 @@
           <t>Bề mặt Admin dùng làm giá trị assert-absent (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding chốt bằng ID rằng cột `Admin` của permission matrix `§D4` L279-286 **không nằm trong phạm vi test v1.0** — để test report không bị hiểu là đã phủ hết matrix. · Căn cứ: `C-TS-01` Resolved 2026-07-27 (không có đặc tả UI Admin) + `KB-TS-01`.</t>
@@ -7601,7 +7761,11 @@
           <t>Tài khoản SSO CBNV còn hiệu lực (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `USR-01` §A6 — bề mặt đăng nhập thuộc host app FoxPro nên chỉ verify được hệ quả danh tính, không verify được nhánh auth âm tính (`RISK-USR-01`).</t>
@@ -7680,7 +7844,7 @@
       <c r="L3" s="7" t="inlineStr"/>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: chốt đúng 4 trường có bằng chứng 2 nguồn — doc `USR-02` liệt kê 6 trường nhưng SĐT / khu vực-văn phòng / kênh liên hệ chưa có bằng chứng UI. · Căn cứ: `§Custom Rules §10.1` + `RISK-USR-02`; 2 trường thiếu bằng chứng theo dõi ở `C-USR-04`, app hiện thêm trường ⇒ mở lại CL chứ không sửa TC.</t>
+          <t>Mục đích: chốt đúng 4 trường có bằng chứng 2 nguồn — doc `USR-02` liệt kê 6 trường nhưng SĐT / khu vực-văn phòng / kênh liên hệ chưa có bằng chứng UI. · Căn cứ: `§Custom Rules §10.1` + `RISK-USR-02`; 2 trường thiếu bằng chứng theo dõi ở `C-USR-04`, app hiện thêm trường ⇒ mở lại CL chứ không sửa TC. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -7758,7 +7922,7 @@
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: TC bảo vệ kết luận `C-USR-03` (Resolved 2026-07-24 — view-only); app xuất hiện control sửa ⇒ FAIL và mở lại CL, không im lặng viết TC sửa hồ sơ.</t>
+          <t>Mục đích: TC bảo vệ kết luận `C-USR-03` (Resolved 2026-07-24 — view-only); app xuất hiện control sửa ⇒ FAIL và mở lại CL, không im lặng viết TC sửa hồ sơ. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
@@ -7831,7 +7995,11 @@
           <t>Phòng ban + MNV dạng `FTEL####` (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M5" s="7" t="inlineStr"/>
       <c r="N5" s="7" t="inlineStr">
         <is>
@@ -7905,7 +8073,7 @@
           <t>Tài khoản có lịch sử đơn; 1 đơn ở trạng thái đã ghép (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Mục đích: oracle là **delta +1**, không phải số tuyệt đối — 2 chỉ số là dữ liệu `Runtime` không seed nhanh được nên assert số tuyệt đối sẽ FAIL oan (`RISK-USR-03` Resolved theo hướng delta).</t>
@@ -7981,7 +8149,11 @@
           <t>Tài khoản "trắng" — cả 2 chỉ số = 0 (test_data_catalog §USR, biên)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp biên với TC-USR-005 — chốt card hiển thị số 0 chứ không ẩn card. · Căn cứ: `USR-05` §A6 L102 định nghĩa chỉ số là số nguyên ≥ 0; text empty state của màn còn chờ `C-ORD-06` nên TC này chỉ assert sự hiện diện và giá trị 0, app ẩn card ⇒ FAIL và dẫn `C-ORD-06`.</t>
@@ -8057,7 +8229,11 @@
           <t>Bộ giá trị assert-absent: Điểm ECO / Điểm uy tín / CO₂ (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-USR-01` Resolved 2026-07-27 — tier/điểm là phase sau, PRD demo mô tả 3 chỉ số là nguồn thua. App hiện các chỉ số này ⇒ FAIL và mở lại CL.</t>
@@ -8138,7 +8314,7 @@
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: badge có bằng chứng Figma nên assert được, nhưng không có logic tier ở v1.0 (`RISK-USR-04`) ⇒ TC này tồn tại để chặn việc viết TC đổi hạng ở lượt sau.</t>
+          <t>Căn cứ: badge có bằng chứng Figma nên assert được, nhưng không có logic tier ở v1.0 (`RISK-USR-04`) ⇒ TC này tồn tại để chặn việc viết TC đổi hạng ở lượt sau. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
@@ -8211,7 +8387,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr">
         <is>
@@ -8283,7 +8463,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: chỉ assert điều hướng; nội dung màn "Quà đã nhận" thuộc module GIFT (`SC-GIFT-006..009`).</t>
@@ -8359,7 +8543,11 @@
           <t>Bộ giá trị assert-absent: SĐT / Workplace / email cấu hình (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `USR-07` có trong BRD nhưng không có ở 82 ảnh Figma lẫn app STG. · Căn cứ: `C-USR-02` Resolved out of scope v1.0; app xuất hiện bề mặt này ⇒ FAIL và mở lại CL để BA chốt scope.</t>
@@ -8438,7 +8626,7 @@
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: đối chiếu cấu trúc theo ảnh Figma `570ad9d3…` và `e5764b10…`; chỉ đối chiếu thành phần và thứ tự, không đối chiếu giá trị dữ liệu trong ảnh.</t>
+          <t>Căn cứ: đối chiếu cấu trúc theo ảnh Figma `570ad9d3…` và `e5764b10…`; chỉ đối chiếu thành phần và thứ tự, không đối chiếu giá trị dữ liệu trong ảnh. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -8514,7 +8702,7 @@
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 3 nguồn ghi 3 nhãn khác nhau cho cùng mục menu này. · Căn cứ: assert theo nguồn chốt mới nhất là BRD `US-D20` + ảnh Figma; app hiển thị nhãn khác (vd "Đánh giá đã nhận") ⇒ FAIL và báo về `C-USR-04` để BA chốt, ⛔ không tự đổi nhãn trong TC.</t>
+          <t>Mục đích: 3 nguồn ghi 3 nhãn khác nhau cho cùng mục menu này. · Căn cứ: assert theo nguồn chốt mới nhất là BRD `US-D20` + ảnh Figma; app hiển thị nhãn khác (vd "Đánh giá đã nhận") ⇒ FAIL và báo về `C-USR-04` để BA chốt, ⛔ không tự đổi nhãn trong TC. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -8703,7 +8891,11 @@
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
+        </is>
+      </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
           <t>v1.0</t>
@@ -8774,7 +8966,7 @@
           <t>Tab active mặc định (test_data_catalog §ACT, biên "lần đầu mở màn")</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="n"/>
       <c r="M3" s="7" t="inlineStr"/>
       <c r="N3" s="7" t="inlineStr">
         <is>
@@ -8846,7 +9038,7 @@
           <t>4 đơn đang hoạt động + 1 đơn "Hoàn thành" + 1 đơn "Hết hạn" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đây là chỗ TC gộp tab của đợt cũ **không bắt được lỗi** — case gốc sinh `§Custom Rules §10.2`. · Căn cứ: `DOC-v1.0-02` §3.7 đoạn 2; biên cuối của tab là "Đã giao" (`§D2` L232).</t>
@@ -8926,7 +9118,7 @@
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: đơn "Hết hạn" là thứ dễ bị bỏ sót nhất vì tên tab gợi ý chỉ chứa đơn thành công. · Căn cứ: `US-D04` §D1b L166 + `DOC-v1.0-02` §3.7 đoạn 3.</t>
+          <t>Mục đích: đơn "Hết hạn" là thứ dễ bị bỏ sót nhất vì tên tab gợi ý chỉ chứa đơn thành công. · Căn cứ: `US-D04` §D1b L166 + `DOC-v1.0-02` §3.7 đoạn 3. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
@@ -8999,7 +9191,7 @@
           <t>Đơn "Đang giao" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: đối chiếu cấu trúc theo `DOC-v1.0-05`; ⛔ không assert định dạng ngày và không assert cách rút gọn địa chỉ — cả hai chưa có đặc tả.</t>
@@ -9076,7 +9268,7 @@
           <t>1 đơn "Đã huỷ" dùng làm giá trị assert-absent (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Mục đích: rule ẩn đơn huỷ đối lập trực tiếp với `TS-01` (log tương tác đầy đủ) — đơn biến mất khỏi cả 2 tab là hành vi đã quan sát, cần chốt bằng TC có ID. · Căn cứ: `KB-ORD-07` (#7); đơn huỷ hiện ở 1 trong 2 tab ⇒ FAIL và mở CL để BA chốt tab nào chứa.</t>
@@ -9153,7 +9345,7 @@
           <t>2 đơn đang hoạt động khác nhau của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Mục đích: assert theo **dữ liệu của đơn**, cố ý không assert tên màn đích — tên màn còn tranh chấp ở `C-ACT-01` và do TC-ACT-011 đảm nhiệm.</t>
@@ -9231,7 +9423,7 @@
           <t>Đơn "Đang giao" + đơn "Hoàn thành" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Mục đích: TC này verify **cơ chế switch**, cố ý KHÔNG verify nội dung data của từng tab — nội dung do TC-ACT-004 và TC-ACT-005 đảm nhiệm (`§Custom Rules §10.2`).</t>
@@ -9310,7 +9502,7 @@
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn lệch phần cuối câu lý do. · Căn cứ: assert theo `KB-ORD-07` (#4) vì đây là nguyên văn quan sát trên app kèm bằng chứng; `US-D04` L166 ghi bản ngắn hơn (dừng ở "trong thời gian đăng") là nguồn thua. App hiện bản ngắn ⇒ FAIL và mở CL để BA chốt bản text chính thức.</t>
+          <t>Mục đích: 2 nguồn lệch phần cuối câu lý do. · Căn cứ: assert theo `KB-ORD-07` (#4) vì đây là nguyên văn quan sát trên app kèm bằng chứng; `US-D04` L166 ghi bản ngắn hơn (dừng ở "trong thời gian đăng") là nguồn thua. App hiện bản ngắn ⇒ FAIL và mở CL để BA chốt bản text chính thức. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
@@ -9383,7 +9575,7 @@
           <t>Đơn "Hết hạn" của `SEED-ACT-01`, dùng chung với TC-ACT-008 (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-ACT-010 — card thao tác được vs không thao tác được.</t>
@@ -9460,7 +9652,7 @@
           <t>1 đơn "Chờ ghép" của chính tài khoản (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Mục đích: 2 nguồn nêu 2 màn **khác bản chất** ("Chi tiết tin" public vs "Theo dõi đơn" role-aware). · Căn cứ: assert theo `DOC-v1.0-02` §3.7 + tính nhất quán với `SC-HOME-015` (Trang chủ đã rõ là mở Theo dõi đơn); `KB-ORD-07` (#5) nghi ghi nhầm tên màn. Nếu app mở Chi tiết tin và hiện nút "Tôi mang giúp được" trên đơn của chính mình ⇒ FAIL, log bug theo cùng gốc với `C-ASN-02` và dẫn `C-ACT-01`.</t>
@@ -9540,7 +9732,7 @@
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-ORD-06` Open — module này là **home canonical** của CL, text empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được; ⛔ không assert chuỗi hay ảnh empty state.</t>
+          <t>Mục đích: neo vào `C-ORD-06` Open — module này là **home canonical** của CL, text empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được; ⛔ không assert chuỗi hay ảnh empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -9616,7 +9808,7 @@
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: chuỗi "★★★★★ Đã đánh giá" trên card là **UI leftover**, dễ khiến người sau viết TC chấm sao. · Căn cứ: `C-GIFT-01` Resolved 2026-07-27 — rating 1–5 sao out of scope v1.0, v1.0 chỉ có Quà ảo; ⛔ không assert số sao và không assert sự tồn tại của chuỗi leftover. App mở được màn chấm sao ⇒ FAIL và mở lại CL scope.</t>
+          <t>Mục đích: chuỗi "★★★★★ Đã đánh giá" trên card là **UI leftover**, dễ khiến người sau viết TC chấm sao. · Căn cứ: `C-GIFT-01` Resolved 2026-07-27 — rating 1–5 sao out of scope v1.0, v1.0 chỉ có Quà ảo; ⛔ không assert số sao và không assert sự tồn tại của chuỗi leftover. App mở được màn chấm sao ⇒ FAIL và mở lại CL scope. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -9694,7 +9886,7 @@
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: cặp với TC-ACT-012 — empty state phải verify riêng cho từng tab (`§Custom Rules §10.2`). · Căn cứ: `C-ORD-06` Open ⇒ ⛔ không assert chuỗi empty state.</t>
+          <t>Mục đích: cặp với TC-ACT-012 — empty state phải verify riêng cho từng tab (`§Custom Rules §10.2`). · Căn cứ: `C-ORD-06` Open ⇒ ⛔ không assert chuỗi empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -9770,7 +9962,11 @@
           <t>1 tin NEED `POSTED` của tài khoản khác (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-CON-01` §A5 L77 — transition duy nhất của module là `POSTED` → `MATCHED`.</t>
@@ -9848,7 +10044,11 @@
           <t>1 tin NEED `POSTED`; 2 tài khoản 2 thiết bị (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-CON-01` §A5 L77 — cơ chế "ghép ngay", không có bước duyệt.</t>
@@ -9926,7 +10126,11 @@
           <t>1 đơn `MATCHED` có khai người nhận (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-CON-02` §A5 L78 + `OPR-07` §D7 L343 + `US-D08` L177 (Carrier thấy cả SĐT người nhận). Đây là vế dương của cặp với TC-ASN-005.</t>
@@ -10008,7 +10212,7 @@
       <c r="L19" s="7" t="inlineStr"/>
       <c r="M19" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: chống double-accept là rủi ro P1 — 2 Carrier cùng nhận sẽ phá tính duy nhất của cặp ghép. · Căn cứ: `ASN-03` §D3 L249 + `OPR-03` §D7 L339. Với 1 tester chỉ kiểm được nhánh gần đồng thời bằng 2 thiết bị; nếu cả hai đều báo thành công ⇒ FAIL và log bug.</t>
+          <t>Mục đích: chống double-accept là rủi ro P1 — 2 Carrier cùng nhận sẽ phá tính duy nhất của cặp ghép. · Căn cứ: `ASN-03` §D3 L249 + `OPR-03` §D7 L339. Với 1 tester chỉ kiểm được nhánh gần đồng thời bằng 2 thiết bị; nếu cả hai đều báo thành công ⇒ FAIL và log bug. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
@@ -10083,7 +10287,11 @@
           <t>1 đơn `MATCHED` (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M20" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-03` §D7 L339 + `OPR-08` §D7 L344.</t>
@@ -10161,7 +10369,11 @@
           <t>1 tin OFFER + 1 tin NEED cùng tài khoản, trùng tuyến (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L21" s="7" t="inlineStr"/>
+      <c r="L21" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M21" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-05` §D7 L341 — cùng gốc rule với `SC-FEED-011`; app gợi ý tin của chính mình ⇒ FAIL và log bug theo cùng `C-ASN-02`.</t>
@@ -10240,7 +10452,11 @@
           <t>1 tin NEED `POSTED` (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M22" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng âm của TC-ASN-001 — modal phải huỷ được mà không tạo tác động.</t>
@@ -10318,7 +10534,11 @@
           <t>1 đơn `MATCHED`; 1 tài khoản ngoài cặp (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L23" s="7" t="inlineStr"/>
+      <c r="L23" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M23" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng âm của TC-ASN-004 — quyền xem SĐT bị giới hạn đúng trong cặp ghép cộng người nhận.</t>
@@ -10399,7 +10619,7 @@
       <c r="L24" s="5" t="inlineStr"/>
       <c r="M24" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `BR-INT-05` §A5 L81 + `DOC-v1.0-02` §4.2. Không assert độ trễ cụ thể — chưa có đặc tả ngưỡng thời gian.</t>
+          <t>Căn cứ: `BR-INT-05` §A5 L81 + `DOC-v1.0-02` §4.2. Không assert độ trễ cụ thể — chưa có đặc tả ngưỡng thời gian. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
@@ -10474,7 +10694,11 @@
           <t>1 tin OFFER + 1 tin NEED trùng 2 điểm, khung giờ giao nhau (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L25" s="7" t="inlineStr"/>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M25" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `MTCH-01` §D3 L254 + `US-D12` §D1b L186. Nội dung thông báo còn chờ `C-NTF-01` chốt danh sách chính thức; assert theo chuỗi ở `US-D12`, lệch ⇒ dẫn `C-NTF-01`.</t>
@@ -10553,7 +10777,11 @@
           <t>1 tin NEED khớp tuyến (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D13` §D1b L187. Nhãn nút "Nhận giao" ở luồng khớp tuyến khác nhãn "Tôi mang giúp được" ở luồng Bảng tin — giữ đúng nhãn từng luồng, ⛔ không đồng nhất hoá.</t>
@@ -10632,7 +10860,7 @@
       <c r="L27" s="7" t="inlineStr"/>
       <c r="M27" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: 1 trong 2 nhánh negative mà `SC-ASN-011` nêu — nhánh lệch địa điểm. · Căn cứ: `OPR-02` §D7 L338 + `KB-ASN-04` — khớp tuyến là **nhị phân trùng địa chỉ**, ⛔ không dùng bán kính GPS.</t>
+          <t>Mục đích: 1 trong 2 nhánh negative mà `SC-ASN-011` nêu — nhánh lệch địa điểm. · Căn cứ: `OPR-02` §D7 L338 + `KB-ASN-04` — khớp tuyến là **nhị phân trùng địa chỉ**, ⛔ không dùng bán kính GPS. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
@@ -10708,7 +10936,7 @@
       <c r="L28" s="5" t="inlineStr"/>
       <c r="M28" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh negative thứ hai của `SC-ASN-011` — lệch khung giờ. · Căn cứ: chỉ dùng 2 khung **tách rời hoàn toàn**; ⛔ không test độ lệch nhỏ vì định nghĩa "khung giờ phù hợp" chưa chốt (`C-NTF-02` Partially Resolved).</t>
+          <t>Mục đích: nhánh negative thứ hai của `SC-ASN-011` — lệch khung giờ. · Căn cứ: chỉ dùng 2 khung **tách rời hoàn toàn**; ⛔ không test độ lệch nhỏ vì định nghĩa "khung giờ phù hợp" chưa chốt (`C-NTF-02` Partially Resolved). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
@@ -10782,7 +11010,11 @@
           <t>6 tin NEED khớp cùng 1 tuyến OFFER (test_data_catalog §ASN, biên vượt trần)</t>
         </is>
       </c>
-      <c r="L29" s="7" t="inlineStr"/>
+      <c r="L29" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M29" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chạm trần gợi ý — dùng mốc 6 để vượt trần 5. · Căn cứ: `OPR-01` §D7 L337; mốc 3/5/6 là **giá trị BA chốt** (`KB-ASN-03`), ⛔ không thay bằng mốc khác.</t>
@@ -10861,7 +11093,7 @@
       <c r="L30" s="5" t="inlineStr"/>
       <c r="M30" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: mốc dưới trần trong bộ ba 3/5/6 — đối chứng để phân biệt "chặn vì trần" với "không bắn thông báo".</t>
+          <t>Mục đích: mốc dưới trần trong bộ ba 3/5/6 — đối chứng để phân biệt "chặn vì trần" với "không bắn thông báo". · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N30" s="5" t="inlineStr">
@@ -10937,7 +11169,7 @@
       <c r="L31" s="7" t="inlineStr"/>
       <c r="M31" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: mốc đúng trần — biên hợp lệ, cặp với TC-ASN-017 (mốc vượt trần).</t>
+          <t>Mục đích: mốc đúng trần — biên hợp lệ, cặp với TC-ASN-017 (mốc vượt trần). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr">
@@ -11015,7 +11247,7 @@
       <c r="L32" s="5" t="inlineStr"/>
       <c r="M32" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: mốc vượt trần — chốt trần tính **riêng theo từng tin OFFER**. · Căn cứ: `KB-ASN-03` (đảo `OPR-06`) — ⛔ trần KHÔNG cộng dồn theo ngày; nếu app chặn theo ngày ⇒ FAIL và mở CL.</t>
+          <t>Mục đích: mốc vượt trần — chốt trần tính **riêng theo từng tin OFFER**. · Căn cứ: `KB-ASN-03` (đảo `OPR-06`) — ⛔ trần KHÔNG cộng dồn theo ngày; nếu app chặn theo ngày ⇒ FAIL và mở CL. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N32" s="5" t="inlineStr">
@@ -11090,7 +11322,11 @@
           <t>1 tin NEED "Hết hạn" (test_data_catalog §ASN — ⛔ không seed được qua UI)</t>
         </is>
       </c>
-      <c r="L33" s="7" t="inlineStr"/>
+      <c r="L33" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M33" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-04` §D7 L340 + `US-D04` L166.</t>
@@ -11170,7 +11406,11 @@
           <t>1 đơn `MATCHED` chưa lấy hàng (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M34" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-08` §D7 L344 + `OPR-09` §D7 L345. Nhánh huỷ nhận sau "Đang giao" bị chặn — verify ở `TC-CNL-*`.</t>
@@ -11249,7 +11489,7 @@
       <c r="L35" s="7" t="inlineStr"/>
       <c r="M35" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `OPR-04` §D7 L340 nêu 2 tiêu chí nhưng "độ gần tuyến" là **nhị phân trùng/không trùng** nên không phân biệt được thứ tự ⇒ chỉ còn thời gian đăng làm oracle kiểm chứng được.</t>
+          <t>Căn cứ: `OPR-04` §D7 L340 nêu 2 tiêu chí nhưng "độ gần tuyến" là **nhị phân trùng/không trùng** nên không phân biệt được thứ tự ⇒ chỉ còn thời gian đăng làm oracle kiểm chứng được. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
@@ -11323,7 +11563,11 @@
           <t>2 tin NEED liên tiếp cùng tài khoản (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L36" s="5" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ASN-03` Open — nghi vấn wizard không tạo listing độc lập. · Căn cứ: `DOC-v1.0-02` §7 dòng 3 ghi "Đăng tin mới sẽ ghi đè đơn đang có" nhưng đó là **giới hạn bản demo**, không phải rule nghiệp vụ (`KB-ASN-05`); assert theo hành vi nghiệp vụ đúng. App ghi đè tin cũ ⇒ FAIL và dẫn `C-ASN-03` để BA xác nhận là giới hạn demo hay bug thật.</t>
@@ -11403,7 +11647,7 @@
           <t>Đơn `POSTED`; lý do ≥5 ký tự (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L37" s="7" t="inlineStr"/>
+      <c r="L37" s="7" t="n"/>
       <c r="M37" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D16` §D1b L195 + `OPR-11` §D7 L347.</t>
@@ -11483,7 +11727,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng; 3 tài khoản 3 vai (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="n"/>
       <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-INT-05` §A5 L81 + `OPR-11` §D7 L347 — quyền huỷ của người gửi còn hiệu lực tới trước "Đang giao".</t>
@@ -11562,7 +11806,7 @@
           <t>Đơn `IN_TRANSIT`; 3 tài khoản 3 vai (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr"/>
+      <c r="L39" s="7" t="n"/>
       <c r="M39" s="7" t="inlineStr">
         <is>
           <t>Mục đích: phủ hàng "Đang giao" của ma trận quyền huỷ — ranh giới mất quyền huỷ là "Đã ghép" → "Đang giao". · Căn cứ: `OPR-11` §D7 L347 "KHÔNG ai được huỷ" + `BR-ASN-03` §D4 L264.</t>
@@ -11641,7 +11885,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="n"/>
       <c r="M40" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt khác biệt cốt lõi giữa "Huỷ nhận đơn" (về `POSTED`) và "Huỷ đơn" (`CANCELLED`). · Căn cứ: `OPR-09` §D7 L345 + `US-D16` §D1b L195.</t>
@@ -11720,7 +11964,7 @@
           <t>Lý do rỗng và lý do ≥5 ký tự (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L41" s="7" t="inlineStr"/>
+      <c r="L41" s="7" t="n"/>
       <c r="M41" s="7" t="inlineStr">
         <is>
           <t>Mục đích: mốc "rỗng" là mốc duy nhất trong 4 mốc lý do mà app chặn đúng — dùng làm đối chứng dương cho TC-CNL-004 và TC-CNL-012.</t>
@@ -11801,7 +12045,7 @@
       <c r="L42" s="5" t="inlineStr"/>
       <c r="M42" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: cặp biên 4↔5 ký tự của `VAL-04`. · Căn cứ: `VAL-04` §D8.3 L395 yêu cầu tối thiểu 5 ký tự; `KB-CNL-02` đã live-verify app **chỉ chặn khi rỗng**. ⚠ Dự kiến FAIL ở bước 3 ⇒ **log bug** (tương ứng `TC_08.7` đợt cũ), ⛔ không hạ chuẩn TC theo hành vi app.</t>
+          <t>Mục đích: cặp biên 4↔5 ký tự của `VAL-04`. · Căn cứ: `VAL-04` §D8.3 L395 yêu cầu tối thiểu 5 ký tự; `KB-CNL-02` đã live-verify app **chỉ chặn khi rỗng**. ⚠ Dự kiến FAIL ở bước 3 ⇒ **log bug** (tương ứng `TC_08.7` đợt cũ), ⛔ không hạ chuẩn TC theo hành vi app. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N42" s="5" t="inlineStr">
@@ -11877,7 +12121,7 @@
           <t>Đơn `MATCHED`; lý do ≥5 ký tự (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L43" s="7" t="inlineStr"/>
+      <c r="L43" s="7" t="n"/>
       <c r="M43" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§D2` L233 + `CNL-01` §D3 L257. Danh sách loại thông báo chính thức còn chờ `C-NTF-01`; lệch nội dung thông báo ⇒ dẫn `C-NTF-01`, không sửa TC.</t>
@@ -11957,7 +12201,7 @@
       <c r="L44" s="5" t="inlineStr"/>
       <c r="M44" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-CNL-02` Resolved 2026-07-30 — user chốt **PHẢI ghi log** cho cả 2 hành động huỷ. · Căn cứ: `TS-01`/`TS-02` L121-122 + `KB-CNL-01`; banner đỏ **không thay thế** được log. ⚠ Dự kiến FAIL — app hiện chỉ hiện banner ⇒ **log bug** (tương ứng `TC_08.22` đợt cũ).</t>
+          <t>Mục đích: neo vào `C-CNL-02` Resolved 2026-07-30 — user chốt **PHẢI ghi log** cho cả 2 hành động huỷ. · Căn cứ: `TS-01`/`TS-02` L121-122 + `KB-CNL-01`; banner đỏ **không thay thế** được log. ⚠ Dự kiến FAIL — app hiện chỉ hiện banner ⇒ **log bug** (tương ứng `TC_08.22` đợt cũ). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N44" s="5" t="inlineStr">
@@ -12036,7 +12280,7 @@
       <c r="L45" s="7" t="inlineStr"/>
       <c r="M45" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: log phải **bất biến** — xoá dòng cũ là phá tính bằng chứng của cả timeline. · Căn cứ: `BR-INT-04` §A5 L80 (audit) + `C-CNL-02`; `KB-CNL-01` đã live-verify app **XOÁ** dòng "Ghép thành công". ⚠ Dự kiến FAIL ⇒ **log bug** (tương ứng `TC_08.23` đợt cũ), cùng gốc với `RISK-TS-01`.</t>
+          <t>Mục đích: log phải **bất biến** — xoá dòng cũ là phá tính bằng chứng của cả timeline. · Căn cứ: `BR-INT-04` §A5 L80 (audit) + `C-CNL-02`; `KB-CNL-01` đã live-verify app **XOÁ** dòng "Ghép thành công". ⚠ Dự kiến FAIL ⇒ **log bug** (tương ứng `TC_08.23` đợt cũ), cùng gốc với `RISK-TS-01`. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N45" s="7" t="inlineStr">
@@ -12111,7 +12355,7 @@
           <t>Đơn `MATCHED`; 3 phiên 3 vai trên 3 thiết bị (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="n"/>
       <c r="M46" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-INT-05` §A5 L81 + `§D2` L233. Không assert độ trễ cụ thể — chưa có đặc tả ngưỡng.</t>
@@ -12190,7 +12434,7 @@
           <t>Đơn `POSTED` có khai người nhận (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L47" s="7" t="inlineStr"/>
+      <c r="L47" s="7" t="n"/>
       <c r="M47" s="7" t="inlineStr">
         <is>
           <t>Mục đích: phủ hàng "Chờ ghép" của ma trận quyền huỷ 3 vai × 3 trạng thái. · Căn cứ: permission matrix `§D4` L285 + `OPR-11` §D7 L347 — người gửi và người nhận huỷ được trước "Đang giao"; ở trạng thái này đơn chưa có người vận chuyển nên hàng Carrier không áp dụng. Vai `Admin` trong matrix ⛔ không test được (`C-TS-01` out of scope).</t>
@@ -12270,7 +12514,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng; 3 tài khoản 3 vai (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="n"/>
       <c r="M48" s="5" t="inlineStr">
         <is>
           <t>Mục đích: phủ hàng "Đã ghép" của ma trận — đây là trạng thái duy nhất cả 3 vai đều có đường huỷ, nhưng **Carrier dùng hành động khác** (huỷ nhận, không phải huỷ đơn). · Căn cứ: permission matrix `§D4` L285 + `OPR-09` §D7 L345.</t>
@@ -12352,7 +12596,7 @@
       <c r="L49" s="7" t="inlineStr"/>
       <c r="M49" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `BR-ASN-03` yêu cầu "phải tạo sự cố" thay cho huỷ thường nhưng bề mặt này không có đặc tả. · Căn cứ: `C-CNL-01` Resolved 2026-07-27 out of scope v1.0. **Hệ quả cần nêu với PM:** user gặp sự cố sau khi đã lấy hàng thì không có đường xử lý nào trong app.</t>
+          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `BR-ASN-03` yêu cầu "phải tạo sự cố" thay cho huỷ thường nhưng bề mặt này không có đặc tả. · Căn cứ: `C-CNL-01` Resolved 2026-07-27 out of scope v1.0. **Hệ quả cần nêu với PM:** user gặp sự cố sau khi đã lấy hàng thì không có đường xử lý nào trong app. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr">
@@ -12429,7 +12673,7 @@
       <c r="L50" s="5" t="inlineStr"/>
       <c r="M50" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: mốc thứ tư trong bộ boundary lý do (rỗng → 4 ký tự → 5 ký tự → 5 dấu cách). · Căn cứ: `VAL-03` §D8.3 L394 (trim) + `VAL-04` L395 — sau khi trim thì lý do rỗng. ⚠ Dự kiến FAIL — `KB-CNL-02` đã live-verify app cho qua ⇒ **log bug** (tương ứng `TC_08.10` đợt cũ).</t>
+          <t>Mục đích: mốc thứ tư trong bộ boundary lý do (rỗng → 4 ký tự → 5 ký tự → 5 dấu cách). · Căn cứ: `VAL-03` §D8.3 L394 (trim) + `VAL-04` L395 — sau khi trim thì lý do rỗng. ⚠ Dự kiến FAIL — `KB-CNL-02` đã live-verify app cho qua ⇒ **log bug** (tương ứng `TC_08.10` đợt cũ). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N50" s="5" t="inlineStr">
@@ -12502,7 +12746,11 @@
           <t>Đơn `DELIVERED`; vai Receiver (test_data_catalog §DLV — ô 4·Receiver)</t>
         </is>
       </c>
-      <c r="L51" s="7" t="inlineStr"/>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M51" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đây là **nút enable duy nhất** ở trạng thái "Đã giao" trong 3 vai; nếu ô này disable thì đơn không bao giờ hoàn tất được và toàn bộ module `GIFT` bị blocked. · Căn cứ: `KB-DLV-01` ô 4·Receiver + `DOC-v1.0-02` §5.2 + `C-DLV-01` Resolved (Receiver-only).</t>
@@ -12582,7 +12830,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L52" s="5" t="inlineStr"/>
+      <c r="L52" s="5" t="n"/>
       <c r="M52" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC này khác `TC-DLV-005` — TC-DLV-005 assert **nhãn nút đúng**, TC này assert **không tồn tại đường vòng nào** (mở từ màn khác, nút ẩn). · Căn cứ: `US-D09` §D1b L178. Nhảy bước được ⇒ đơn "đã giao" mà chưa từng lấy hàng, phá tính bằng chứng của timeline và cả `TS-01`.</t>
@@ -12661,7 +12909,7 @@
           <t>Đơn `DELIVERED`; 3 tài khoản 3 vai (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L53" s="7" t="inlineStr"/>
+      <c r="L53" s="7" t="n"/>
       <c r="M53" s="7" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-DLV-01` Resolved 2026-07-24 — `DLV-03` §D3 ghi "RECEIVER/**SENDER**" nhưng `BR-INT-03` §A5 L79 + demo §5.2 + 5 ảnh Figma đều cho **Receiver-only**. · Căn cứ: nguồn chốt là `BR-INT-03` + bằng chứng Figma; app cho Sender chốt đơn ⇒ FAIL và mở lại CL.</t>
@@ -12738,7 +12986,7 @@
           <t>Đơn `DELIVERED` (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L54" s="5" t="inlineStr"/>
+      <c r="L54" s="5" t="n"/>
       <c r="M54" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đây là điểm đóng đơn — nếu có bước chờ ẩn thì người gửi không bao giờ tặng quà được và module `GIFT` bị blocked. · Căn cứ: `DOC-v1.0-02` §5.2 dòng "Sau khi xác nhận". ⛔ Không assert chuỗi "Hoàn thành &amp; đã đánh giá" — chuỗi đó là UI leftover của cơ chế rating đã bị `C-GIFT-01` loại khỏi v1.0.</t>
@@ -12816,7 +13064,11 @@
           <t>Đơn `POSTED`; vai Sender (test_data_catalog §DLV — ô 1·Sender)</t>
         </is>
       </c>
-      <c r="L55" s="7" t="inlineStr"/>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M55" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 1·Sender + ảnh Figma `dc8cf987…`.</t>
@@ -12893,7 +13145,7 @@
           <t>Đơn `POSTED`; vai Carrier (test_data_catalog §DLV — ô 1·Carrier)</t>
         </is>
       </c>
-      <c r="L56" s="5" t="inlineStr"/>
+      <c r="L56" s="5" t="n"/>
       <c r="M56" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 1·Carrier. ⚠ Ô ma trận này nằm ở màn **Chi tiết tin**, không phải màn Theo dõi đơn — Carrier chưa thuộc đơn nên chưa có màn Theo dõi đơn.</t>
@@ -12971,7 +13223,7 @@
           <t>Đơn `POSTED`; vai Receiver (test_data_catalog §DLV — ô 1·Receiver)</t>
         </is>
       </c>
-      <c r="L57" s="7" t="inlineStr"/>
+      <c r="L57" s="7" t="n"/>
       <c r="M57" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 1·Receiver — quyền "Chỉnh sửa" chỉ thuộc người gửi.</t>
@@ -13050,7 +13302,7 @@
           <t>Đơn `MATCHED`; vai Sender (test_data_catalog §DLV — ô 2·Sender)</t>
         </is>
       </c>
-      <c r="L58" s="5" t="inlineStr"/>
+      <c r="L58" s="5" t="n"/>
       <c r="M58" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt thời điểm mất quyền "Chỉnh sửa" là khi đơn được ghép — cặp với TC-DLV-001. · Căn cứ: `KB-DLV-01` ô 2·Sender.</t>
@@ -13129,7 +13381,7 @@
           <t>Đơn `MATCHED`; vai Carrier (test_data_catalog §DLV — ô 2·Carrier)</t>
         </is>
       </c>
-      <c r="L59" s="7" t="inlineStr"/>
+      <c r="L59" s="7" t="n"/>
       <c r="M59" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 2·Carrier + ảnh Figma `2e2ff7bc…`.</t>
@@ -13208,7 +13460,7 @@
           <t>Đơn `MATCHED`; vai Receiver (test_data_catalog §DLV — ô 2·Receiver)</t>
         </is>
       </c>
-      <c r="L60" s="5" t="inlineStr"/>
+      <c r="L60" s="5" t="n"/>
       <c r="M60" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 2·Receiver.</t>
@@ -13286,7 +13538,7 @@
           <t>Đơn `IN_TRANSIT`; vai Sender (test_data_catalog §DLV — ô 3·Sender)</t>
         </is>
       </c>
-      <c r="L61" s="7" t="inlineStr"/>
+      <c r="L61" s="7" t="n"/>
       <c r="M61" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt ranh giới mất quyền huỷ là "Đã ghép" → "Đang giao" — cùng rule với `TC-CNL-005`. · Căn cứ: `KB-DLV-01` ô 3·Sender + ảnh Figma `c8cae4c3…`.</t>
@@ -13362,7 +13614,11 @@
           <t>Đơn `IN_TRANSIT`; vai Carrier (test_data_catalog §DLV — ô 3·Carrier)</t>
         </is>
       </c>
-      <c r="L62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M62" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 3·Carrier.</t>
@@ -13438,7 +13694,11 @@
           <t>Đơn `IN_TRANSIT`; vai Receiver (test_data_catalog §DLV — ô 3·Receiver)</t>
         </is>
       </c>
-      <c r="L63" s="7" t="inlineStr"/>
+      <c r="L63" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M63" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 3·Receiver + ảnh Figma `ca5e7239…`.</t>
@@ -13514,7 +13774,11 @@
           <t>Đơn `DELIVERED`; vai Sender (test_data_catalog §DLV — ô 4·Sender)</t>
         </is>
       </c>
-      <c r="L64" s="5" t="inlineStr"/>
+      <c r="L64" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M64" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 4·Sender + ảnh Figma `8563adc1…`.</t>
@@ -13592,7 +13856,11 @@
           <t>Đơn `DELIVERED`; vai Carrier (test_data_catalog §DLV — ô 4·Carrier)</t>
         </is>
       </c>
-      <c r="L65" s="7" t="inlineStr"/>
+      <c r="L65" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M65" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt quyền hoàn tất đơn đã chuyển sang người nhận — bộ ba TC-DLV-010/011/012 là điểm phân định của `C-DLV-01`. · Căn cứ: `KB-DLV-01` ô 4·Carrier + `DOC-v1.0-02` §4.3.</t>
@@ -13668,7 +13936,7 @@
           <t>Đơn `COMPLETED` chưa gửi quà; vai Sender (test_data_catalog §DLV — ô 5·Sender)</t>
         </is>
       </c>
-      <c r="L66" s="5" t="inlineStr"/>
+      <c r="L66" s="5" t="n"/>
       <c r="M66" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 5·Sender + ảnh Figma `19490aa9…`. Nhãn sau khi gửi quà đổi thành "Bạn đã đánh giá" — verify ở `TC-GIFT-005`.</t>
@@ -13744,7 +14012,11 @@
           <t>Đơn `COMPLETED`; vai Carrier (test_data_catalog §DLV — ô 5·Carrier)</t>
         </is>
       </c>
-      <c r="L67" s="7" t="inlineStr"/>
+      <c r="L67" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M67" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 5·Carrier + ảnh Figma `2658b17b…`.</t>
@@ -13820,7 +14092,11 @@
           <t>Đơn `COMPLETED`; vai Receiver (test_data_catalog §DLV — ô 5·Receiver)</t>
         </is>
       </c>
-      <c r="L68" s="5" t="inlineStr"/>
+      <c r="L68" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M68" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 5·Receiver + ảnh Figma `76e115a2…`.</t>
@@ -13899,7 +14175,7 @@
           <t>Đơn qua 3 trạng thái đầu (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L69" s="7" t="inlineStr"/>
+      <c r="L69" s="7" t="n"/>
       <c r="M69" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D09` §D1b L178 + `§D2` L232. ⚠ Mốc thứ hai trên thanh ghi "Lấy hàng" trong khi badge trạng thái ghi "Đã ghép" — 2 chữ cho cùng 1 trạng thái, ⛔ không sửa TC theo chữ của badge.</t>
@@ -13978,7 +14254,7 @@
           <t>Đơn `MATCHED`; nội dung popup lấy hàng (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L70" s="5" t="inlineStr"/>
+      <c r="L70" s="5" t="n"/>
       <c r="M70" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` bảng popup — tiêu đề popup cố định là "Xác nhận" cho cả 3 hành động.</t>
@@ -14057,7 +14333,7 @@
           <t>Đơn `IN_TRANSIT`; nội dung popup đã giao (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L71" s="7" t="inlineStr"/>
+      <c r="L71" s="7" t="n"/>
       <c r="M71" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` bảng popup.</t>
@@ -14136,7 +14412,7 @@
           <t>Đơn `DELIVERED`; nội dung popup nhận hàng (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L72" s="5" t="inlineStr"/>
+      <c r="L72" s="5" t="n"/>
       <c r="M72" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` bảng popup + `KB-DLV-03`.</t>
@@ -14215,7 +14491,7 @@
           <t>Đơn `MATCHED` (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L73" s="7" t="inlineStr"/>
+      <c r="L73" s="7" t="n"/>
       <c r="M73" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng âm cho TC-DLV-017 — popup phải huỷ được mà không tạo tác động, kể cả tác động lên log. · Căn cứ: `DOC-v1.0-02` §6 L191.</t>
@@ -14293,7 +14569,7 @@
           <t>Đơn `DELIVERED` với mốc thời gian 2 giờ và 4 giờ (test_data_catalog §DLV — cần dev seed timestamp)</t>
         </is>
       </c>
-      <c r="L74" s="5" t="inlineStr"/>
+      <c r="L74" s="5" t="n"/>
       <c r="M74" s="5" t="inlineStr">
         <is>
           <t>Mục đích: dùng chung tiền đề với `SC-TS-006` ⇒ chạy 1 lần lấy dữ liệu cho cả 2 TC. · Căn cứ: `BR-CNF-04` §D4 L266 + `US-D14` §D1b L193; nhánh xử lý của admin thuộc Admin Portal, ⛔ ngoài phạm vi v1.0. Chưa chạy đủ mốc thời gian thì đánh `Blocked` và ghi rõ, ⛔ không đánh PASS cho xong.</t>
@@ -14369,7 +14645,7 @@
           <t>Bộ giá trị assert-absent: ảnh bằng chứng / điểm uy tín / chi phí (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L75" s="7" t="inlineStr"/>
+      <c r="L75" s="7" t="n"/>
       <c r="M75" s="7" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-DLV-03` Resolved 2026-07-27 — form đầy đủ ở PRD §5.3 **không áp dụng v1.0**. · Căn cứ: `KB-DLV-03` (bằng chứng app dùng modal đơn giản); app hiện form đầy đủ ⇒ FAIL và mở lại CL scope.</t>
@@ -14447,7 +14723,11 @@
           <t>Đơn qua `POSTED` → `MATCHED`; vai Sender (test_data_catalog §DLV, biên thời điểm lộ liên hệ)</t>
         </is>
       </c>
-      <c r="L76" s="5" t="inlineStr"/>
+      <c r="L76" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M76" s="5" t="inlineStr">
         <is>
           <t>Mục đích: ranh giới "Chờ ghép" → "Đã ghép" là thời điểm cụm liên hệ được phép xuất hiện — cùng rule với `TC-FEED-010`. · Căn cứ: `DOC-v1.0-02` §3.6 + `BR-CON-02` §A5 L78.</t>
@@ -14523,7 +14803,11 @@
           <t>Đơn `MATCHED` có khai người nhận; vai Carrier (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L77" s="7" t="inlineStr"/>
+      <c r="L77" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M77" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §4.3 + `US-D08` §D1b L177 — người vận chuyển là vai duy nhất thấy liên hệ 2 đầu.</t>
@@ -14600,7 +14884,11 @@
           <t>Đơn `MATCHED`; vai Receiver (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L78" s="5" t="n"/>
+      <c r="L78" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M78" s="5" t="inlineStr">
         <is>
           <t>Mục đích: giới hạn phạm vi lộ liên hệ theo vai — người nhận không có nhu cầu liên hệ người gửi trong luồng v1.0. · Căn cứ: `DOC-v1.0-02` §5.2 dòng "Liên hệ".</t>
@@ -14676,7 +14964,11 @@
           <t>Đơn đi thẳng tới `COMPLETED` (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L79" s="7" t="inlineStr"/>
+      <c r="L79" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M79" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.6 dòng "Lịch sử" + `US-D09` §D1b L178. ⚠ Danh sách mốc này **khác** thanh trạng thái ở `TC-DLV-016` (có "Đăng tin" và "Ghép thành công"). ⛔ Không dùng đơn từng bị huỷ nhận — đơn đó thiếu dòng "Ghép thành công" do bug đã biết (`TC-CNL-010`).</t>
@@ -14755,7 +15047,7 @@
           <t>Tập 3 nhãn phụ theo vai (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L80" s="5" t="inlineStr"/>
+      <c r="L80" s="5" t="n"/>
       <c r="M80" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: tiêu đề section `DOC-v1.0-02` §3.6/§4.3/§5.2.</t>
@@ -14832,7 +15124,7 @@
           <t>1 tin NEED `POSTED`; tài khoản xem không thuộc cặp ghép (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L81" s="7" t="inlineStr"/>
+      <c r="L81" s="7" t="n"/>
       <c r="M81" s="7" t="inlineStr">
         <is>
           <t>Mục đích: assert đúng thời điểm được phép lộ SĐT — đây là ranh giới "Chờ ghép → Đã ghép". · Căn cứ: `BR-CON-02` §A5 L78 + `OPR-07` §D7 L343; `C-ASN-01` Resolved 2026-07-27 xác nhận SĐT **chỉ** lộ sau ghép và hành vi lộ sớm là **bug**. ⚠ Dự kiến FAIL trên app/prototype hiện tại (`KP-05 §5` #6) ⇒ **log bug**, ⛔ không sửa TC theo hành vi app.</t>
@@ -14908,7 +15200,7 @@
           <t>1 tin NEED của chính tài khoản đang xem (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L82" s="5" t="inlineStr"/>
+      <c r="L82" s="5" t="n"/>
       <c r="M82" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-05` §D7 L341; `C-ASN-02` Resolved 2026-07-27 — chủ tin KHÔNG được tự nhận mang giúp, hành vi prototype cho phép là **bug**. ⚠ Dự kiến FAIL (`KP-05 §5` #7) ⇒ **log bug**, ⛔ không sửa TC.</t>
@@ -14986,7 +15278,7 @@
           <t>≥2 tin NEED `POSTED` + 1 tin OFFER (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L83" s="7" t="inlineStr"/>
+      <c r="L83" s="7" t="n"/>
       <c r="M83" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-03` §D7 L339 — tin đã ghép bị ẩn khỏi bảng tin nên chỉ đếm tin ở trạng thái "Chờ ghép".</t>
@@ -15066,7 +15358,7 @@
       <c r="L84" s="5" t="inlineStr"/>
       <c r="M84" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: ⛔ không assert nút CTA trên card — `C-FEED-01(a)` Open (`US-D07` nói có ở card, PRD §3.3 không liệt kê); badge "Tin của bạn" verify riêng ở TC-FEED-003/004.</t>
+          <t>Căn cứ: ⛔ không assert nút CTA trên card — `C-FEED-01(a)` Open (`US-D07` nói có ở card, PRD §3.3 không liệt kê); badge "Tin của bạn" verify riêng ở TC-FEED-003/004. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N84" s="5" t="inlineStr">
@@ -15141,7 +15433,7 @@
           <t>≥2 tin NEED `POSTED` khác nhau (test_data_catalog §FEED, biên "≥2 tin")</t>
         </is>
       </c>
-      <c r="L85" s="7" t="inlineStr"/>
+      <c r="L85" s="7" t="n"/>
       <c r="M85" s="7" t="inlineStr"/>
       <c r="N85" s="7" t="inlineStr">
         <is>
@@ -15214,7 +15506,7 @@
           <t>1 tin có ảnh JPG ≤5MB + ghi chú ≤300 ký tự (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L86" s="5" t="inlineStr"/>
+      <c r="L86" s="5" t="n"/>
       <c r="M86" s="5" t="inlineStr"/>
       <c r="N86" s="5" t="inlineStr">
         <is>
@@ -15291,7 +15583,7 @@
       <c r="L87" s="7" t="inlineStr"/>
       <c r="M87" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: ⛔ không assert giá trị số "~X km" — dữ liệu runtime, không seed được.</t>
+          <t>Căn cứ: ⛔ không assert giá trị số "~X km" — dữ liệu runtime, không seed được. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N87" s="7" t="inlineStr">
@@ -15365,7 +15657,7 @@
           <t>1 tin NEED khai người nhận là tài khoản đang xem (test_data_catalog §FEED, biên chủ thể thứ ba)</t>
         </is>
       </c>
-      <c r="L88" s="5" t="inlineStr"/>
+      <c r="L88" s="5" t="n"/>
       <c r="M88" s="5" t="inlineStr">
         <is>
           <t>Mục đích: ca chủ thể thứ ba — không phải chủ tin nhưng cũng không được nhận đơn. · Căn cứ: `DOC-v1.0-02` §7 dòng 9 (nguồn duy nhất mô tả ca này). ⚠ Dự kiến FAIL ⇒ log bug, dẫn `OPR-05` để BA xác nhận rule áp cho cả vai người nhận.</t>
@@ -15441,7 +15733,7 @@
           <t>1 tin NEED của chính tài khoản đang xem (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L89" s="7" t="inlineStr"/>
+      <c r="L89" s="7" t="n"/>
       <c r="M89" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-FEED-004.</t>
@@ -15519,7 +15811,7 @@
           <t>1 tin NEED của tài khoản khác (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L90" s="5" t="inlineStr"/>
+      <c r="L90" s="5" t="n"/>
       <c r="M90" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-FEED-003.</t>
@@ -15596,7 +15888,7 @@
           <t>1 tin không có ảnh (test_data_catalog §FEED, biên)</t>
         </is>
       </c>
-      <c r="L91" s="7" t="inlineStr"/>
+      <c r="L91" s="7" t="n"/>
       <c r="M91" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: ⛔ không assert nội dung ảnh mặc định — chưa có đặc tả hình ảnh.</t>
@@ -15678,7 +15970,7 @@
       <c r="L92" s="5" t="inlineStr"/>
       <c r="M92" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-FEED-01(b)` Open — chính doc `§7 dòng 10` đặt câu hỏi bản chính thức có tích hợp bản đồ thật hay không. · Căn cứ: assert theo trạng thái đã mô tả ở PRD (placeholder); app v1.0 có bản đồ thật ⇒ FAIL và dẫn `C-FEED-01` để BA chốt scope, ⛔ không tự mở rộng TC sang bản đồ thật.</t>
+          <t>Mục đích: neo vào `C-FEED-01(b)` Open — chính doc `§7 dòng 10` đặt câu hỏi bản chính thức có tích hợp bản đồ thật hay không. · Căn cứ: assert theo trạng thái đã mô tả ở PRD (placeholder); app v1.0 có bản đồ thật ⇒ FAIL và dẫn `C-FEED-01` để BA chốt scope, ⛔ không tự mở rộng TC sang bản đồ thật. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N92" s="5" t="inlineStr">
@@ -15756,7 +16048,7 @@
       <c r="L93" s="7" t="inlineStr"/>
       <c r="M93" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-ORD-06` Open — text và ảnh empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được (không có card, khung màn còn nguyên); ⛔ không assert chuỗi empty state.</t>
+          <t>Mục đích: neo vào `C-ORD-06` Open — text và ảnh empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được (không có card, khung màn còn nguyên); ⛔ không assert chuỗi empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N93" s="7" t="inlineStr">
@@ -15832,7 +16124,7 @@
           <t>≥6 tin NEED `POSTED` (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L94" s="5" t="inlineStr"/>
+      <c r="L94" s="5" t="n"/>
       <c r="M94" s="5" t="inlineStr"/>
       <c r="N94" s="5" t="inlineStr">
         <is>
@@ -15905,7 +16197,11 @@
           <t>1 đơn "Hoàn thành" chưa gửi quà (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L95" s="7" t="inlineStr"/>
+      <c r="L95" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M95" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§A7` L107 + `KB-GIFT-01` (ô 5·Sender của ma trận nhãn nút).</t>
@@ -15984,7 +16280,7 @@
       <c r="L96" s="5" t="inlineStr"/>
       <c r="M96" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `§A7` L108 + `GIFT-01` §D3 L258 + `DOC-v1.0-02` §3.8 — ba nguồn khớp nhau về 4 loại.</t>
+          <t>Căn cứ: `§A7` L108 + `GIFT-01` §D3 L258 + `DOC-v1.0-02` §3.8 — ba nguồn khớp nhau về 4 loại. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N96" s="5" t="inlineStr">
@@ -16061,7 +16357,7 @@
       <c r="L97" s="7" t="inlineStr"/>
       <c r="M97" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn ghi 2 chuỗi popup khác nhau. · Căn cứ: assert theo PRD §3.8 + Figma; `US-D15` L194 ghi "Cảm ơn của bạn đã được gửi" là nguồn thua. App hiện chuỗi của `US-D15` ⇒ FAIL và dẫn `C-GIFT-03` để BA chốt text. Lượt chạy TC này tiêu 1 đơn Hoàn thành.</t>
+          <t>Mục đích: 2 nguồn ghi 2 chuỗi popup khác nhau. · Căn cứ: assert theo PRD §3.8 + Figma; `US-D15` L194 ghi "Cảm ơn của bạn đã được gửi" là nguồn thua. App hiện chuỗi của `US-D15` ⇒ FAIL và dẫn `C-GIFT-03` để BA chốt text. Lượt chạy TC này tiêu 1 đơn Hoàn thành. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N97" s="7" t="inlineStr">
@@ -16138,7 +16434,11 @@
           <t>1 đơn "Hoàn thành"; số lần gửi quà lần 1 → lần 2 (test_data_catalog §GIFT, biên)</t>
         </is>
       </c>
-      <c r="L98" s="5" t="inlineStr"/>
+      <c r="L98" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M98" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp biên lần 1 enable → lần 2 disable; TC này tiêu 1 đơn Hoàn thành. · Căn cứ: `KB-GIFT-01` — nhãn "Bạn đã đánh giá" là **UI leftover** của cơ chế rating đã out of scope, ⛔ không suy ra là có chức năng chấm điểm.</t>
@@ -16217,7 +16517,7 @@
       <c r="L99" s="7" t="inlineStr"/>
       <c r="M99" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: rule *"chỉ hiện loại count&gt;0"* là điểm dễ hiểu sai thành "hiện 4 loại với số 0". · Căn cứ: `KB-GIFT-03` + `US-D20` §D1b L196.</t>
+          <t>Mục đích: rule *"chỉ hiện loại count&gt;0"* là điểm dễ hiểu sai thành "hiện 4 loại với số 0". · Căn cứ: `KB-GIFT-03` + `US-D20` §D1b L196. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N99" s="7" t="inlineStr">
@@ -16292,7 +16592,11 @@
           <t>1 đơn "Hoàn thành"; text thông báo `NTF-07` (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L100" s="5" t="inlineStr"/>
+      <c r="L100" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M100" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `NTF-07` §D6 L325 + `§A7` L109; Figma bổ sung dòng thứ hai *"[Tên] đã gửi tặng bạn một món quà…"* nên ⛔ không assert thông báo chỉ có đúng 1 dòng. Danh sách loại thông báo chính thức còn chờ `C-NTF-01`. · Cập nhật 2026-09-21 (QC GiangDC2 chốt): nhấn thông báo `NTF-07` mở màn "Quà đã nhận" là ĐÚNG hành vi — sửa Expected step 4 theo app (trước ghi "màn Cá nhân"); không phải bug. ⚠ App chưa hiển thị emoji 🎁 ở thông báo — trang trí, ⛔ không assert.</t>
@@ -16368,7 +16672,11 @@
           <t>Bộ giá trị assert-absent: giá tiền / ví / cổng thanh toán / quy đổi điểm (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L101" s="7" t="inlineStr"/>
+      <c r="L101" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M101" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-GIFT-01` §D4 L271 + `§A7` L111 — quà là biểu tượng phi vật chất; app xuất hiện thành phần thanh toán ⇒ FAIL và mở CL scope.</t>
@@ -16447,7 +16755,7 @@
       <c r="L102" s="5" t="inlineStr"/>
       <c r="M102" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-GIFT-03` Open — vế "có danh sách lịch sử hay không". · Căn cứ: assert theo `US-D20` §D1b L196 (nguồn văn bản duy nhất nêu danh sách này), chưa có ảnh Figma hay app xác nhận. ⚠ Dự kiến FAIL ⇒ báo về `C-GIFT-03`, ⛔ không im lặng bỏ qua như đợt cũ.</t>
+          <t>Mục đích: neo vào `C-GIFT-03` Open — vế "có danh sách lịch sử hay không". · Căn cứ: assert theo `US-D20` §D1b L196 (nguồn văn bản duy nhất nêu danh sách này), chưa có ảnh Figma hay app xác nhận. ⚠ Dự kiến FAIL ⇒ báo về `C-GIFT-03`, ⛔ không im lặng bỏ qua như đợt cũ. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N102" s="5" t="inlineStr">
@@ -16523,7 +16831,7 @@
       <c r="L103" s="7" t="inlineStr"/>
       <c r="M103" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-ORD-06` Open — text empty state chưa có đặc tả. · Căn cứ: suy từ rule `KB-GIFT-03` (chỉ hiện loại count&gt;0) ⇒ 0 loại thì không có card loại nào; ⛔ không assert chuỗi empty state.</t>
+          <t>Mục đích: neo vào `C-ORD-06` Open — text empty state chưa có đặc tả. · Căn cứ: suy từ rule `KB-GIFT-03` (chỉ hiện loại count&gt;0) ⇒ 0 loại thì không có card loại nào; ⛔ không assert chuỗi empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N103" s="7" t="inlineStr">
@@ -16596,7 +16904,11 @@
           <t>Tài khoản đã nhận ≥1 quà (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L104" s="5" t="inlineStr"/>
+      <c r="L104" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M104" s="5" t="inlineStr"/>
       <c r="N104" s="5" t="inlineStr">
         <is>
@@ -16670,10 +16982,10 @@
           <t>2 đơn "Hoàn thành" khác tuyến (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L105" s="7" t="inlineStr"/>
+      <c r="L105" s="7" t="n"/>
       <c r="M105" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-GIFT-02` Open — đã quan sát back nhảy sang màn "Xác nhận đã nhận hàng" của **đơn khác**. · Căn cứ: `KB-GIFT-04`; dùng 2 đơn để phát hiện nhảy sai đơn. ⚠ Dự kiến FAIL ⇒ **log bug** (`KP-05 §5` #9).</t>
+          <t>Mục đích: neo vào `C-GIFT-02` Open — đã quan sát back nhảy sang màn "Xác nhận đã nhận hàng" của **đơn khác**. · Căn cứ: `KB-GIFT-04`; dùng 2 đơn để phát hiện nhảy sai đơn. ⚠ Dự kiến FAIL ⇒ **log bug** (`KP-05 §5` #9). · ⚠️ Đã chạy nhưng THIẾU EVIDENCE hợp lệ ⇒ không ghi PASS, tính Not Run (gate verify_evidence.py).</t>
         </is>
       </c>
       <c r="N105" s="7" t="inlineStr">
@@ -16752,7 +17064,7 @@
       <c r="L106" s="5" t="inlineStr"/>
       <c r="M106" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `RAT-01/02` có trong BRD nhưng `C-GIFT-01` Resolved 2026-07-27 loại khỏi v1.0. · Căn cứ: `BR-INT-06` §A5 L82 + `§A8` L125; chuỗi "★★★★★ Đã đánh giá" và nhãn "Bạn đã đánh giá" là UI leftover, ⛔ không suy ra có chức năng.</t>
+          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `RAT-01/02` có trong BRD nhưng `C-GIFT-01` Resolved 2026-07-27 loại khỏi v1.0. · Căn cứ: `BR-INT-06` §A5 L82 + `§A8` L125; chuỗi "★★★★★ Đã đánh giá" và nhãn "Bạn đã đánh giá" là UI leftover, ⛔ không suy ra có chức năng. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N106" s="5" t="inlineStr">
@@ -16824,7 +17136,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L107" s="7" t="inlineStr"/>
+      <c r="L107" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M107" s="7" t="inlineStr"/>
       <c r="N107" s="7" t="inlineStr">
         <is>
@@ -16895,7 +17211,11 @@
           <t>Tên hiển thị từ hồ sơ nhân viên (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L108" s="5" t="inlineStr"/>
+      <c r="L108" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M108" s="5" t="inlineStr"/>
       <c r="N108" s="5" t="inlineStr">
         <is>
@@ -16966,7 +17286,11 @@
           <t>≥1 thông báo chưa đọc (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L109" s="7" t="inlineStr"/>
+      <c r="L109" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M109" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-HOME-006.</t>
@@ -17044,7 +17368,7 @@
       <c r="L110" s="5" t="inlineStr"/>
       <c r="M110" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `§A7` L111 loại điểm/CO₂ khỏi v1.0 (`C-USR-01` Resolved). ⛔ Không assert giá trị của [x]/[y] — số toàn hệ thống, không seed được.</t>
+          <t>Căn cứ: `§A7` L111 loại điểm/CO₂ khỏi v1.0 (`C-USR-01` Resolved). ⛔ Không assert giá trị của [x]/[y] — số toàn hệ thống, không seed được. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N110" s="5" t="inlineStr">
@@ -17117,7 +17441,11 @@
           <t>1 đơn Fixture ở trạng thái "Chờ ghép" (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L111" s="7" t="inlineStr"/>
+      <c r="L111" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M111" s="7" t="inlineStr"/>
       <c r="N111" s="7" t="inlineStr">
         <is>
@@ -17268,7 +17596,11 @@
           <t>Nhãn vai `Gửi:` (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L113" s="7" t="inlineStr"/>
+      <c r="L113" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M113" s="7" t="inlineStr">
         <is>
           <t>Mục đích: 1 trong 3 ca phân biệt nhãn theo vai — bộ ba TC-HOME-011/012/013 phải khác nhãn nhau.</t>
@@ -17345,7 +17677,11 @@
           <t>Nhãn vai `Giao:`; 1 tin NEED của tài khoản khác (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L114" s="5" t="inlineStr"/>
+      <c r="L114" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M114" s="5" t="inlineStr">
         <is>
           <t>Mục đích: 1 trong 3 ca phân biệt nhãn theo vai.</t>
@@ -17421,7 +17757,11 @@
           <t>Nhãn vai `Nhận:`; 1 đơn có tài khoản ở vai người nhận (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L115" s="7" t="inlineStr"/>
+      <c r="L115" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M115" s="7" t="inlineStr">
         <is>
           <t>Mục đích: 1 trong 3 ca phân biệt nhãn theo vai. · Căn cứ: vai Receiver do Sender chỉ định khi đăng tin nên phải seed từ tài khoản khác, không dựng được bằng chính tài khoản đang test.</t>
@@ -17497,7 +17837,11 @@
           <t>1 đơn Fixture ở trạng thái "Chờ ghép" (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L116" s="5" t="inlineStr"/>
+      <c r="L116" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M116" s="5" t="inlineStr"/>
       <c r="N116" s="5" t="inlineStr">
         <is>
@@ -17570,7 +17914,7 @@
           <t>≥1 tin cộng đồng còn hiệu lực (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L117" s="7" t="inlineStr"/>
+      <c r="L117" s="7" t="n"/>
       <c r="M117" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt "Tin mới" KHÔNG phải tính năng riêng của Carrier — neo vào `C-ORD-07` và `KB-ORD-08`.</t>
@@ -17647,7 +17991,7 @@
           <t>≥1 tin cộng đồng còn hiệu lực (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L118" s="5" t="inlineStr"/>
+      <c r="L118" s="5" t="n"/>
       <c r="M118" s="5" t="inlineStr"/>
       <c r="N118" s="5" t="inlineStr">
         <is>
@@ -17718,7 +18062,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L119" s="7" t="inlineStr"/>
+      <c r="L119" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M119" s="7" t="inlineStr"/>
       <c r="N119" s="7" t="inlineStr">
         <is>
@@ -17796,7 +18144,11 @@
           <t>1 đơn đang hoạt động + ≥1 tin cộng đồng (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L120" s="5" t="inlineStr"/>
+      <c r="L120" s="5" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
       <c r="M120" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: màn "Tặng quà" nằm trong cùng luật nhưng cần đơn ở trạng thái Hoàn thành nên verify ở `TC-GIFT-*`, không nhồi vào TC này.</t>
@@ -17875,7 +18227,7 @@
           <t>3 tài khoản 3 vai trên cùng 1 đơn (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L121" s="7" t="inlineStr"/>
+      <c r="L121" s="7" t="n"/>
       <c r="M121" s="7" t="inlineStr">
         <is>
           <t>Mục đích: assert được vế "có icon và phân biệt theo vai" mà không cần mapping icon cụ thể. · Căn cứ: `DOC-v1.0-02` §2 nêu header có icon vai trò; mapping icon↔vai **chưa chốt** (`C-HOME-01` Open) nên ⛔ không assert hình icon. Ba vai cùng một icon hoặc thiếu icon ⇒ FAIL và dẫn `C-HOME-01`.</t>
@@ -17952,7 +18304,11 @@
           <t>0 thông báo chưa đọc (test_data_catalog §HOME, biên)</t>
         </is>
       </c>
-      <c r="L122" s="5" t="inlineStr"/>
+      <c r="L122" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M122" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-HOME-005. · Căn cứ: cơ chế đánh dấu đã đọc còn chờ `C-NTF-03(a)`; TC dùng đường mở từng item nên không phụ thuộc nút mark-all, app không hạ chấm sau khi đọc hết ⇒ FAIL và dẫn `C-NTF-03`.</t>
@@ -18029,7 +18385,11 @@
           <t>Tagline banner (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L123" s="7" t="inlineStr"/>
+      <c r="L123" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M123" s="7" t="inlineStr">
         <is>
           <t>Mục đích: banner hiển thị đúng tagline đã chốt. · Căn cứ: dùng chuỗi PRD "Tiện đường — Giúp đồng nghiệp" (`C-HOME-01(b)` RESOLVED 2026-09-15 — khớp design HOME_01/02/04; PRD thắng khi mô tả chi tiết màn hình, `MASTER-MEMORY §2`). BRD `§A3` L29 "Đồng nghiệp giúp nhau" là nguồn lỗi thời. · 2026-09-21: sửa Expected từ chuỗi BRD sang chuỗi PRD sau VR-005 (app hiện đúng chuỗi PRD).</t>
@@ -18111,7 +18471,7 @@
           <t>Badge thuộc tập {Chờ ghép, Đã ghép, Đang giao, Đã giao, Hoàn thành}; 5 mốc progress (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L124" s="5" t="inlineStr"/>
+      <c r="L124" s="5" t="n"/>
       <c r="M124" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: 5 mốc lấy từ `§D2` L232. Trạng thái "Hoàn thành" verify ở `TC-ACT-*` vì đó là ranh giới đơn còn/không còn "đang hoạt động" và chưa có đặc tả rõ (`test_data_catalog §HOME` biên).</t>
@@ -18187,7 +18547,11 @@
           <t>1 đơn Fixture ở trạng thái "Chờ ghép" (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L125" s="7" t="inlineStr"/>
+      <c r="L125" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M125" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: nút này không có mô tả trong BRD/PRD (`KP-05 §3` #1) nên chỉ assert đích điều hướng, ⛔ không assert tab mặc định hay bộ lọc của màn Hoạt động.</t>
@@ -18267,7 +18631,7 @@
       <c r="L126" s="5" t="inlineStr"/>
       <c r="M126" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn ghi 2 con số cho cùng một section (1 tin vs tối đa 5 tin). · Căn cứ: assert theo BRD `US-D06` §D1b L175 "chỉ hiện tối đa 5 tin" — BRD thắng PRD khi mâu thuẫn về rule (`MASTER-MEMORY §2`); app hiện đúng 1 tin ⇒ FAIL và dẫn `C-HOME-03` để BA chốt.</t>
+          <t>Mục đích: 2 nguồn ghi 2 con số cho cùng một section (1 tin vs tối đa 5 tin). · Căn cứ: assert theo BRD `US-D06` §D1b L175 "chỉ hiện tối đa 5 tin" — BRD thắng PRD khi mâu thuẫn về rule (`MASTER-MEMORY §2`); app hiện đúng 1 tin ⇒ FAIL và dẫn `C-HOME-03` để BA chốt. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N126" s="5" t="inlineStr">
@@ -18341,7 +18705,7 @@
           <t>≥1 tin cộng đồng còn hiệu lực (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L127" s="7" t="inlineStr"/>
+      <c r="L127" s="7" t="n"/>
       <c r="M127" s="7" t="inlineStr"/>
       <c r="N127" s="7" t="inlineStr">
         <is>
@@ -18419,7 +18783,7 @@
       <c r="L128" s="5" t="inlineStr"/>
       <c r="M128" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: rule hiện/ẩn nút theo mốc 5 vs ≥6 tin **không có nguồn tài liệu** (`KP-05 §3` #2) nên TC chỉ assert nhánh có đủ tin, ⛔ không assert nhánh ẩn nút.</t>
+          <t>Căn cứ: rule hiện/ẩn nút theo mốc 5 vs ≥6 tin **không có nguồn tài liệu** (`KP-05 §3` #2) nên TC chỉ assert nhánh có đủ tin, ⛔ không assert nhánh ẩn nút. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N128" s="5" t="inlineStr">
@@ -18493,7 +18857,7 @@
           <t>≥1 tin NEED của tài khoản khác (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L129" s="7" t="inlineStr"/>
+      <c r="L129" s="7" t="n"/>
       <c r="M129" s="7" t="inlineStr"/>
       <c r="N129" s="7" t="inlineStr">
         <is>
@@ -18652,7 +19016,7 @@
       <c r="L131" s="7" t="inlineStr"/>
       <c r="M131" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: ranh giới hợp lệ/vi phạm — `NTF-01` **được phép nhắc** "SĐT đã được lộ" nhưng ⛔ không được kèm số. Push là kênh dễ lọt nhất vì nội dung do backend đẩy, không qua UI. · Căn cứ: `OPR-07` §D7 L343 + `§D6` L315. Có thông báo chứa số ⇒ FAIL và log bug mức cao (rò rỉ dữ liệu cá nhân).</t>
+          <t>Mục đích: ranh giới hợp lệ/vi phạm — `NTF-01` **được phép nhắc** "SĐT đã được lộ" nhưng ⛔ không được kèm số. Push là kênh dễ lọt nhất vì nội dung do backend đẩy, không qua UI. · Căn cứ: `OPR-07` §D7 L343 + `§D6` L315. Có thông báo chứa số ⇒ FAIL và log bug mức cao (rò rỉ dữ liệu cá nhân). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N131" s="7" t="inlineStr">
@@ -18727,7 +19091,7 @@
           <t>1 đơn `MATCHED` có khai người nhận (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L132" s="5" t="inlineStr"/>
+      <c r="L132" s="5" t="n"/>
       <c r="M132" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L319-320 (`NTF-01` và `NTF-02`). Danh sách loại thông báo chính thức còn chờ `C-NTF-01`; nội dung lệch ⇒ dẫn `C-NTF-01` để BA chốt, ⛔ không tự sửa chuỗi trong TC.</t>
@@ -18803,7 +19167,7 @@
           <t>1 tin OFFER + 1 tin NEED khớp tuyến (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L133" s="7" t="inlineStr"/>
+      <c r="L133" s="7" t="n"/>
       <c r="M133" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L321 (`NTF-03`) + `US-D12` §D1b L186. ⛔ Không assert độ trễ hay chu kỳ quét — chưa chốt (`C-NTF-02` Partially Resolved).</t>
@@ -18881,7 +19245,7 @@
           <t>1 đơn `MATCHED` đủ 3 vai (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L134" s="5" t="inlineStr"/>
+      <c r="L134" s="5" t="n"/>
       <c r="M134" s="5" t="inlineStr">
         <is>
           <t>Mục đích: `NTF-04` có **2 người nhận** ⇒ phải kiểm cả hai, thiếu một vai là bỏ sót nửa rule. · Căn cứ: `§D6` L322.</t>
@@ -18959,7 +19323,7 @@
           <t>1 đơn `IN_TRANSIT` đủ 3 vai (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L135" s="7" t="inlineStr"/>
+      <c r="L135" s="7" t="n"/>
       <c r="M135" s="7" t="inlineStr">
         <is>
           <t>Mục đích: `NTF-05` có 2 người nhận. · Căn cứ: `§D6` L323.</t>
@@ -19040,7 +19404,7 @@
       <c r="L136" s="5" t="inlineStr"/>
       <c r="M136" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn 2 chuỗi text cho cùng `NTF-06`. · Căn cứ: assert theo BRD `§D6` L324 vì bản PRD+Figma ("Đơn đã hoàn thành — đánh giá ngay") dẫn tới cơ chế **đánh giá đã bị `C-GIFT-01` loại khỏi v1.0** ⇒ chuỗi đó không nhất quán với scope đã chốt. App hiện bản PRD ⇒ FAIL và dẫn `C-NTF-01` để BA chốt text.</t>
+          <t>Mục đích: 2 nguồn 2 chuỗi text cho cùng `NTF-06`. · Căn cứ: assert theo BRD `§D6` L324 vì bản PRD+Figma ("Đơn đã hoàn thành — đánh giá ngay") dẫn tới cơ chế **đánh giá đã bị `C-GIFT-01` loại khỏi v1.0** ⇒ chuỗi đó không nhất quán với scope đã chốt. App hiện bản PRD ⇒ FAIL và dẫn `C-NTF-01` để BA chốt text. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N136" s="5" t="inlineStr">
@@ -19115,7 +19479,7 @@
           <t>1 đơn `MATCHED`; lý do huỷ ≥5 ký tự (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L137" s="7" t="inlineStr"/>
+      <c r="L137" s="7" t="n"/>
       <c r="M137" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L326 (`NTF-08`). Nhánh Carrier huỷ nhận có thêm câu "Đơn đang chờ người vận chuyển mới…" theo Figma (`KP-07` hàng #8) — nhánh đó thuộc `TC-CNL-007`, ⛔ không nhồi vào TC này.</t>
@@ -19191,7 +19555,7 @@
           <t>1 tin NEED "Hết hạn" (test_data_catalog §NTF — ⛔ không seed được qua UI)</t>
         </is>
       </c>
-      <c r="L138" s="5" t="inlineStr"/>
+      <c r="L138" s="5" t="n"/>
       <c r="M138" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `§D6` L327 (`NTF-09`).</t>
@@ -19267,7 +19631,7 @@
           <t>Thông báo ở 3 mốc thời gian (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L139" s="7" t="inlineStr"/>
+      <c r="L139" s="7" t="n"/>
       <c r="M139" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.2 + ảnh Figma `3e626d39…`. ⛔ Không assert nhóm cho thông báo cũ hơn 1 tuần — không có nguồn mô tả.</t>
@@ -19347,7 +19711,7 @@
           <t>Đúng 2 thông báo chưa đọc (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L140" s="5" t="inlineStr"/>
+      <c r="L140" s="5" t="n"/>
       <c r="M140" s="5" t="inlineStr">
         <is>
           <t>Mục đích: ranh giới của chấm đỏ là **thông báo chưa đọc cuối cùng** — bước 4 tồn tại để bắt lỗi tắt chấm đỏ quá sớm.</t>
@@ -19424,7 +19788,7 @@
           <t>3 thông báo cùng nhóm thời gian, 1 đã đọc (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L141" s="7" t="inlineStr"/>
+      <c r="L141" s="7" t="n"/>
       <c r="M141" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-NTF-01` + ảnh Figma `3e626d39…` — trạng thái đọc theo **từng item**.</t>
@@ -19502,7 +19866,7 @@
           <t>2 thông báo chưa đọc (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L142" s="5" t="inlineStr"/>
+      <c r="L142" s="5" t="n"/>
       <c r="M142" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-NTF-03(a)` Open — chỉ assert vế suy được từ `KB-NTF-01` (trạng thái theo từng item). · Căn cứ: ⛔ không assert nút "Đánh dấu đã đọc" là mark-all hay mark-per-item; cơ chế nút chờ BA chốt.</t>
@@ -19580,7 +19944,7 @@
           <t>Danh sách thông báo dài hơn 1 trang (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L143" s="7" t="inlineStr"/>
+      <c r="L143" s="7" t="n"/>
       <c r="M143" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-NTF-02`. ⛔ Không assert số item mỗi trang — không có nguồn mô tả.</t>
@@ -19661,7 +20025,7 @@
       <c r="L144" s="5" t="inlineStr"/>
       <c r="M144" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-NTF-01` Open — 3 nguồn cho 3 danh sách khác nhau nên ⛔ không assert danh sách nào là đủ; TC chỉ assert 2 loại **đã bị loại khỏi scope**. · Căn cứ: `KP-07` hàng #6b (`C-GIFT-01` loại rating) và hàng #11 (`C-USR-01` loại CO₂/điểm). Nếu app bắn loại ngoài `§D6` như `KP-07` hàng #10 ("Sắp đến khung giờ hẹn giao") thì **không tính FAIL** — ghi vào `C-NTF-01` làm ứng viên bổ sung.</t>
+          <t>Mục đích: neo vào `C-NTF-01` Open — 3 nguồn cho 3 danh sách khác nhau nên ⛔ không assert danh sách nào là đủ; TC chỉ assert 2 loại **đã bị loại khỏi scope**. · Căn cứ: `KP-07` hàng #6b (`C-GIFT-01` loại rating) và hàng #11 (`C-USR-01` loại CO₂/điểm). Nếu app bắn loại ngoài `§D6` như `KP-07` hàng #10 ("Sắp đến khung giờ hẹn giao") thì **không tính FAIL** — ghi vào `C-NTF-01` làm ứng viên bổ sung. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N144" s="5" t="inlineStr">
@@ -19734,7 +20098,7 @@
           <t>Tài khoản 0 thông báo (test_data_catalog §NTF, biên)</t>
         </is>
       </c>
-      <c r="L145" s="7" t="inlineStr"/>
+      <c r="L145" s="7" t="n"/>
       <c r="M145" s="7" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-06` Open — text empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được; ⛔ không assert chuỗi hay ảnh empty state.</t>
@@ -19811,7 +20175,7 @@
           <t>Tài khoản có ≥1 thông báo (test_data_catalog §NTF)</t>
         </is>
       </c>
-      <c r="L146" s="5" t="inlineStr"/>
+      <c r="L146" s="5" t="n"/>
       <c r="M146" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: đích "Trang chủ" suy từ đường vào (chuông ở header Trang chủ) — `KP-05 §3` #6 ghi nhận nút back này chưa có mô tả trong doc. Mở chuông từ màn khác là ca khác, ⛔ không nhồi vào TC này.</t>
@@ -19892,7 +20256,11 @@
           <t>Loại hàng "Giấy tờ, hồ sơ", giá trị "Thấp", email nội bộ tra được, khung giờ tương đối so với hiện tại (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L147" s="7" t="inlineStr"/>
+      <c r="L147" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M147" s="7" t="inlineStr">
         <is>
           <t>Mục đích: happy path xuyên 3 bước — nền để so mọi nhánh negative của module. · Căn cứ: `ORD-02` §D3 L240 + `US-D01` §D1b L164. ⛔ Khung giờ chọn **tương đối** so với hiện tại, không hardcode giờ.</t>
@@ -19970,7 +20338,11 @@
           <t>Email nội bộ tra được `stag_anhdc4@fpt.com` (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L148" s="5" t="inlineStr"/>
+      <c r="L148" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M148" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-ORD-020. · Căn cứ: `USR-EML` §D3 L253 + `US-D18` §D1b L168.</t>
@@ -20047,7 +20419,11 @@
           <t>Nhóm người nhận để trống (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L149" s="7" t="inlineStr"/>
+      <c r="L149" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M149" s="7" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-01` Resolved 2026-07-28 — nhóm Người nhận là **bắt buộc**. · Căn cứ: `KB-ORD-01` + `DOC-v1.0-02` §7 dòng 2 ghi nhận hành vi prototype cho để trống mà vẫn đăng thành công là **giới hạn bản demo**. ⚠ Dự kiến FAIL nếu app còn hành vi prototype ⇒ log bug.</t>
@@ -20126,7 +20502,11 @@
           <t>Checkbox chưa tick và đã tick (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L150" s="5" t="inlineStr"/>
+      <c r="L150" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M150" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `ORD-09` §D3 L245 + `D8.1` L373 — đây là điểm chặn consent bắt buộc, cùng rule với `TC-TS-004`.</t>
@@ -20204,7 +20584,11 @@
           <t>1 tin OFFER (test_data_catalog §ORD, bảng OFFER)</t>
         </is>
       </c>
-      <c r="L151" s="7" t="inlineStr"/>
+      <c r="L151" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M151" s="7" t="inlineStr">
         <is>
           <t>Mục đích: tuyến OFFER là dữ liệu **không công khai** — lộ lên Bảng tin là rò rỉ lịch trình di chuyển của nhân viên. · Căn cứ: `US-D11` §D1b L185 + `ORD-01` §D3 L240.</t>
@@ -20284,7 +20668,7 @@
       <c r="L152" s="5" t="inlineStr"/>
       <c r="M152" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: ranh giới khoá sửa là "Chờ ghép" → "Đã ghép"; cặp với TC-ORD-046. · Căn cứ: `BR-EDIT-01` §D4 L269 + `OPR-10` §D7 L346. Sửa được sau khi ghép ⇒ Carrier đã nhận đơn theo thông tin cũ, log bug mức cao.</t>
+          <t>Mục đích: ranh giới khoá sửa là "Chờ ghép" → "Đã ghép"; cặp với TC-ORD-046. · Căn cứ: `BR-EDIT-01` §D4 L269 + `OPR-10` §D7 L346. Sửa được sau khi ghép ⇒ Carrier đã nhận đơn theo thông tin cũ, log bug mức cao. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N152" s="5" t="inlineStr">
@@ -20360,7 +20744,7 @@
       <c r="L153" s="7" t="inlineStr"/>
       <c r="M153" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `US-D04` §D1b L166 + `KB-ORD-02`. Bản text đầy đủ của dòng lý do assert ở `TC-ACT-008`; TC này chỉ assert transition trạng thái và sự có mặt của lý do.</t>
+          <t>Căn cứ: `US-D04` §D1b L166 + `KB-ORD-02`. Bản text đầy đủ của dòng lý do assert ở `TC-ACT-008`; TC này chỉ assert transition trạng thái và sự có mặt của lý do. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N153" s="7" t="inlineStr">
@@ -20435,7 +20819,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L154" s="5" t="inlineStr"/>
+      <c r="L154" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M154" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: đối chiếu cấu trúc theo ảnh Figma `f821ba30…`.</t>
@@ -20512,7 +20900,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L155" s="7" t="inlineStr"/>
+      <c r="L155" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M155" s="7" t="inlineStr"/>
       <c r="N155" s="7" t="inlineStr">
         <is>
@@ -20585,7 +20977,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L156" s="5" t="inlineStr"/>
+      <c r="L156" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M156" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng cấu trúc với luồng NEED 3 bước ở TC-ORD-002.</t>
@@ -20666,7 +21062,7 @@
       <c r="L157" s="7" t="inlineStr"/>
       <c r="M157" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `D8.1` §D8.1 L357 + `KB-VIBE-01`/`KB-VIBE-02`.</t>
+          <t>Căn cứ: `D8.1` §D8.1 L357 + `KB-VIBE-01`/`KB-VIBE-02`. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N157" s="7" t="inlineStr">
@@ -20742,7 +21138,11 @@
           <t>Giá trị hàng rỗng (test_data_catalog §ORD, biên chặn bước)</t>
         </is>
       </c>
-      <c r="L158" s="5" t="inlineStr"/>
+      <c r="L158" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M158" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L359 + `KP-01` §10.4.</t>
@@ -20818,7 +21218,11 @@
           <t>Giá trị hàng "Cao" (test_data_catalog §ORD, biên)</t>
         </is>
       </c>
-      <c r="L159" s="7" t="inlineStr"/>
+      <c r="L159" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M159" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-ORD-010. · Căn cứ: `D8.1` §D8.1 L359 + `KB-ORD-05` (nguyên văn banner lấy từ app). ⚠ Phân biệt: cảnh báo theo **mức định tính "Cao"** là CÓ ở v1.0; ngưỡng bằng **số tiền** (`BR-ORD-03`) thì out of scope (`TC-ORD-054`).</t>
@@ -20894,7 +21298,11 @@
           <t>Tên và SĐT từ hồ sơ nhân viên (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L160" s="5" t="inlineStr"/>
+      <c r="L160" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M160" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L362-363. ⛔ Không assert giá trị SĐT cụ thể — dữ liệu `Master` không seed được, và đang có nghi vấn tự đổi giá trị (`TC-ORD-018`).</t>
@@ -20971,7 +21379,11 @@
           <t>Tên người gửi pre-fill, chỉ đọc (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L161" s="7" t="inlineStr"/>
+      <c r="L161" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M161" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L362 ghi rõ "Chỉ đọc". ⚠ Dự kiến FAIL — `KP-01` §10.5 đã live-verify app cho sửa và **xoá trắng khi chạm**, không tự phục hồi trong phiên ⇒ **log bug** (`KP-05 §5` #1), ⛔ không hạ chuẩn TC theo hành vi app.</t>
@@ -21047,7 +21459,11 @@
           <t>Địa chỉ lấy hàng pre-fill theo nơi làm việc (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L162" s="5" t="inlineStr"/>
+      <c r="L162" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M162" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-10` Open — quyết định đây là **bug hay tài khoản test chưa cấu hình**. · Căn cứ: `D8.1` §D8.1 L364. ⚠ Dự kiến FAIL — `KP-01` §10.6 ghi app để trống, chỉ có placeholder (`VR-002 TC_04.21` FAIL). ⇒ **Xác nhận với dev trước khi log bug**: nếu hồ sơ tài khoản test thiếu nơi làm việc thì là lỗi dữ liệu test, không phải bug app.</t>
@@ -21125,7 +21541,11 @@
           <t>Email nội bộ không có trong danh bạ (test_data_catalog §ORD, biên)</t>
         </is>
       </c>
-      <c r="L163" s="7" t="inlineStr"/>
+      <c r="L163" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M163" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-ORD-019 — phân biệt "không tra thấy" với "email sai định dạng" ở TC-ORD-021. · Căn cứ: `US-D18` §D1b L168 + `D8.1` L366.</t>
@@ -21204,7 +21624,11 @@
           <t>Email thiếu "@" và email ngoài tên miền nội bộ (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L164" s="5" t="inlineStr"/>
+      <c r="L164" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M164" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L366 — 2 lớp lỗi cùng field, cùng hệ quả "không tra danh bạ" nên giữ trong 1 TC với 2 dòng expected riêng.</t>
@@ -21282,7 +21706,11 @@
           <t>SĐT người nhận do app auto-fill, vd `0000286248` (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L165" s="7" t="inlineStr"/>
+      <c r="L165" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M165" s="7" t="inlineStr">
         <is>
           <t>Mục đích: dữ liệu do chính app điền phải qua được validate của chính nó. · Căn cứ: `KB-VIBE-08` (`KP-01` §10.9). ⚠ Dự kiến FAIL — app báo "Số điện thoại không hợp lệ" cho `0000286248` do chính nó điền ⇒ **log bug** (`KP-05 §5` #4); bug có thể ở tầng dữ liệu danh bạ hoặc tầng validate, ghi rõ cả 2 khả năng khi log.</t>
@@ -21363,7 +21791,11 @@
           <t>Tên người nhận 1 / 2 / 60 / 61 ký tự (test_data_catalog §ORD, 4 mốc biên)</t>
         </is>
       </c>
-      <c r="L166" s="5" t="inlineStr"/>
+      <c r="L166" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M166" s="5" t="inlineStr">
         <is>
           <t>Mục đích: bộ 4 mốc biên của cùng 1 field, chạy liền mạch trong 1 form nên giữ 1 TC; tách khỏi TC-ORD-025 vì SĐT là lớp validate khác. · Căn cứ: `D8.1` §D8.1 L367.</t>
@@ -21446,7 +21878,11 @@
           <t>SĐT 9 / 10 / 11 số, không bắt đầu bằng 0, có chữ (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L167" s="7" t="inlineStr"/>
+      <c r="L167" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M167" s="7" t="inlineStr">
         <is>
           <t>Mục đích: 5 lớp lỗi của cùng field SĐT — tách khỏi biên độ dài tên ở TC-ORD-024 để khi FAIL biết ngay lớp nào sai. · Căn cứ: `D8.1` §D8.1 L368.</t>
@@ -21523,7 +21959,11 @@
           <t>2 địa chỉ trùng nhau (test_data_catalog §ORD, biên chặn)</t>
         </is>
       </c>
-      <c r="L168" s="5" t="inlineStr"/>
+      <c r="L168" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M168" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L369.</t>
@@ -21604,7 +22044,7 @@
       <c r="L169" s="7" t="inlineStr"/>
       <c r="M169" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `KB-ORD-06` (`KP-01` §3).</t>
+          <t>Căn cứ: `KB-ORD-06` (`KP-01` §3). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N169" s="7" t="inlineStr">
@@ -21684,7 +22124,7 @@
       <c r="L170" s="5" t="inlineStr"/>
       <c r="M170" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: cặp đối chứng (a)/(b) của cùng cơ chế. · Căn cứ: `KB-ORD-06`. Ghi chú cho automation về sau: `set text` đơn thuần **không lưu** giá trị, phải tap suggestion (`KP-01` §10.12).</t>
+          <t>Mục đích: cặp đối chứng (a)/(b) của cùng cơ chế. · Căn cứ: `KB-ORD-06`. Ghi chú cho automation về sau: `set text` đơn thuần **không lưu** giá trị, phải tap suggestion (`KP-01` §10.12). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N170" s="5" t="inlineStr">
@@ -21762,7 +22202,7 @@
       <c r="L171" s="7" t="inlineStr"/>
       <c r="M171" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh mặc định và nhánh quá khứ — tách khỏi quan hệ Đến/Từ ở TC-ORD-031 vì hai rule khác nhau. · Căn cứ: `D8.1` §D8.1 L370.</t>
+          <t>Mục đích: nhánh mặc định và nhánh quá khứ — tách khỏi quan hệ Đến/Từ ở TC-ORD-031 vì hai rule khác nhau. · Căn cứ: `D8.1` §D8.1 L370. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N171" s="7" t="inlineStr">
@@ -21841,7 +22281,7 @@
       <c r="L172" s="5" t="inlineStr"/>
       <c r="M172" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: biên "= nhau" là mốc hợp lệ dễ bị chặn oan. · Căn cứ: `D8.1` §D8.1 L371.</t>
+          <t>Mục đích: biên "= nhau" là mốc hợp lệ dễ bị chặn oan. · Căn cứ: `D8.1` §D8.1 L371. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N172" s="5" t="inlineStr">
@@ -21920,7 +22360,7 @@
       <c r="L173" s="7" t="inlineStr"/>
       <c r="M173" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `D8.1` §D8.1 L372. ⛔ Chọn giờ **tương đối** so với hiện tại, không hardcode giờ — app validate theo đồng hồ thật (`KP-01` §10.11).</t>
+          <t>Căn cứ: `D8.1` §D8.1 L372. ⛔ Chọn giờ **tương đối** so với hiện tại, không hardcode giờ — app validate theo đồng hồ thật (`KP-01` §10.11). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N173" s="7" t="inlineStr">
@@ -21995,7 +22435,11 @@
           <t>Bộ dữ liệu xác định ở B1 và B2 (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L174" s="5" t="inlineStr"/>
+      <c r="L174" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M174" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.5.3.</t>
@@ -22070,7 +22514,11 @@
           <t>Checkbox điều khoản mặc định (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L175" s="7" t="inlineStr"/>
+      <c r="L175" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M175" s="7" t="inlineStr">
         <is>
           <t>Mục đích: 2 nguồn trái nhau, và TC `TC_04.71` của đợt cũ expected "tick sẵn" là **sai nguồn**. · Căn cứ: `C-ORD-12` Resolved 2026-09-07 theo `D8.1` L373 + app STG (`KP-01` §10.7); PRD §3.5.3 ghi "mặc định đã tick sẵn" là nguồn thua.</t>
@@ -22149,7 +22597,7 @@
       <c r="L176" s="5" t="inlineStr"/>
       <c r="M176" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `US-D02` §D1b L165.</t>
+          <t>Căn cứ: `US-D02` §D1b L165. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N176" s="5" t="inlineStr">
@@ -22225,7 +22673,11 @@
           <t>2 tin NEED (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L177" s="7" t="inlineStr"/>
+      <c r="L177" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M177" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.5.4.</t>
@@ -22301,7 +22753,11 @@
           <t>Hồ sơ đầy đủ tên + SĐT + nơi làm việc (test_data_catalog §ORD, bảng OFFER)</t>
         </is>
       </c>
-      <c r="L178" s="5" t="inlineStr"/>
+      <c r="L178" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M178" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D10` §D1b L184 + `DOC-v1.0-02` §4.4 + `KB-ORD-11`.</t>
@@ -22381,7 +22837,11 @@
           <t>Điểm xuất phát pre-fill; điểm đến trùng điểm xuất phát (test_data_catalog §ORD, bảng OFFER)</t>
         </is>
       </c>
-      <c r="L179" s="7" t="inlineStr"/>
+      <c r="L179" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M179" s="7" t="inlineStr">
         <is>
           <t>Mục đích: khác biệt cần chốt — điểm xuất phát của OFFER **sửa được**, trong khi tên người gửi của NEED là chỉ đọc (`TC-ORD-016`). · Căn cứ: `D8.2` §D8.2 L381-382.</t>
@@ -22462,7 +22922,7 @@
       <c r="L180" s="5" t="inlineStr"/>
       <c r="M180" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: `US-D11` §D1b L185.</t>
+          <t>Căn cứ: `US-D11` §D1b L185. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N180" s="5" t="inlineStr">
@@ -22541,7 +23001,7 @@
       <c r="L181" s="7" t="inlineStr"/>
       <c r="M181" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `ORD-10` §D3 L252 + `US-D19` §D1b L169.</t>
+          <t>Căn cứ: `ORD-10` §D3 L252 + `US-D19` §D1b L169. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N181" s="7" t="inlineStr">
@@ -22614,7 +23074,11 @@
           <t>1 tin NEED vừa đăng (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L182" s="5" t="inlineStr"/>
+      <c r="L182" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M182" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `ORD-04` §D3 L243.</t>
@@ -22695,7 +23159,11 @@
           <t>Bộ dữ liệu thiếu trường bắt buộc và bộ đủ trường (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L183" s="7" t="inlineStr"/>
+      <c r="L183" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M183" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `VAL-01` §D8.3 L392 — rule áp cho **cả 2 luồng đăng tin**, nên TC kiểm cả hai.</t>
@@ -22772,7 +23240,11 @@
           <t>8 chip app STG; nhãn "Tài liệu" là giá trị assert-absent (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L184" s="5" t="inlineStr"/>
+      <c r="L184" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M184" s="5" t="inlineStr">
         <is>
           <t>Mục đích: ⭐ CL lan rộng nhất dự án — mọi TC đợt cũ nhắc "Tài liệu" đều sai chữ. · Căn cứ: assert theo `DOC-v1.0-06` KP-01 §10.2 (`KB-VIBE-01`, có screenshot `VR-002 TC_04.5`) — nguồn có bằng chứng app thắng doc (`MASTER-MEMORY §2`); BRD `D8.1` ghi 5 giá trị và PRD §3.5.1 ghi 8 chip, cả hai đều có "Tài liệu". App xuất hiện chip "Tài liệu" ⇒ FAIL và dẫn `C-ORD-09` để BA chốt danh mục.</t>
@@ -22850,7 +23322,11 @@
           <t>8 chip app STG (test_data_catalog §ORD, biên "không tái hiện được trạng thái chưa chọn")</t>
         </is>
       </c>
-      <c r="L185" s="7" t="inlineStr"/>
+      <c r="L185" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M185" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt bằng TC lý do **không viết được TC negative "để trống loại hàng"** — cơ chế UI không cho tạo tiền đề đó. · Căn cứ: `KB-VIBE-02`; rule "Không cho để trống" của `D8.1` vì vậy không kiểm chứng được qua UI.</t>
@@ -22927,7 +23403,11 @@
           <t>Giá trị hàng "Thấp" và "Vừa" (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L186" s="5" t="inlineStr"/>
+      <c r="L186" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M186" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-ORD-009 — banner chỉ gắn với mức "Cao".</t>
@@ -23006,7 +23486,11 @@
           <t>Ghi chú 300 ký tự và 301 ký tự (test_data_catalog §ORD, biên)</t>
         </is>
       </c>
-      <c r="L187" s="7" t="inlineStr"/>
+      <c r="L187" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M187" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L358.</t>
@@ -23089,7 +23573,7 @@
       <c r="L188" s="5" t="inlineStr"/>
       <c r="M188" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh hợp lệ của ràng buộc ảnh — cặp với TC-ORD-013 (nhánh bị chặn). · Căn cứ: `D8.1` §D8.1 L360.</t>
+          <t>Mục đích: nhánh hợp lệ của ràng buộc ảnh — cặp với TC-ORD-013 (nhánh bị chặn). · Căn cứ: `D8.1` §D8.1 L360. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N188" s="5" t="inlineStr">
@@ -23169,7 +23653,7 @@
       <c r="L189" s="7" t="inlineStr"/>
       <c r="M189" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh bị chặn — tách khỏi TC-ORD-012 vì 2 lớp lỗi khác nhau (dung lượng ⟷ định dạng) và để khi FAIL biết ngay lớp nào sai.</t>
+          <t>Mục đích: nhánh bị chặn — tách khỏi TC-ORD-012 vì 2 lớp lỗi khác nhau (dung lượng ⟷ định dạng) và để khi FAIL biết ngay lớp nào sai. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N189" s="7" t="inlineStr">
@@ -23242,7 +23726,11 @@
           <t>Ảnh rỗng (test_data_catalog §ORD, biên hợp lệ)</t>
         </is>
       </c>
-      <c r="L190" s="5" t="inlineStr"/>
+      <c r="L190" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M190" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `D8.1` §D8.1 L360 — ảnh là trường tuỳ chọn.</t>
@@ -23319,7 +23807,11 @@
           <t>SĐT người gửi pre-fill (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L191" s="7" t="inlineStr"/>
+      <c r="L191" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M191" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt bằng TC nghi vấn đã quan sát 1 lần — SĐT tự đổi từ `0000142378` sang `0964633313` giữa phiên. · Căn cứ: `KB-VIBE-09` (`KP-01` §10.10). Nếu tái hiện ⇒ **log bug** (`KP-05 §5` #5).</t>
@@ -23396,7 +23888,11 @@
           <t>Cơ chế field địa chỉ (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L192" s="5" t="inlineStr"/>
+      <c r="L192" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M192" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-11` Open — 3 nguồn nêu 3 cơ chế cho cùng field. · Căn cứ: assert theo `KB-ORD-06` (nguồn có bằng chứng app, thắng doc); `LOC-03` §D3 L246 nói preset 6 văn phòng và `US-D01` nói không có chip gợi ý. App hiện 6 chip preset ⇒ FAIL và dẫn `C-ORD-11` để BA chốt.</t>
@@ -23473,7 +23969,11 @@
           <t>Khung giờ mặc định đã trôi qua (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L193" s="7" t="inlineStr"/>
+      <c r="L193" s="7" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
       <c r="M193" s="7" t="inlineStr">
         <is>
           <t>Mục đích: **đây là hành vi ĐÚNG, không phải bug** — ghi thành TC để lượt sau không log bug oan khi form mở lâu. · Căn cứ: `KB-VIBE-10` (`KP-01` §10.11). ⛔ Không assert giá trị mặc định cụ thể — 3 nguồn cho 3 giá trị khác nhau.</t>
@@ -23548,7 +24048,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L194" s="5" t="inlineStr"/>
+      <c r="L194" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M194" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.5.3 + `§A8` L115.</t>
@@ -23625,7 +24129,11 @@
           <t>Chip loại hàng "Thuốc/Y tế" (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L195" s="7" t="inlineStr"/>
+      <c r="L195" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M195" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt bằng TC rằng banner hàng cấm ở v1.0 **chỉ là thông tin tĩnh**, không phải cơ chế chặn — để lượt sau không viết TC negative "bị chặn". · Căn cứ: `C-ORD-04` Resolved 2026-07-27 + `KB-ORD-03`; `BR-ORD-04` §D4 L263 là rule của phase sau.</t>
@@ -23700,7 +24208,11 @@
           <t>Mã tin là giá trị assert-absent (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L196" s="5" t="inlineStr"/>
+      <c r="L196" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M196" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ORD-05` Open — Figma có **2 biến thể** màn này (1 bản có "Mã tin", 1 bản không). · Căn cứ: assert theo `US-D02` §D1b L165 *"KHÔNG hiển thị mã đơn — mã kỹ thuật vô nghĩa với người dùng"* (BRD thắng khi mâu thuẫn về rule). App hiện mã tin ⇒ FAIL và dẫn `C-ORD-05` để BA chốt biến thể.</t>
@@ -23779,7 +24291,11 @@
           <t>Tên 1 ký tự; nhiều field lỗi cùng lúc (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L197" s="7" t="inlineStr"/>
+      <c r="L197" s="7" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M197" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `VAL-02` §D8.3 L393.</t>
@@ -23856,7 +24372,11 @@
           <t>Tên có khoảng trắng đầu cuối; SĐT "090 123.4567" (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L198" s="5" t="inlineStr"/>
+      <c r="L198" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M198" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `VAL-03` §D8.3 L394. Cùng rule trim với lý do huỷ đơn ở `TC-CNL-012` — nếu TC này PASS mà TC-CNL-012 FAIL thì trim chỉ được áp ở một số form, ghi rõ khi log bug.</t>
@@ -23937,7 +24457,7 @@
       <c r="L199" s="7" t="inlineStr"/>
       <c r="M199" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: chỉ assert vế có nguồn (điểm vào wizard luôn là bước 1, theo `SC-ORD-002`). · Căn cứ: ⛔ **KHÔNG assert** form giữ hay xoá dữ liệu đã nhập — `C-ORD-08` Open, chưa có đặc tả, áp `§Custom Rules §10.1`. Khi chạy thì ghi lại hành vi thật vào `C-ORD-08` để BA chốt.</t>
+          <t>Mục đích: chỉ assert vế có nguồn (điểm vào wizard luôn là bước 1, theo `SC-ORD-002`). · Căn cứ: ⛔ **KHÔNG assert** form giữ hay xoá dữ liệu đã nhập — `C-ORD-08` Open, chưa có đặc tả, áp `§Custom Rules §10.1`. Khi chạy thì ghi lại hành vi thật vào `C-ORD-08` để BA chốt. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N199" s="7" t="inlineStr">
@@ -24011,7 +24531,11 @@
           <t>Field số tiền là giá trị assert-absent (test_data_catalog §ORD)</t>
         </is>
       </c>
-      <c r="L200" s="5" t="inlineStr"/>
+      <c r="L200" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M200" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding chốt ranh giới dễ trộn nhất của module — ngưỡng bằng **số tiền** (`BR-ORD-03`) out of scope, còn cảnh báo theo **mức định tính "Cao"** thì CÓ ở v1.0 (`TC-ORD-009`). · Căn cứ: `C-ORD-02` Resolved 2026-07-27 (từng là blocker cứng duy nhất của đợt cũ, đã gỡ) + `KB-ORD-04`.</t>
@@ -24092,7 +24616,7 @@
           <t>Đơn `MATCHED` có ≥2 mốc log; 3 hành động thử: huỷ nhận · sửa tin · huỷ đơn (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L201" s="7" t="inlineStr"/>
+      <c r="L201" s="7" t="n"/>
       <c r="M201" s="7" t="inlineStr">
         <is>
           <t>Mục đích: mở rộng hơn `TC-CNL-010` — không chỉ kiểm 1 hành động đã biết vi phạm mà tìm xem còn đường nào khác cũng làm đổi log. · Căn cứ: `TS-02` §A8 L122 + `BR-INT-04` §A5 L80 (audit bất biến). ⚠ Dự kiến FAIL ở bước 4 — `KB-CNL-01` đã live-verify app XOÁ dòng "Ghép thành công" ⇒ **log bug**; nếu bước 5 hoặc 6 cũng lệch thì log thêm bug riêng cho từng đường.</t>
@@ -24169,7 +24693,7 @@
           <t>1 đơn đi thẳng tới "Hoàn thành" (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L202" s="5" t="inlineStr"/>
+      <c r="L202" s="5" t="n"/>
       <c r="M202" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `TS-01` §A8 L121 + `ORD-04` §D3 L243. ⛔ Không dùng đơn từng bị huỷ nhận — đơn đó thiếu mốc "Ghép thành công" do bug đã biết, sẽ chẩn đoán sai nguyên nhân.</t>
@@ -24245,7 +24769,7 @@
           <t>1 đơn đi thẳng, 3 vai thao tác khác nhau (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L203" s="7" t="inlineStr"/>
+      <c r="L203" s="7" t="n"/>
       <c r="M203" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `TS-01` §A8 L121 — nhóm thông tin "ai thực hiện". Nhóm thứ 5 của rule (actor + lý do của mốc huỷ) verify ở `TC-CNL-009`, không nhồi vào TC này.</t>
@@ -24324,7 +24848,7 @@
           <t>Checkbox điều khoản ở NEED B3 và form OFFER (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L204" s="5" t="inlineStr"/>
+      <c r="L204" s="5" t="n"/>
       <c r="M204" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chỉ assert vế đã chốt (consent ở luồng **đăng tin**). · Căn cứ: `§A8` L115 + `ORD-09` §D3 L245 + `D8.1` L373 + `D8.2` L386. ⚠ Rule `§A8` yêu cầu consent trước khi đăng **VÀ** trước khi ghép, nhưng luồng ghép hiện chỉ có modal xác nhận lộ SĐT — `RISK-TS-04` nghi đây là **gap tuân thủ pháp lý**, đang chờ BA ⇒ ⛔ không assert checkbox ở luồng ghép trong TC này để không trộn 2 phán quyết.</t>
@@ -24404,7 +24928,7 @@
           <t>Cơ chế chặn user dùng làm giá trị assert-absent (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L205" s="7" t="inlineStr"/>
+      <c r="L205" s="7" t="n"/>
       <c r="M205" s="7" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding chứng minh app **đúng phạm vi** — `§A8` L125 khai rõ v1.0 "KHÔNG có chặn (block) người dùng". · Căn cứ: app xuất hiện chức năng này ⇒ FAIL và mở CL scope, không phải log bug.</t>
@@ -24482,7 +25006,7 @@
           <t>1 đơn "Đã giao" quá 4 giờ chưa xác nhận (test_data_catalog §TS — cùng tiền đề `SC-DLV-024`)</t>
         </is>
       </c>
-      <c r="L206" s="5" t="inlineStr"/>
+      <c r="L206" s="5" t="n"/>
       <c r="M206" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chỉ verify **hệ quả phía end-user**; nhánh xử lý của admin thuộc Admin Portal, ⛔ ngoài phạm vi test v1.0. · Căn cứ: `TS-03` §A8 L123 + `BR-CNF-04` §D4 L266 (2 giờ nhắc + 2 giờ admin). Chưa chạy đủ mốc thời gian thì đánh `Blocked` và ghi rõ, ⛔ không đánh PASS.</t>
@@ -24561,7 +25085,7 @@
           <t>Bề mặt Admin dùng làm giá trị assert-absent (test_data_catalog §TS)</t>
         </is>
       </c>
-      <c r="L207" s="7" t="inlineStr"/>
+      <c r="L207" s="7" t="n"/>
       <c r="M207" s="7" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding chốt bằng ID rằng cột `Admin` của permission matrix `§D4` L279-286 **không nằm trong phạm vi test v1.0** — để test report không bị hiểu là đã phủ hết matrix. · Căn cứ: `C-TS-01` Resolved 2026-07-27 (không có đặc tả UI Admin) + `KB-TS-01`.</t>
@@ -24639,7 +25163,11 @@
           <t>Tài khoản SSO CBNV còn hiệu lực (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L208" s="5" t="inlineStr"/>
+      <c r="L208" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M208" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `USR-01` §A6 — bề mặt đăng nhập thuộc host app FoxPro nên chỉ verify được hệ quả danh tính, không verify được nhánh auth âm tính (`RISK-USR-01`).</t>
@@ -24718,7 +25246,7 @@
       <c r="L209" s="7" t="inlineStr"/>
       <c r="M209" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: chốt đúng 4 trường có bằng chứng 2 nguồn — doc `USR-02` liệt kê 6 trường nhưng SĐT / khu vực-văn phòng / kênh liên hệ chưa có bằng chứng UI. · Căn cứ: `§Custom Rules §10.1` + `RISK-USR-02`; 2 trường thiếu bằng chứng theo dõi ở `C-USR-04`, app hiện thêm trường ⇒ mở lại CL chứ không sửa TC.</t>
+          <t>Mục đích: chốt đúng 4 trường có bằng chứng 2 nguồn — doc `USR-02` liệt kê 6 trường nhưng SĐT / khu vực-văn phòng / kênh liên hệ chưa có bằng chứng UI. · Căn cứ: `§Custom Rules §10.1` + `RISK-USR-02`; 2 trường thiếu bằng chứng theo dõi ở `C-USR-04`, app hiện thêm trường ⇒ mở lại CL chứ không sửa TC. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N209" s="7" t="inlineStr">
@@ -24796,7 +25324,7 @@
       <c r="L210" s="5" t="inlineStr"/>
       <c r="M210" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: TC bảo vệ kết luận `C-USR-03` (Resolved 2026-07-24 — view-only); app xuất hiện control sửa ⇒ FAIL và mở lại CL, không im lặng viết TC sửa hồ sơ.</t>
+          <t>Mục đích: TC bảo vệ kết luận `C-USR-03` (Resolved 2026-07-24 — view-only); app xuất hiện control sửa ⇒ FAIL và mở lại CL, không im lặng viết TC sửa hồ sơ. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N210" s="5" t="inlineStr">
@@ -24869,7 +25397,11 @@
           <t>Phòng ban + MNV dạng `FTEL####` (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L211" s="7" t="inlineStr"/>
+      <c r="L211" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M211" s="7" t="inlineStr"/>
       <c r="N211" s="7" t="inlineStr">
         <is>
@@ -24943,7 +25475,7 @@
           <t>Tài khoản có lịch sử đơn; 1 đơn ở trạng thái đã ghép (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L212" s="5" t="inlineStr"/>
+      <c r="L212" s="5" t="n"/>
       <c r="M212" s="5" t="inlineStr">
         <is>
           <t>Mục đích: oracle là **delta +1**, không phải số tuyệt đối — 2 chỉ số là dữ liệu `Runtime` không seed nhanh được nên assert số tuyệt đối sẽ FAIL oan (`RISK-USR-03` Resolved theo hướng delta).</t>
@@ -25019,7 +25551,11 @@
           <t>Bộ giá trị assert-absent: Điểm ECO / Điểm uy tín / CO₂ (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L213" s="7" t="inlineStr"/>
+      <c r="L213" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M213" s="7" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-USR-01` Resolved 2026-07-27 — tier/điểm là phase sau, PRD demo mô tả 3 chỉ số là nguồn thua. App hiện các chỉ số này ⇒ FAIL và mở lại CL.</t>
@@ -25095,7 +25631,11 @@
           <t>Tài khoản "trắng" — cả 2 chỉ số = 0 (test_data_catalog §USR, biên)</t>
         </is>
       </c>
-      <c r="L214" s="5" t="inlineStr"/>
+      <c r="L214" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M214" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp biên với TC-USR-005 — chốt card hiển thị số 0 chứ không ẩn card. · Căn cứ: `USR-05` §A6 L102 định nghĩa chỉ số là số nguyên ≥ 0; text empty state của màn còn chờ `C-ORD-06` nên TC này chỉ assert sự hiện diện và giá trị 0, app ẩn card ⇒ FAIL và dẫn `C-ORD-06`.</t>
@@ -25176,7 +25716,7 @@
       <c r="L215" s="7" t="inlineStr"/>
       <c r="M215" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: badge có bằng chứng Figma nên assert được, nhưng không có logic tier ở v1.0 (`RISK-USR-04`) ⇒ TC này tồn tại để chặn việc viết TC đổi hạng ở lượt sau.</t>
+          <t>Căn cứ: badge có bằng chứng Figma nên assert được, nhưng không có logic tier ở v1.0 (`RISK-USR-04`) ⇒ TC này tồn tại để chặn việc viết TC đổi hạng ở lượt sau. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N215" s="7" t="inlineStr">
@@ -25249,7 +25789,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L216" s="5" t="inlineStr"/>
+      <c r="L216" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M216" s="5" t="inlineStr"/>
       <c r="N216" s="5" t="inlineStr">
         <is>
@@ -25321,7 +25865,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L217" s="7" t="inlineStr"/>
+      <c r="L217" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M217" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: chỉ assert điều hướng; nội dung màn "Quà đã nhận" thuộc module GIFT (`SC-GIFT-006..009`).</t>
@@ -25397,7 +25945,11 @@
           <t>Bộ giá trị assert-absent: SĐT / Workplace / email cấu hình (test_data_catalog §USR)</t>
         </is>
       </c>
-      <c r="L218" s="5" t="inlineStr"/>
+      <c r="L218" s="5" t="inlineStr">
+        <is>
+          <t>Fail</t>
+        </is>
+      </c>
       <c r="M218" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `USR-07` có trong BRD nhưng không có ở 82 ảnh Figma lẫn app STG. · Căn cứ: `C-USR-02` Resolved out of scope v1.0; app xuất hiện bề mặt này ⇒ FAIL và mở lại CL để BA chốt scope.</t>
@@ -25476,7 +26028,7 @@
       <c r="L219" s="7" t="inlineStr"/>
       <c r="M219" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: đối chiếu cấu trúc theo ảnh Figma `570ad9d3…` và `e5764b10…`; chỉ đối chiếu thành phần và thứ tự, không đối chiếu giá trị dữ liệu trong ảnh.</t>
+          <t>Căn cứ: đối chiếu cấu trúc theo ảnh Figma `570ad9d3…` và `e5764b10…`; chỉ đối chiếu thành phần và thứ tự, không đối chiếu giá trị dữ liệu trong ảnh. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N219" s="7" t="inlineStr">
@@ -25552,7 +26104,7 @@
       <c r="L220" s="5" t="inlineStr"/>
       <c r="M220" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 3 nguồn ghi 3 nhãn khác nhau cho cùng mục menu này. · Căn cứ: assert theo nguồn chốt mới nhất là BRD `US-D20` + ảnh Figma; app hiển thị nhãn khác (vd "Đánh giá đã nhận") ⇒ FAIL và báo về `C-USR-04` để BA chốt, ⛔ không tự đổi nhãn trong TC.</t>
+          <t>Mục đích: 3 nguồn ghi 3 nhãn khác nhau cho cùng mục menu này. · Căn cứ: assert theo nguồn chốt mới nhất là BRD `US-D20` + ảnh Figma; app hiển thị nhãn khác (vd "Đánh giá đã nhận") ⇒ FAIL và báo về `C-USR-04` để BA chốt, ⛔ không tự đổi nhãn trong TC. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N220" s="5" t="inlineStr">
@@ -25741,7 +26293,11 @@
         </is>
       </c>
       <c r="L2" s="5" t="inlineStr"/>
-      <c r="M2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr">
+        <is>
+          <t>⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
+        </is>
+      </c>
       <c r="N2" s="5" t="inlineStr">
         <is>
           <t>v1.0</t>
@@ -25812,7 +26368,7 @@
           <t>Tab active mặc định (test_data_catalog §ACT, biên "lần đầu mở màn")</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="n"/>
       <c r="M3" s="7" t="inlineStr"/>
       <c r="N3" s="7" t="inlineStr">
         <is>
@@ -25886,7 +26442,7 @@
           <t>Đơn "Đang giao" + đơn "Hoàn thành" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC này verify **cơ chế switch**, cố ý KHÔNG verify nội dung data của từng tab — nội dung do TC-ACT-004 và TC-ACT-005 đảm nhiệm (`§Custom Rules §10.2`).</t>
@@ -25962,7 +26518,7 @@
           <t>4 đơn đang hoạt động + 1 đơn "Hoàn thành" + 1 đơn "Hết hạn" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đây là chỗ TC gộp tab của đợt cũ **không bắt được lỗi** — case gốc sinh `§Custom Rules §10.2`. · Căn cứ: `DOC-v1.0-02` §3.7 đoạn 2; biên cuối của tab là "Đã giao" (`§D2` L232).</t>
@@ -26042,7 +26598,7 @@
       <c r="L6" s="5" t="inlineStr"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: đơn "Hết hạn" là thứ dễ bị bỏ sót nhất vì tên tab gợi ý chỉ chứa đơn thành công. · Căn cứ: `US-D04` §D1b L166 + `DOC-v1.0-02` §3.7 đoạn 3.</t>
+          <t>Mục đích: đơn "Hết hạn" là thứ dễ bị bỏ sót nhất vì tên tab gợi ý chỉ chứa đơn thành công. · Căn cứ: `US-D04` §D1b L166 + `DOC-v1.0-02` §3.7 đoạn 3. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N6" s="5" t="inlineStr">
@@ -26115,7 +26671,7 @@
           <t>Đơn "Đang giao" của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: đối chiếu cấu trúc theo `DOC-v1.0-05`; ⛔ không assert định dạng ngày và không assert cách rút gọn địa chỉ — cả hai chưa có đặc tả.</t>
@@ -26192,7 +26748,7 @@
           <t>1 đơn "Đã huỷ" dùng làm giá trị assert-absent (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Mục đích: rule ẩn đơn huỷ đối lập trực tiếp với `TS-01` (log tương tác đầy đủ) — đơn biến mất khỏi cả 2 tab là hành vi đã quan sát, cần chốt bằng TC có ID. · Căn cứ: `KB-ORD-07` (#7); đơn huỷ hiện ở 1 trong 2 tab ⇒ FAIL và mở CL để BA chốt tab nào chứa.</t>
@@ -26271,7 +26827,7 @@
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn lệch phần cuối câu lý do. · Căn cứ: assert theo `KB-ORD-07` (#4) vì đây là nguyên văn quan sát trên app kèm bằng chứng; `US-D04` L166 ghi bản ngắn hơn (dừng ở "trong thời gian đăng") là nguồn thua. App hiện bản ngắn ⇒ FAIL và mở CL để BA chốt bản text chính thức.</t>
+          <t>Mục đích: 2 nguồn lệch phần cuối câu lý do. · Căn cứ: assert theo `KB-ORD-07` (#4) vì đây là nguyên văn quan sát trên app kèm bằng chứng; `US-D04` L166 ghi bản ngắn hơn (dừng ở "trong thời gian đăng") là nguồn thua. App hiện bản ngắn ⇒ FAIL và mở CL để BA chốt bản text chính thức. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
@@ -26344,7 +26900,7 @@
           <t>Đơn "Hết hạn" của `SEED-ACT-01`, dùng chung với TC-ACT-008 (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="n"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-ACT-010 — card thao tác được vs không thao tác được.</t>
@@ -26421,7 +26977,7 @@
           <t>2 đơn đang hoạt động khác nhau của `SEED-ACT-01` (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Mục đích: assert theo **dữ liệu của đơn**, cố ý không assert tên màn đích — tên màn còn tranh chấp ở `C-ACT-01` và do TC-ACT-011 đảm nhiệm.</t>
@@ -26498,7 +27054,7 @@
           <t>1 đơn "Chờ ghép" của chính tài khoản (test_data_catalog §ACT)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Mục đích: 2 nguồn nêu 2 màn **khác bản chất** ("Chi tiết tin" public vs "Theo dõi đơn" role-aware). · Căn cứ: assert theo `DOC-v1.0-02` §3.7 + tính nhất quán với `SC-HOME-015` (Trang chủ đã rõ là mở Theo dõi đơn); `KB-ORD-07` (#5) nghi ghi nhầm tên màn. Nếu app mở Chi tiết tin và hiện nút "Tôi mang giúp được" trên đơn của chính mình ⇒ FAIL, log bug theo cùng gốc với `C-ASN-02` và dẫn `C-ACT-01`.</t>
@@ -26578,7 +27134,7 @@
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-ORD-06` Open — module này là **home canonical** của CL, text empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được; ⛔ không assert chuỗi hay ảnh empty state.</t>
+          <t>Mục đích: neo vào `C-ORD-06` Open — module này là **home canonical** của CL, text empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được; ⛔ không assert chuỗi hay ảnh empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -26654,7 +27210,7 @@
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: chuỗi "★★★★★ Đã đánh giá" trên card là **UI leftover**, dễ khiến người sau viết TC chấm sao. · Căn cứ: `C-GIFT-01` Resolved 2026-07-27 — rating 1–5 sao out of scope v1.0, v1.0 chỉ có Quà ảo; ⛔ không assert số sao và không assert sự tồn tại của chuỗi leftover. App mở được màn chấm sao ⇒ FAIL và mở lại CL scope.</t>
+          <t>Mục đích: chuỗi "★★★★★ Đã đánh giá" trên card là **UI leftover**, dễ khiến người sau viết TC chấm sao. · Căn cứ: `C-GIFT-01` Resolved 2026-07-27 — rating 1–5 sao out of scope v1.0, v1.0 chỉ có Quà ảo; ⛔ không assert số sao và không assert sự tồn tại của chuỗi leftover. App mở được màn chấm sao ⇒ FAIL và mở lại CL scope. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -26732,7 +27288,7 @@
       <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: cặp với TC-ACT-012 — empty state phải verify riêng cho từng tab (`§Custom Rules §10.2`). · Căn cứ: `C-ORD-06` Open ⇒ ⛔ không assert chuỗi empty state.</t>
+          <t>Mục đích: cặp với TC-ACT-012 — empty state phải verify riêng cho từng tab (`§Custom Rules §10.2`). · Căn cứ: `C-ORD-06` Open ⇒ ⛔ không assert chuỗi empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr">
@@ -26930,7 +27486,11 @@
           <t>1 tin NEED `POSTED` của tài khoản khác (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-CON-01` §A5 L77 — transition duy nhất của module là `POSTED` → `MATCHED`.</t>
@@ -27009,7 +27569,11 @@
           <t>1 tin NEED `POSTED` (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng âm của TC-ASN-001 — modal phải huỷ được mà không tạo tác động.</t>
@@ -27087,7 +27651,11 @@
           <t>1 tin NEED `POSTED`; 2 tài khoản 2 thiết bị (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-CON-01` §A5 L77 — cơ chế "ghép ngay", không có bước duyệt.</t>
@@ -27172,7 +27740,11 @@
           <t>1 đơn `MATCHED` có khai người nhận (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-CON-02` §A5 L78 + `OPR-07` §D7 L343 + `US-D08` L177 (Carrier thấy cả SĐT người nhận). Đây là vế dương của cặp với TC-ASN-005.</t>
@@ -27250,7 +27822,11 @@
           <t>1 đơn `MATCHED`; 1 tài khoản ngoài cặp (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng âm của TC-ASN-004 — quyền xem SĐT bị giới hạn đúng trong cặp ghép cộng người nhận.</t>
@@ -27339,7 +27915,7 @@
       <c r="L10" s="7" t="inlineStr"/>
       <c r="M10" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: chống double-accept là rủi ro P1 — 2 Carrier cùng nhận sẽ phá tính duy nhất của cặp ghép. · Căn cứ: `ASN-03` §D3 L249 + `OPR-03` §D7 L339. Với 1 tester chỉ kiểm được nhánh gần đồng thời bằng 2 thiết bị; nếu cả hai đều báo thành công ⇒ FAIL và log bug.</t>
+          <t>Mục đích: chống double-accept là rủi ro P1 — 2 Carrier cùng nhận sẽ phá tính duy nhất của cặp ghép. · Căn cứ: `ASN-03` §D3 L249 + `OPR-03` §D7 L339. Với 1 tester chỉ kiểm được nhánh gần đồng thời bằng 2 thiết bị; nếu cả hai đều báo thành công ⇒ FAIL và log bug. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N10" s="7" t="inlineStr">
@@ -27414,7 +27990,11 @@
           <t>1 đơn `MATCHED` (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-03` §D7 L339 + `OPR-08` §D7 L344.</t>
@@ -27495,7 +28075,7 @@
       <c r="L12" s="7" t="inlineStr"/>
       <c r="M12" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `BR-INT-05` §A5 L81 + `DOC-v1.0-02` §4.2. Không assert độ trễ cụ thể — chưa có đặc tả ngưỡng thời gian.</t>
+          <t>Căn cứ: `BR-INT-05` §A5 L81 + `DOC-v1.0-02` §4.2. Không assert độ trễ cụ thể — chưa có đặc tả ngưỡng thời gian. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N12" s="7" t="inlineStr">
@@ -27577,7 +28157,11 @@
           <t>1 tin OFFER + 1 tin NEED trùng 2 điểm, khung giờ giao nhau (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `MTCH-01` §D3 L254 + `US-D12` §D1b L186. Nội dung thông báo còn chờ `C-NTF-01` chốt danh sách chính thức; assert theo chuỗi ở `US-D12`, lệch ⇒ dẫn `C-NTF-01`.</t>
@@ -27656,7 +28240,11 @@
           <t>1 tin NEED khớp tuyến (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D13` §D1b L187. Nhãn nút "Nhận giao" ở luồng khớp tuyến khác nhãn "Tôi mang giúp được" ở luồng Bảng tin — giữ đúng nhãn từng luồng, ⛔ không đồng nhất hoá.</t>
@@ -27735,7 +28323,7 @@
       <c r="L16" s="5" t="inlineStr"/>
       <c r="M16" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 1 trong 2 nhánh negative mà `SC-ASN-011` nêu — nhánh lệch địa điểm. · Căn cứ: `OPR-02` §D7 L338 + `KB-ASN-04` — khớp tuyến là **nhị phân trùng địa chỉ**, ⛔ không dùng bán kính GPS.</t>
+          <t>Mục đích: 1 trong 2 nhánh negative mà `SC-ASN-011` nêu — nhánh lệch địa điểm. · Căn cứ: `OPR-02` §D7 L338 + `KB-ASN-04` — khớp tuyến là **nhị phân trùng địa chỉ**, ⛔ không dùng bán kính GPS. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N16" s="5" t="inlineStr">
@@ -27811,7 +28399,7 @@
       <c r="L17" s="7" t="inlineStr"/>
       <c r="M17" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: nhánh negative thứ hai của `SC-ASN-011` — lệch khung giờ. · Căn cứ: chỉ dùng 2 khung **tách rời hoàn toàn**; ⛔ không test độ lệch nhỏ vì định nghĩa "khung giờ phù hợp" chưa chốt (`C-NTF-02` Partially Resolved).</t>
+          <t>Mục đích: nhánh negative thứ hai của `SC-ASN-011` — lệch khung giờ. · Căn cứ: chỉ dùng 2 khung **tách rời hoàn toàn**; ⛔ không test độ lệch nhỏ vì định nghĩa "khung giờ phù hợp" chưa chốt (`C-NTF-02` Partially Resolved). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
@@ -27886,7 +28474,11 @@
           <t>1 tin OFFER + 1 tin NEED cùng tài khoản, trùng tuyến (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M18" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-05` §D7 L341 — cùng gốc rule với `SC-FEED-011`; app gợi ý tin của chính mình ⇒ FAIL và log bug theo cùng `C-ASN-02`.</t>
@@ -27970,7 +28562,11 @@
           <t>6 tin NEED khớp cùng 1 tuyến OFFER (test_data_catalog §ASN, biên vượt trần)</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr"/>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chạm trần gợi ý — dùng mốc 6 để vượt trần 5. · Căn cứ: `OPR-01` §D7 L337; mốc 3/5/6 là **giá trị BA chốt** (`KB-ASN-03`), ⛔ không thay bằng mốc khác.</t>
@@ -28049,7 +28645,7 @@
       <c r="L21" s="5" t="inlineStr"/>
       <c r="M21" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: mốc dưới trần trong bộ ba 3/5/6 — đối chứng để phân biệt "chặn vì trần" với "không bắn thông báo".</t>
+          <t>Mục đích: mốc dưới trần trong bộ ba 3/5/6 — đối chứng để phân biệt "chặn vì trần" với "không bắn thông báo". · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N21" s="5" t="inlineStr">
@@ -28125,7 +28721,7 @@
       <c r="L22" s="7" t="inlineStr"/>
       <c r="M22" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: mốc đúng trần — biên hợp lệ, cặp với TC-ASN-017 (mốc vượt trần).</t>
+          <t>Mục đích: mốc đúng trần — biên hợp lệ, cặp với TC-ASN-017 (mốc vượt trần). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr">
@@ -28203,7 +28799,7 @@
       <c r="L23" s="5" t="inlineStr"/>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: mốc vượt trần — chốt trần tính **riêng theo từng tin OFFER**. · Căn cứ: `KB-ASN-03` (đảo `OPR-06`) — ⛔ trần KHÔNG cộng dồn theo ngày; nếu app chặn theo ngày ⇒ FAIL và mở CL.</t>
+          <t>Mục đích: mốc vượt trần — chốt trần tính **riêng theo từng tin OFFER**. · Căn cứ: `KB-ASN-03` (đảo `OPR-06`) — ⛔ trần KHÔNG cộng dồn theo ngày; nếu app chặn theo ngày ⇒ FAIL và mở CL. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
@@ -28286,7 +28882,7 @@
       <c r="L25" s="7" t="inlineStr"/>
       <c r="M25" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `OPR-04` §D7 L340 nêu 2 tiêu chí nhưng "độ gần tuyến" là **nhị phân trùng/không trùng** nên không phân biệt được thứ tự ⇒ chỉ còn thời gian đăng làm oracle kiểm chứng được.</t>
+          <t>Căn cứ: `OPR-04` §D7 L340 nêu 2 tiêu chí nhưng "độ gần tuyến" là **nhị phân trùng/không trùng** nên không phân biệt được thứ tự ⇒ chỉ còn thời gian đăng làm oracle kiểm chứng được. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
@@ -28361,7 +28957,11 @@
           <t>1 tin NEED "Hết hạn" (test_data_catalog §ASN — ⛔ không seed được qua UI)</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M26" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-04` §D7 L340 + `US-D04` L166.</t>
@@ -28441,7 +29041,11 @@
           <t>1 đơn `MATCHED` chưa lấy hàng (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L27" s="7" t="inlineStr"/>
+      <c r="L27" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M27" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-08` §D7 L344 + `OPR-09` §D7 L345. Nhánh huỷ nhận sau "Đang giao" bị chặn — verify ở `TC-CNL-*`.</t>
@@ -28518,7 +29122,11 @@
           <t>2 tin NEED liên tiếp cùng tài khoản (test_data_catalog §ASN)</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M28" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-ASN-03` Open — nghi vấn wizard không tạo listing độc lập. · Căn cứ: `DOC-v1.0-02` §7 dòng 3 ghi "Đăng tin mới sẽ ghi đè đơn đang có" nhưng đó là **giới hạn bản demo**, không phải rule nghiệp vụ (`KB-ASN-05`); assert theo hành vi nghiệp vụ đúng. App ghi đè tin cũ ⇒ FAIL và dẫn `C-ASN-03` để BA xác nhận là giới hạn demo hay bug thật.</t>
@@ -28721,7 +29329,7 @@
           <t>Đơn `POSTED`; lý do ≥5 ký tự (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="n"/>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D16` §D1b L195 + `OPR-11` §D7 L347.</t>
@@ -28801,7 +29409,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng; 3 tài khoản 3 vai (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="n"/>
       <c r="M3" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-INT-05` §A5 L81 + `OPR-11` §D7 L347 — quyền huỷ của người gửi còn hiệu lực tới trước "Đang giao".</t>
@@ -28880,7 +29488,7 @@
           <t>Lý do rỗng và lý do ≥5 ký tự (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Mục đích: mốc "rỗng" là mốc duy nhất trong 4 mốc lý do mà app chặn đúng — dùng làm đối chứng dương cho TC-CNL-004 và TC-CNL-012.</t>
@@ -28961,7 +29569,7 @@
       <c r="L5" s="7" t="inlineStr"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: cặp biên 4↔5 ký tự của `VAL-04`. · Căn cứ: `VAL-04` §D8.3 L395 yêu cầu tối thiểu 5 ký tự; `KB-CNL-02` đã live-verify app **chỉ chặn khi rỗng**. ⚠ Dự kiến FAIL ở bước 3 ⇒ **log bug** (tương ứng `TC_08.7` đợt cũ), ⛔ không hạ chuẩn TC theo hành vi app.</t>
+          <t>Mục đích: cặp biên 4↔5 ký tự của `VAL-04`. · Căn cứ: `VAL-04` §D8.3 L395 yêu cầu tối thiểu 5 ký tự; `KB-CNL-02` đã live-verify app **chỉ chặn khi rỗng**. ⚠ Dự kiến FAIL ở bước 3 ⇒ **log bug** (tương ứng `TC_08.7` đợt cũ), ⛔ không hạ chuẩn TC theo hành vi app. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr">
@@ -29037,7 +29645,7 @@
           <t>Đơn `IN_TRANSIT`; 3 tài khoản 3 vai (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Mục đích: phủ hàng "Đang giao" của ma trận quyền huỷ — ranh giới mất quyền huỷ là "Đã ghép" → "Đang giao". · Căn cứ: `OPR-11` §D7 L347 "KHÔNG ai được huỷ" + `BR-ASN-03` §D4 L264.</t>
@@ -29119,7 +29727,7 @@
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `BR-ASN-03` yêu cầu "phải tạo sự cố" thay cho huỷ thường nhưng bề mặt này không có đặc tả. · Căn cứ: `C-CNL-01` Resolved 2026-07-27 out of scope v1.0. **Hệ quả cần nêu với PM:** user gặp sự cố sau khi đã lấy hàng thì không có đường xử lý nào trong app.</t>
+          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `BR-ASN-03` yêu cầu "phải tạo sự cố" thay cho huỷ thường nhưng bề mặt này không có đặc tả. · Căn cứ: `C-CNL-01` Resolved 2026-07-27 out of scope v1.0. **Hệ quả cần nêu với PM:** user gặp sự cố sau khi đã lấy hàng thì không có đường xử lý nào trong app. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -29195,7 +29803,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt khác biệt cốt lõi giữa "Huỷ nhận đơn" (về `POSTED`) và "Huỷ đơn" (`CANCELLED`). · Căn cứ: `OPR-09` §D7 L345 + `US-D16` §D1b L195.</t>
@@ -29274,7 +29882,7 @@
           <t>Đơn `MATCHED`; lý do ≥5 ký tự (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `§D2` L233 + `CNL-01` §D3 L257. Danh sách loại thông báo chính thức còn chờ `C-NTF-01`; lệch nội dung thông báo ⇒ dẫn `C-NTF-01`, không sửa TC.</t>
@@ -29354,7 +29962,7 @@
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-CNL-02` Resolved 2026-07-30 — user chốt **PHẢI ghi log** cho cả 2 hành động huỷ. · Căn cứ: `TS-01`/`TS-02` L121-122 + `KB-CNL-01`; banner đỏ **không thay thế** được log. ⚠ Dự kiến FAIL — app hiện chỉ hiện banner ⇒ **log bug** (tương ứng `TC_08.22` đợt cũ).</t>
+          <t>Mục đích: neo vào `C-CNL-02` Resolved 2026-07-30 — user chốt **PHẢI ghi log** cho cả 2 hành động huỷ. · Căn cứ: `TS-01`/`TS-02` L121-122 + `KB-CNL-01`; banner đỏ **không thay thế** được log. ⚠ Dự kiến FAIL — app hiện chỉ hiện banner ⇒ **log bug** (tương ứng `TC_08.22` đợt cũ). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
@@ -29433,7 +30041,7 @@
       <c r="L11" s="7" t="inlineStr"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: log phải **bất biến** — xoá dòng cũ là phá tính bằng chứng của cả timeline. · Căn cứ: `BR-INT-04` §A5 L80 (audit) + `C-CNL-02`; `KB-CNL-01` đã live-verify app **XOÁ** dòng "Ghép thành công". ⚠ Dự kiến FAIL ⇒ **log bug** (tương ứng `TC_08.23` đợt cũ), cùng gốc với `RISK-TS-01`.</t>
+          <t>Mục đích: log phải **bất biến** — xoá dòng cũ là phá tính bằng chứng của cả timeline. · Căn cứ: `BR-INT-04` §A5 L80 (audit) + `C-CNL-02`; `KB-CNL-01` đã live-verify app **XOÁ** dòng "Ghép thành công". ⚠ Dự kiến FAIL ⇒ **log bug** (tương ứng `TC_08.23` đợt cũ), cùng gốc với `RISK-TS-01`. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -29508,7 +30116,7 @@
           <t>Đơn `MATCHED`; 3 phiên 3 vai trên 3 thiết bị (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-INT-05` §A5 L81 + `§D2` L233. Không assert độ trễ cụ thể — chưa có đặc tả ngưỡng.</t>
@@ -29588,7 +30196,7 @@
       <c r="L13" s="7" t="inlineStr"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: mốc thứ tư trong bộ boundary lý do (rỗng → 4 ký tự → 5 ký tự → 5 dấu cách). · Căn cứ: `VAL-03` §D8.3 L394 (trim) + `VAL-04` L395 — sau khi trim thì lý do rỗng. ⚠ Dự kiến FAIL — `KB-CNL-02` đã live-verify app cho qua ⇒ **log bug** (tương ứng `TC_08.10` đợt cũ).</t>
+          <t>Mục đích: mốc thứ tư trong bộ boundary lý do (rỗng → 4 ký tự → 5 ký tự → 5 dấu cách). · Căn cứ: `VAL-03` §D8.3 L394 (trim) + `VAL-04` L395 — sau khi trim thì lý do rỗng. ⚠ Dự kiến FAIL — `KB-CNL-02` đã live-verify app cho qua ⇒ **log bug** (tương ứng `TC_08.10` đợt cũ). · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr">
@@ -29664,7 +30272,7 @@
           <t>Đơn `POSTED` có khai người nhận (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="n"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
           <t>Mục đích: phủ hàng "Chờ ghép" của ma trận quyền huỷ 3 vai × 3 trạng thái. · Căn cứ: permission matrix `§D4` L285 + `OPR-11` §D7 L347 — người gửi và người nhận huỷ được trước "Đang giao"; ở trạng thái này đơn chưa có người vận chuyển nên hàng Carrier không áp dụng. Vai `Admin` trong matrix ⛔ không test được (`C-TS-01` out of scope).</t>
@@ -29744,7 +30352,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng; 3 tài khoản 3 vai (test_data_catalog §CNL)</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="n"/>
       <c r="M15" s="7" t="inlineStr">
         <is>
           <t>Mục đích: phủ hàng "Đã ghép" của ma trận — đây là trạng thái duy nhất cả 3 vai đều có đường huỷ, nhưng **Carrier dùng hành động khác** (huỷ nhận, không phải huỷ đơn). · Căn cứ: permission matrix `§D4` L285 + `OPR-09` §D7 L345.</t>
@@ -29944,7 +30552,11 @@
           <t>Đơn `POSTED`; vai Sender (test_data_catalog §DLV — ô 1·Sender)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 1·Sender + ảnh Figma `dc8cf987…`.</t>
@@ -30021,7 +30633,7 @@
           <t>Đơn `POSTED`; vai Carrier (test_data_catalog §DLV — ô 1·Carrier)</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="n"/>
       <c r="M4" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 1·Carrier. ⚠ Ô ma trận này nằm ở màn **Chi tiết tin**, không phải màn Theo dõi đơn — Carrier chưa thuộc đơn nên chưa có màn Theo dõi đơn.</t>
@@ -30099,7 +30711,7 @@
           <t>Đơn `POSTED`; vai Receiver (test_data_catalog §DLV — ô 1·Receiver)</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="n"/>
       <c r="M5" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 1·Receiver — quyền "Chỉnh sửa" chỉ thuộc người gửi.</t>
@@ -30185,7 +30797,7 @@
           <t>Đơn `MATCHED`; vai Sender (test_data_catalog §DLV — ô 2·Sender)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
           <t>Mục đích: chốt thời điểm mất quyền "Chỉnh sửa" là khi đơn được ghép — cặp với TC-DLV-001. · Căn cứ: `KB-DLV-01` ô 2·Sender.</t>
@@ -30264,7 +30876,7 @@
           <t>Đơn `MATCHED`; vai Carrier (test_data_catalog §DLV — ô 2·Carrier)</t>
         </is>
       </c>
-      <c r="L8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="n"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 2·Carrier + ảnh Figma `2e2ff7bc…`.</t>
@@ -30343,7 +30955,7 @@
           <t>Đơn `MATCHED`; vai Receiver (test_data_catalog §DLV — ô 2·Receiver)</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 2·Receiver.</t>
@@ -30428,7 +31040,7 @@
           <t>Đơn `IN_TRANSIT`; vai Sender (test_data_catalog §DLV — ô 3·Sender)</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr"/>
+      <c r="L11" s="5" t="n"/>
       <c r="M11" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt ranh giới mất quyền huỷ là "Đã ghép" → "Đang giao" — cùng rule với `TC-CNL-005`. · Căn cứ: `KB-DLV-01` ô 3·Sender + ảnh Figma `c8cae4c3…`.</t>
@@ -30504,7 +31116,11 @@
           <t>Đơn `IN_TRANSIT`; vai Carrier (test_data_catalog §DLV — ô 3·Carrier)</t>
         </is>
       </c>
-      <c r="L12" s="7" t="inlineStr"/>
+      <c r="L12" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M12" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 3·Carrier.</t>
@@ -30580,7 +31196,11 @@
           <t>Đơn `IN_TRANSIT`; vai Receiver (test_data_catalog §DLV — ô 3·Receiver)</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr"/>
+      <c r="L13" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 3·Receiver + ảnh Figma `ca5e7239…`.</t>
@@ -30663,7 +31283,11 @@
           <t>Đơn `DELIVERED`; vai Sender (test_data_catalog §DLV — ô 4·Sender)</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 4·Sender + ảnh Figma `8563adc1…`.</t>
@@ -30741,7 +31365,11 @@
           <t>Đơn `DELIVERED`; vai Carrier (test_data_catalog §DLV — ô 4·Carrier)</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt quyền hoàn tất đơn đã chuyển sang người nhận — bộ ba TC-DLV-010/011/012 là điểm phân định của `C-DLV-01`. · Căn cứ: `KB-DLV-01` ô 4·Carrier + `DOC-v1.0-02` §4.3.</t>
@@ -30817,7 +31445,11 @@
           <t>Đơn `DELIVERED`; vai Receiver (test_data_catalog §DLV — ô 4·Receiver)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đây là **nút enable duy nhất** ở trạng thái "Đã giao" trong 3 vai; nếu ô này disable thì đơn không bao giờ hoàn tất được và toàn bộ module `GIFT` bị blocked. · Căn cứ: `KB-DLV-01` ô 4·Receiver + `DOC-v1.0-02` §5.2 + `C-DLV-01` Resolved (Receiver-only).</t>
@@ -30900,7 +31532,7 @@
           <t>Đơn `COMPLETED` chưa gửi quà; vai Sender (test_data_catalog §DLV — ô 5·Sender)</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr"/>
+      <c r="L19" s="5" t="n"/>
       <c r="M19" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 5·Sender + ảnh Figma `19490aa9…`. Nhãn sau khi gửi quà đổi thành "Bạn đã đánh giá" — verify ở `TC-GIFT-005`.</t>
@@ -30976,7 +31608,11 @@
           <t>Đơn `COMPLETED`; vai Carrier (test_data_catalog §DLV — ô 5·Carrier)</t>
         </is>
       </c>
-      <c r="L20" s="7" t="inlineStr"/>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M20" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 5·Carrier + ảnh Figma `2658b17b…`.</t>
@@ -31052,7 +31688,11 @@
           <t>Đơn `COMPLETED`; vai Receiver (test_data_catalog §DLV — ô 5·Receiver)</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M21" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` ô 5·Receiver + ảnh Figma `76e115a2…`.</t>
@@ -31138,7 +31778,7 @@
           <t>Đơn qua 3 trạng thái đầu (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L23" s="7" t="inlineStr"/>
+      <c r="L23" s="7" t="n"/>
       <c r="M23" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `US-D09` §D1b L178 + `§D2` L232. ⚠ Mốc thứ hai trên thanh ghi "Lấy hàng" trong khi badge trạng thái ghi "Đã ghép" — 2 chữ cho cùng 1 trạng thái, ⛔ không sửa TC theo chữ của badge.</t>
@@ -31217,7 +31857,7 @@
           <t>Đơn `MATCHED`; nội dung popup lấy hàng (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr"/>
+      <c r="L24" s="5" t="n"/>
       <c r="M24" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` bảng popup — tiêu đề popup cố định là "Xác nhận" cho cả 3 hành động.</t>
@@ -31296,7 +31936,7 @@
           <t>Đơn `IN_TRANSIT`; nội dung popup đã giao (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L25" s="7" t="inlineStr"/>
+      <c r="L25" s="7" t="n"/>
       <c r="M25" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` bảng popup.</t>
@@ -31375,7 +32015,7 @@
           <t>Đơn `DELIVERED`; nội dung popup nhận hàng (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="n"/>
       <c r="M26" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `KB-DLV-01` bảng popup + `KB-DLV-03`.</t>
@@ -31454,7 +32094,7 @@
           <t>Đơn `MATCHED` (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L27" s="7" t="inlineStr"/>
+      <c r="L27" s="7" t="n"/>
       <c r="M27" s="7" t="inlineStr">
         <is>
           <t>Mục đích: đối chứng âm cho TC-DLV-017 — popup phải huỷ được mà không tạo tác động, kể cả tác động lên log. · Căn cứ: `DOC-v1.0-02` §6 L191.</t>
@@ -31541,7 +32181,7 @@
           <t>Đơn `MATCHED` chưa lấy hàng (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L29" s="5" t="inlineStr"/>
+      <c r="L29" s="5" t="n"/>
       <c r="M29" s="5" t="inlineStr">
         <is>
           <t>Mục đích: TC này khác `TC-DLV-005` — TC-DLV-005 assert **nhãn nút đúng**, TC này assert **không tồn tại đường vòng nào** (mở từ màn khác, nút ẩn). · Căn cứ: `US-D09` §D1b L178. Nhảy bước được ⇒ đơn "đã giao" mà chưa từng lấy hàng, phá tính bằng chứng của timeline và cả `TS-01`.</t>
@@ -31620,7 +32260,7 @@
           <t>Đơn `DELIVERED`; 3 tài khoản 3 vai (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L30" s="7" t="inlineStr"/>
+      <c r="L30" s="7" t="n"/>
       <c r="M30" s="7" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-DLV-01` Resolved 2026-07-24 — `DLV-03` §D3 ghi "RECEIVER/**SENDER**" nhưng `BR-INT-03` §A5 L79 + demo §5.2 + 5 ảnh Figma đều cho **Receiver-only**. · Căn cứ: nguồn chốt là `BR-INT-03` + bằng chứng Figma; app cho Sender chốt đơn ⇒ FAIL và mở lại CL.</t>
@@ -31697,7 +32337,7 @@
           <t>Đơn `DELIVERED` (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr"/>
+      <c r="L31" s="5" t="n"/>
       <c r="M31" s="5" t="inlineStr">
         <is>
           <t>Mục đích: đây là điểm đóng đơn — nếu có bước chờ ẩn thì người gửi không bao giờ tặng quà được và module `GIFT` bị blocked. · Căn cứ: `DOC-v1.0-02` §5.2 dòng "Sau khi xác nhận". ⛔ Không assert chuỗi "Hoàn thành &amp; đã đánh giá" — chuỗi đó là UI leftover của cơ chế rating đã bị `C-GIFT-01` loại khỏi v1.0.</t>
@@ -31775,7 +32415,7 @@
           <t>Đơn `DELIVERED` với mốc thời gian 2 giờ và 4 giờ (test_data_catalog §DLV — cần dev seed timestamp)</t>
         </is>
       </c>
-      <c r="L32" s="7" t="inlineStr"/>
+      <c r="L32" s="7" t="n"/>
       <c r="M32" s="7" t="inlineStr">
         <is>
           <t>Mục đích: dùng chung tiền đề với `SC-TS-006` ⇒ chạy 1 lần lấy dữ liệu cho cả 2 TC. · Căn cứ: `BR-CNF-04` §D4 L266 + `US-D14` §D1b L193; nhánh xử lý của admin thuộc Admin Portal, ⛔ ngoài phạm vi v1.0. Chưa chạy đủ mốc thời gian thì đánh `Blocked` và ghi rõ, ⛔ không đánh PASS cho xong.</t>
@@ -31851,7 +32491,7 @@
           <t>Bộ giá trị assert-absent: ảnh bằng chứng / điểm uy tín / chi phí (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr"/>
+      <c r="L33" s="5" t="n"/>
       <c r="M33" s="5" t="inlineStr">
         <is>
           <t>Mục đích: neo vào `C-DLV-03` Resolved 2026-07-27 — form đầy đủ ở PRD §5.3 **không áp dụng v1.0**. · Căn cứ: `KB-DLV-03` (bằng chứng app dùng modal đơn giản); app hiện form đầy đủ ⇒ FAIL và mở lại CL scope.</t>
@@ -31936,7 +32576,11 @@
           <t>Đơn qua `POSTED` → `MATCHED`; vai Sender (test_data_catalog §DLV, biên thời điểm lộ liên hệ)</t>
         </is>
       </c>
-      <c r="L35" s="7" t="inlineStr"/>
+      <c r="L35" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M35" s="7" t="inlineStr">
         <is>
           <t>Mục đích: ranh giới "Chờ ghép" → "Đã ghép" là thời điểm cụm liên hệ được phép xuất hiện — cùng rule với `TC-FEED-010`. · Căn cứ: `DOC-v1.0-02` §3.6 + `BR-CON-02` §A5 L78.</t>
@@ -32012,7 +32656,11 @@
           <t>Đơn `MATCHED` có khai người nhận; vai Carrier (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L36" s="5" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M36" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §4.3 + `US-D08` §D1b L177 — người vận chuyển là vai duy nhất thấy liên hệ 2 đầu.</t>
@@ -32089,7 +32737,11 @@
           <t>Đơn `MATCHED`; vai Receiver (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L37" s="7" t="n"/>
+      <c r="L37" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M37" s="7" t="inlineStr">
         <is>
           <t>Mục đích: giới hạn phạm vi lộ liên hệ theo vai — người nhận không có nhu cầu liên hệ người gửi trong luồng v1.0. · Căn cứ: `DOC-v1.0-02` §5.2 dòng "Liên hệ".</t>
@@ -32165,7 +32817,11 @@
           <t>Đơn đi thẳng tới `COMPLETED` (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M38" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `DOC-v1.0-02` §3.6 dòng "Lịch sử" + `US-D09` §D1b L178. ⚠ Danh sách mốc này **khác** thanh trạng thái ở `TC-DLV-016` (có "Đăng tin" và "Ghép thành công"). ⛔ Không dùng đơn từng bị huỷ nhận — đơn đó thiếu dòng "Ghép thành công" do bug đã biết (`TC-CNL-010`).</t>
@@ -32244,7 +32900,7 @@
           <t>Tập 3 nhãn phụ theo vai (test_data_catalog §DLV)</t>
         </is>
       </c>
-      <c r="L39" s="7" t="inlineStr"/>
+      <c r="L39" s="7" t="n"/>
       <c r="M39" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: tiêu đề section `DOC-v1.0-02` §3.6/§4.3/§5.2.</t>
@@ -32447,7 +33103,7 @@
           <t>≥2 tin NEED `POSTED` + 1 tin OFFER (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="n"/>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-03` §D7 L339 — tin đã ghép bị ẩn khỏi bảng tin nên chỉ đếm tin ở trạng thái "Chờ ghép".</t>
@@ -32527,7 +33183,7 @@
       <c r="L3" s="7" t="inlineStr"/>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: ⛔ không assert nút CTA trên card — `C-FEED-01(a)` Open (`US-D07` nói có ở card, PRD §3.3 không liệt kê); badge "Tin của bạn" verify riêng ở TC-FEED-003/004.</t>
+          <t>Căn cứ: ⛔ không assert nút CTA trên card — `C-FEED-01(a)` Open (`US-D07` nói có ở card, PRD §3.3 không liệt kê); badge "Tin của bạn" verify riêng ở TC-FEED-003/004. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -32600,7 +33256,7 @@
           <t>1 tin NEED của chính tài khoản đang xem (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="n"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-FEED-004.</t>
@@ -32678,7 +33334,7 @@
           <t>1 tin NEED của tài khoản khác (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="n"/>
       <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-FEED-003.</t>
@@ -32756,7 +33412,7 @@
           <t>≥2 tin NEED `POSTED` khác nhau (test_data_catalog §FEED, biên "≥2 tin")</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="n"/>
       <c r="M6" s="5" t="inlineStr"/>
       <c r="N6" s="5" t="inlineStr">
         <is>
@@ -32829,7 +33485,7 @@
           <t>1 tin có ảnh JPG ≤5MB + ghi chú ≤300 ký tự (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="n"/>
       <c r="M7" s="7" t="inlineStr"/>
       <c r="N7" s="7" t="inlineStr">
         <is>
@@ -32906,7 +33562,7 @@
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: ⛔ không assert giá trị số "~X km" — dữ liệu runtime, không seed được.</t>
+          <t>Căn cứ: ⛔ không assert giá trị số "~X km" — dữ liệu runtime, không seed được. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -32980,7 +33636,7 @@
           <t>1 tin không có ảnh (test_data_catalog §FEED, biên)</t>
         </is>
       </c>
-      <c r="L9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="n"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: ⛔ không assert nội dung ảnh mặc định — chưa có đặc tả hình ảnh.</t>
@@ -33062,7 +33718,7 @@
       <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-FEED-01(b)` Open — chính doc `§7 dòng 10` đặt câu hỏi bản chính thức có tích hợp bản đồ thật hay không. · Căn cứ: assert theo trạng thái đã mô tả ở PRD (placeholder); app v1.0 có bản đồ thật ⇒ FAIL và dẫn `C-FEED-01` để BA chốt scope, ⛔ không tự mở rộng TC sang bản đồ thật.</t>
+          <t>Mục đích: neo vào `C-FEED-01(b)` Open — chính doc `§7 dòng 10` đặt câu hỏi bản chính thức có tích hợp bản đồ thật hay không. · Căn cứ: assert theo trạng thái đã mô tả ở PRD (placeholder); app v1.0 có bản đồ thật ⇒ FAIL và dẫn `C-FEED-01` để BA chốt scope, ⛔ không tự mở rộng TC sang bản đồ thật. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N10" s="5" t="inlineStr">
@@ -33136,7 +33792,7 @@
           <t>1 tin NEED `POSTED`; tài khoản xem không thuộc cặp ghép (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
           <t>Mục đích: assert đúng thời điểm được phép lộ SĐT — đây là ranh giới "Chờ ghép → Đã ghép". · Căn cứ: `BR-CON-02` §A5 L78 + `OPR-07` §D7 L343; `C-ASN-01` Resolved 2026-07-27 xác nhận SĐT **chỉ** lộ sau ghép và hành vi lộ sớm là **bug**. ⚠ Dự kiến FAIL trên app/prototype hiện tại (`KP-05 §5` #6) ⇒ **log bug**, ⛔ không sửa TC theo hành vi app.</t>
@@ -33212,7 +33868,7 @@
           <t>1 tin NEED của chính tài khoản đang xem (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="n"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `OPR-05` §D7 L341; `C-ASN-02` Resolved 2026-07-27 — chủ tin KHÔNG được tự nhận mang giúp, hành vi prototype cho phép là **bug**. ⚠ Dự kiến FAIL (`KP-05 §5` #7) ⇒ **log bug**, ⛔ không sửa TC.</t>
@@ -33289,7 +33945,7 @@
           <t>1 tin NEED khai người nhận là tài khoản đang xem (test_data_catalog §FEED, biên chủ thể thứ ba)</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="n"/>
       <c r="M13" s="7" t="inlineStr">
         <is>
           <t>Mục đích: ca chủ thể thứ ba — không phải chủ tin nhưng cũng không được nhận đơn. · Căn cứ: `DOC-v1.0-02` §7 dòng 9 (nguồn duy nhất mô tả ca này). ⚠ Dự kiến FAIL ⇒ log bug, dẫn `OPR-05` để BA xác nhận rule áp cho cả vai người nhận.</t>
@@ -33370,7 +34026,7 @@
       <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-ORD-06` Open — text và ảnh empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được (không có card, khung màn còn nguyên); ⛔ không assert chuỗi empty state.</t>
+          <t>Mục đích: neo vào `C-ORD-06` Open — text và ảnh empty state chưa có đặc tả. · Căn cứ: chỉ assert phần suy được (không có card, khung màn còn nguyên); ⛔ không assert chuỗi empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N14" s="5" t="inlineStr">
@@ -33446,7 +34102,7 @@
           <t>≥6 tin NEED `POSTED` (test_data_catalog §FEED)</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="n"/>
       <c r="M15" s="7" t="inlineStr"/>
       <c r="N15" s="7" t="inlineStr">
         <is>
@@ -33634,7 +34290,11 @@
           <t>1 đơn "Hoàn thành" chưa gửi quà (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M2" s="5" t="inlineStr">
         <is>
           <t>Căn cứ: `§A7` L107 + `KB-GIFT-01` (ô 5·Sender của ma trận nhãn nút).</t>
@@ -33713,7 +34373,7 @@
       <c r="L3" s="7" t="inlineStr"/>
       <c r="M3" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `§A7` L108 + `GIFT-01` §D3 L258 + `DOC-v1.0-02` §3.8 — ba nguồn khớp nhau về 4 loại.</t>
+          <t>Căn cứ: `§A7` L108 + `GIFT-01` §D3 L258 + `DOC-v1.0-02` §3.8 — ba nguồn khớp nhau về 4 loại. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N3" s="7" t="inlineStr">
@@ -33790,7 +34450,7 @@
       <c r="L4" s="5" t="inlineStr"/>
       <c r="M4" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn ghi 2 chuỗi popup khác nhau. · Căn cứ: assert theo PRD §3.8 + Figma; `US-D15` L194 ghi "Cảm ơn của bạn đã được gửi" là nguồn thua. App hiện chuỗi của `US-D15` ⇒ FAIL và dẫn `C-GIFT-03` để BA chốt text. Lượt chạy TC này tiêu 1 đơn Hoàn thành.</t>
+          <t>Mục đích: 2 nguồn ghi 2 chuỗi popup khác nhau. · Căn cứ: assert theo PRD §3.8 + Figma; `US-D15` L194 ghi "Cảm ơn của bạn đã được gửi" là nguồn thua. App hiện chuỗi của `US-D15` ⇒ FAIL và dẫn `C-GIFT-03` để BA chốt text. Lượt chạy TC này tiêu 1 đơn Hoàn thành. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
@@ -33863,7 +34523,11 @@
           <t>Bộ giá trị assert-absent: giá tiền / ví / cổng thanh toán / quy đổi điểm (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M5" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `BR-GIFT-01` §D4 L271 + `§A7` L111 — quà là biểu tượng phi vật chất; app xuất hiện thành phần thanh toán ⇒ FAIL và mở CL scope.</t>
@@ -33943,7 +34607,11 @@
           <t>1 đơn "Hoàn thành"; số lần gửi quà lần 1 → lần 2 (test_data_catalog §GIFT, biên)</t>
         </is>
       </c>
-      <c r="L6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M6" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp biên lần 1 enable → lần 2 disable; TC này tiêu 1 đơn Hoàn thành. · Căn cứ: `KB-GIFT-01` — nhãn "Bạn đã đánh giá" là **UI leftover** của cơ chế rating đã out of scope, ⛔ không suy ra là có chức năng chấm điểm.</t>
@@ -34022,7 +34690,7 @@
       <c r="L7" s="7" t="inlineStr"/>
       <c r="M7" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: rule *"chỉ hiện loại count&gt;0"* là điểm dễ hiểu sai thành "hiện 4 loại với số 0". · Căn cứ: `KB-GIFT-03` + `US-D20` §D1b L196.</t>
+          <t>Mục đích: rule *"chỉ hiện loại count&gt;0"* là điểm dễ hiểu sai thành "hiện 4 loại với số 0". · Căn cứ: `KB-GIFT-03` + `US-D20` §D1b L196. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr">
@@ -34098,7 +34766,7 @@
       <c r="L8" s="5" t="inlineStr"/>
       <c r="M8" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-GIFT-03` Open — vế "có danh sách lịch sử hay không". · Căn cứ: assert theo `US-D20` §D1b L196 (nguồn văn bản duy nhất nêu danh sách này), chưa có ảnh Figma hay app xác nhận. ⚠ Dự kiến FAIL ⇒ báo về `C-GIFT-03`, ⛔ không im lặng bỏ qua như đợt cũ.</t>
+          <t>Mục đích: neo vào `C-GIFT-03` Open — vế "có danh sách lịch sử hay không". · Căn cứ: assert theo `US-D20` §D1b L196 (nguồn văn bản duy nhất nêu danh sách này), chưa có ảnh Figma hay app xác nhận. ⚠ Dự kiến FAIL ⇒ báo về `C-GIFT-03`, ⛔ không im lặng bỏ qua như đợt cũ. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N8" s="5" t="inlineStr">
@@ -34174,7 +34842,7 @@
       <c r="L9" s="7" t="inlineStr"/>
       <c r="M9" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-ORD-06` Open — text empty state chưa có đặc tả. · Căn cứ: suy từ rule `KB-GIFT-03` (chỉ hiện loại count&gt;0) ⇒ 0 loại thì không có card loại nào; ⛔ không assert chuỗi empty state.</t>
+          <t>Mục đích: neo vào `C-ORD-06` Open — text empty state chưa có đặc tả. · Căn cứ: suy từ rule `KB-GIFT-03` (chỉ hiện loại count&gt;0) ⇒ 0 loại thì không có card loại nào; ⛔ không assert chuỗi empty state. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr">
@@ -34247,7 +34915,11 @@
           <t>Tài khoản đã nhận ≥1 quà (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M10" s="5" t="inlineStr"/>
       <c r="N10" s="5" t="inlineStr">
         <is>
@@ -34321,10 +34993,10 @@
           <t>2 đơn "Hoàn thành" khác tuyến (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="n"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Mục đích: neo vào `C-GIFT-02` Open — đã quan sát back nhảy sang màn "Xác nhận đã nhận hàng" của **đơn khác**. · Căn cứ: `KB-GIFT-04`; dùng 2 đơn để phát hiện nhảy sai đơn. ⚠ Dự kiến FAIL ⇒ **log bug** (`KP-05 §5` #9).</t>
+          <t>Mục đích: neo vào `C-GIFT-02` Open — đã quan sát back nhảy sang màn "Xác nhận đã nhận hàng" của **đơn khác**. · Căn cứ: `KB-GIFT-04`; dùng 2 đơn để phát hiện nhảy sai đơn. ⚠ Dự kiến FAIL ⇒ **log bug** (`KP-05 §5` #9). · ⚠️ Đã chạy nhưng THIẾU EVIDENCE hợp lệ ⇒ không ghi PASS, tính Not Run (gate verify_evidence.py).</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -34403,7 +35075,7 @@
       <c r="L12" s="5" t="inlineStr"/>
       <c r="M12" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `RAT-01/02` có trong BRD nhưng `C-GIFT-01` Resolved 2026-07-27 loại khỏi v1.0. · Căn cứ: `BR-INT-06` §A5 L82 + `§A8` L125; chuỗi "★★★★★ Đã đánh giá" và nhãn "Bạn đã đánh giá" là UI leftover, ⛔ không suy ra có chức năng.</t>
+          <t>Mục đích: TC dạng GAP finding theo `§Custom Rules §10.1` — `RAT-01/02` có trong BRD nhưng `C-GIFT-01` Resolved 2026-07-27 loại khỏi v1.0. · Căn cứ: `BR-INT-06` §A5 L82 + `§A8` L125; chuỗi "★★★★★ Đã đánh giá" và nhãn "Bạn đã đánh giá" là UI leftover, ⛔ không suy ra có chức năng. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N12" s="5" t="inlineStr">
@@ -34478,7 +35150,11 @@
           <t>1 đơn "Hoàn thành"; text thông báo `NTF-07` (test_data_catalog §GIFT)</t>
         </is>
       </c>
-      <c r="L13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M13" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: `NTF-07` §D6 L325 + `§A7` L109; Figma bổ sung dòng thứ hai *"[Tên] đã gửi tặng bạn một món quà…"* nên ⛔ không assert thông báo chỉ có đúng 1 dòng. Danh sách loại thông báo chính thức còn chờ `C-NTF-01`. · Cập nhật 2026-09-21 (QC GiangDC2 chốt): nhấn thông báo `NTF-07` mở màn "Quà đã nhận" là ĐÚNG hành vi — sửa Expected step 4 theo app (trước ghi "màn Cá nhân"); không phải bug. ⚠ App chưa hiển thị emoji 🎁 ở thông báo — trang trí, ⛔ không assert.</t>
@@ -34675,7 +35351,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M3" s="5" t="inlineStr"/>
       <c r="N3" s="5" t="inlineStr">
         <is>
@@ -34753,7 +35433,11 @@
           <t>1 đơn đang hoạt động + ≥1 tin cộng đồng (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L4" s="7" t="inlineStr"/>
+      <c r="L4" s="7" t="inlineStr">
+        <is>
+          <t>Blocked</t>
+        </is>
+      </c>
       <c r="M4" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: màn "Tặng quà" nằm trong cùng luật nhưng cần đơn ở trạng thái Hoàn thành nên verify ở `TC-GIFT-*`, không nhồi vào TC này.</t>
@@ -34828,7 +35512,11 @@
           <t>Tên hiển thị từ hồ sơ nhân viên (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L5" s="5" t="inlineStr"/>
+      <c r="L5" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M5" s="5" t="inlineStr"/>
       <c r="N5" s="5" t="inlineStr">
         <is>
@@ -34903,7 +35591,7 @@
           <t>3 tài khoản 3 vai trên cùng 1 đơn (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L6" s="7" t="inlineStr"/>
+      <c r="L6" s="7" t="n"/>
       <c r="M6" s="7" t="inlineStr">
         <is>
           <t>Mục đích: assert được vế "có icon và phân biệt theo vai" mà không cần mapping icon cụ thể. · Căn cứ: `DOC-v1.0-02` §2 nêu header có icon vai trò; mapping icon↔vai **chưa chốt** (`C-HOME-01` Open) nên ⛔ không assert hình icon. Ba vai cùng một icon hoặc thiếu icon ⇒ FAIL và dẫn `C-HOME-01`.</t>
@@ -34978,7 +35666,11 @@
           <t>≥1 thông báo chưa đọc (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L7" s="5" t="inlineStr"/>
+      <c r="L7" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng dương với TC-HOME-006.</t>
@@ -35055,7 +35747,11 @@
           <t>0 thông báo chưa đọc (test_data_catalog §HOME, biên)</t>
         </is>
       </c>
-      <c r="L8" s="7" t="inlineStr"/>
+      <c r="L8" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M8" s="7" t="inlineStr">
         <is>
           <t>Mục đích: cặp đối chứng âm với TC-HOME-005. · Căn cứ: cơ chế đánh dấu đã đọc còn chờ `C-NTF-03(a)`; TC dùng đường mở từng item nên không phụ thuộc nút mark-all, app không hạ chấm sau khi đọc hết ⇒ FAIL và dẫn `C-NTF-03`.</t>
@@ -35132,7 +35828,11 @@
           <t>Tagline banner (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr"/>
+      <c r="L9" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
           <t>Mục đích: banner hiển thị đúng tagline đã chốt. · Căn cứ: dùng chuỗi PRD "Tiện đường — Giúp đồng nghiệp" (`C-HOME-01(b)` RESOLVED 2026-09-15 — khớp design HOME_01/02/04; PRD thắng khi mô tả chi tiết màn hình, `MASTER-MEMORY §2`). BRD `§A3` L29 "Đồng nghiệp giúp nhau" là nguồn lỗi thời. · 2026-09-21: sửa Expected từ chuỗi BRD sang chuỗi PRD sau VR-005 (app hiện đúng chuỗi PRD).</t>
@@ -35217,7 +35917,7 @@
       <c r="L11" s="7" t="inlineStr"/>
       <c r="M11" s="7" t="inlineStr">
         <is>
-          <t>Căn cứ: `§A7` L111 loại điểm/CO₂ khỏi v1.0 (`C-USR-01` Resolved). ⛔ Không assert giá trị của [x]/[y] — số toàn hệ thống, không seed được.</t>
+          <t>Căn cứ: `§A7` L111 loại điểm/CO₂ khỏi v1.0 (`C-USR-01` Resolved). ⛔ Không assert giá trị của [x]/[y] — số toàn hệ thống, không seed được. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
@@ -35290,7 +35990,11 @@
           <t>1 đơn Fixture ở trạng thái "Chờ ghép" (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M12" s="5" t="inlineStr"/>
       <c r="N12" s="5" t="inlineStr">
         <is>
@@ -35441,7 +36145,11 @@
           <t>Nhãn vai `Gửi:` (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M14" s="5" t="inlineStr">
         <is>
           <t>Mục đích: 1 trong 3 ca phân biệt nhãn theo vai — bộ ba TC-HOME-011/012/013 phải khác nhãn nhau.</t>
@@ -35518,7 +36226,11 @@
           <t>Nhãn vai `Giao:`; 1 tin NEED của tài khoản khác (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M15" s="7" t="inlineStr">
         <is>
           <t>Mục đích: 1 trong 3 ca phân biệt nhãn theo vai.</t>
@@ -35594,7 +36306,11 @@
           <t>Nhãn vai `Nhận:`; 1 đơn có tài khoản ở vai người nhận (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M16" s="5" t="inlineStr">
         <is>
           <t>Mục đích: 1 trong 3 ca phân biệt nhãn theo vai. · Căn cứ: vai Receiver do Sender chỉ định khi đăng tin nên phải seed từ tài khoản khác, không dựng được bằng chính tài khoản đang test.</t>
@@ -35676,7 +36392,7 @@
           <t>Badge thuộc tập {Chờ ghép, Đã ghép, Đang giao, Đã giao, Hoàn thành}; 5 mốc progress (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="n"/>
       <c r="M17" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: 5 mốc lấy từ `§D2` L232. Trạng thái "Hoàn thành" verify ở `TC-ACT-*` vì đó là ranh giới đơn còn/không còn "đang hoạt động" và chưa có đặc tả rõ (`test_data_catalog §HOME` biên).</t>
@@ -35752,7 +36468,11 @@
           <t>1 đơn Fixture ở trạng thái "Chờ ghép" (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M18" s="5" t="inlineStr"/>
       <c r="N18" s="5" t="inlineStr">
         <is>
@@ -35824,7 +36544,11 @@
           <t>1 đơn Fixture ở trạng thái "Chờ ghép" (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L19" s="7" t="inlineStr"/>
+      <c r="L19" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M19" s="7" t="inlineStr">
         <is>
           <t>Căn cứ: nút này không có mô tả trong BRD/PRD (`KP-05 §3` #1) nên chỉ assert đích điều hướng, ⛔ không assert tab mặc định hay bộ lọc của màn Hoạt động.</t>
@@ -35908,7 +36632,7 @@
           <t>≥1 tin cộng đồng còn hiệu lực (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr"/>
+      <c r="L21" s="5" t="n"/>
       <c r="M21" s="5" t="inlineStr">
         <is>
           <t>Mục đích: chốt "Tin mới" KHÔNG phải tính năng riêng của Carrier — neo vào `C-ORD-07` và `KB-ORD-08`.</t>
@@ -35985,7 +36709,7 @@
           <t>≥1 tin cộng đồng còn hiệu lực (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L22" s="7" t="inlineStr"/>
+      <c r="L22" s="7" t="n"/>
       <c r="M22" s="7" t="inlineStr"/>
       <c r="N22" s="7" t="inlineStr">
         <is>
@@ -36061,7 +36785,7 @@
       <c r="L23" s="5" t="inlineStr"/>
       <c r="M23" s="5" t="inlineStr">
         <is>
-          <t>Mục đích: 2 nguồn ghi 2 con số cho cùng một section (1 tin vs tối đa 5 tin). · Căn cứ: assert theo BRD `US-D06` §D1b L175 "chỉ hiện tối đa 5 tin" — BRD thắng PRD khi mâu thuẫn về rule (`MASTER-MEMORY §2`); app hiện đúng 1 tin ⇒ FAIL và dẫn `C-HOME-03` để BA chốt.</t>
+          <t>Mục đích: 2 nguồn ghi 2 con số cho cùng một section (1 tin vs tối đa 5 tin). · Căn cứ: assert theo BRD `US-D06` §D1b L175 "chỉ hiện tối đa 5 tin" — BRD thắng PRD khi mâu thuẫn về rule (`MASTER-MEMORY §2`); app hiện đúng 1 tin ⇒ FAIL và dẫn `C-HOME-03` để BA chốt. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N23" s="5" t="inlineStr">
@@ -36135,7 +36859,7 @@
           <t>≥1 tin cộng đồng còn hiệu lực (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L24" s="7" t="inlineStr"/>
+      <c r="L24" s="7" t="n"/>
       <c r="M24" s="7" t="inlineStr"/>
       <c r="N24" s="7" t="inlineStr">
         <is>
@@ -36213,7 +36937,7 @@
       <c r="L25" s="5" t="inlineStr"/>
       <c r="M25" s="5" t="inlineStr">
         <is>
-          <t>Căn cứ: rule hiện/ẩn nút theo mốc 5 vs ≥6 tin **không có nguồn tài liệu** (`KP-05 §3` #2) nên TC chỉ assert nhánh có đủ tin, ⛔ không assert nhánh ẩn nút.</t>
+          <t>Căn cứ: rule hiện/ẩn nút theo mốc 5 vs ≥6 tin **không có nguồn tài liệu** (`KP-05 §3` #2) nên TC chỉ assert nhánh có đủ tin, ⛔ không assert nhánh ẩn nút. · ⬆️ SUPERSEDED bởi bản v1.1 cùng ID — verdict chính thức nằm ở TC-MASTER-v1.1.xlsx, ⛔ không đếm dòng này vào thống kê round.</t>
         </is>
       </c>
       <c r="N25" s="5" t="inlineStr">
@@ -36285,7 +37009,11 @@
           <t>—</t>
         </is>
       </c>
-      <c r="L26" s="7" t="inlineStr"/>
+      <c r="L26" s="7" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
       <c r="M26" s="7" t="inlineStr"/>
       <c r="N26" s="7" t="inlineStr">
         <is>
@@ -36358,7 +37086,7 @@
           <t>≥1 tin NEED của tài khoản khác (test_data_catalog §HOME)</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr"/>
+      <c r="L27" s="5" t="n"/>
       <c r="M27" s="5" t="inlineStr"/>
       <c r="N27" s="5" t="inlineStr">
         <is>

</xml_diff>